<commit_message>
chore: actualiza recorrido 2026-06-11T08:46Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/06/10 22:56:10</t>
+          <t>2026/06/10 23:56:10</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>166:06:10</t>
+          <t>167:06:10</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026/06/10 22:49:56</t>
+          <t>2026/06/10 23:49:59</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>03:58:20</t>
+          <t>04:58:23</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026/06/10 21:57:22</t>
+          <t>2026/06/10 23:57:22</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L167" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-12T08:25Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/06/11 22:56:10</t>
+          <t>2026/06/11 23:56:10</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>166:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -9528,7 +9528,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>2026/06/11 22:57:22</t>
+          <t>2026/06/11 23:57:27</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>53:48:44</t>
+          <t>54:48:49</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>2026/06/11 22:52:36</t>
+          <t>2026/06/11 23:52:36</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -9838,7 +9838,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>04:03:30</t>
+          <t>05:03:30</t>
         </is>
       </c>
       <c r="L161" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-13T07:45Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/06/12 22:56:08</t>
+          <t>2026/06/12 23:56:08</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>165:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/06/12 22:57:22</t>
+          <t>2026/06/12 23:57:21</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>77:48:44</t>
+          <t>78:48:43</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/06/12 22:46:50</t>
+          <t>2026/06/12 23:46:40</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>29:57:47</t>
+          <t>30:57:37</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/06/12 22:49:34</t>
+          <t>2026/06/12 23:49:34</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>01:04:15</t>
+          <t>02:04:15</t>
         </is>
       </c>
       <c r="L154" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-14T08:18Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -6696,7 +6696,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>2026/06/13 22:57:37</t>
+          <t>2026/06/13 23:57:21</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>101:48:59</t>
+          <t>102:48:43</t>
         </is>
       </c>
       <c r="L108" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-16T09:32Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -5398,7 +5398,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>2026/06/15 22:57:33</t>
+          <t>2026/06/15 23:57:53</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5413,7 +5413,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>149:48:55</t>
+          <t>150:49:15</t>
         </is>
       </c>
       <c r="L86" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-18T08:46Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -619,7 +619,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/06/17 22:57:24</t>
+          <t>2026/06/17 23:56:58</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>166:50:48</t>
+          <t>167:50:22</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/06/17 22:56:10</t>
+          <t>2026/06/17 23:56:10</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -9056,7 +9056,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2026/06/17 21:53:19</t>
+          <t>2026/06/17 23:53:19</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>04:11:14</t>
+          <t>06:11:14</t>
         </is>
       </c>
       <c r="L148" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-18T22:07Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N153"/>
+  <dimension ref="A1:N157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7966,11 +7966,11 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>LPR20251P02790030-ALD</t>
+          <t>SLP20250627045</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -7979,165 +7979,165 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2026/06/15 16:57:33</t>
+          <t>2026/06/15 14:07:26</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>-34.579669, -70.961426</t>
+          <t>-33.38846, -70.617173</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>-34.57967, -70.96143</t>
+          <t>-33.38846, -70.61717</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/06/16 01:37:04</t>
+          <t>2026/06/15 18:13:36</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>-34.579474, -70.961408</t>
+          <t>-33.388382, -70.617199</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>-34.57947, -70.96141</t>
+          <t>-33.38838, -70.61720</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>08:39:31</t>
+          <t>04:06:10</t>
         </is>
       </c>
       <c r="L130" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="M130" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N130" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>SLP20250425120</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2026/06/15 16:58:46</t>
+          <t>2026/06/15 14:19:46</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>-32.7975933, -70.887045</t>
+          <t>-33.388383, -70.617094</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>-32.79759, -70.88705</t>
+          <t>-33.38838, -70.61709</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/06/15 18:12:44</t>
+          <t>2026/06/15 18:32:49</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>-32.7833433, -70.854065</t>
+          <t>-33.388513, -70.617131</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>-32.78334, -70.85407</t>
+          <t>-33.38851, -70.61713</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>01:13:58</t>
+          <t>04:13:03</t>
         </is>
       </c>
       <c r="L131" t="n">
-        <v>4.01</v>
+        <v>0.02</v>
       </c>
       <c r="M131" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="N131" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>LPR20251P02790030-ALD</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2026/06/15 17:40:35</t>
+          <t>2026/06/15 16:57:33</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>-33.36033, -70.8051983</t>
+          <t>-34.579669, -70.961426</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>-33.36033, -70.80520</t>
+          <t>-34.57967, -70.96143</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/06/15 19:12:40</t>
+          <t>2026/06/16 01:37:04</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>-33.0873083, -71.3622833</t>
+          <t>-34.579474, -70.961408</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>-33.08731, -71.36228</t>
+          <t>-34.57947, -70.96141</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>01:32:05</t>
+          <t>08:39:31</t>
         </is>
       </c>
       <c r="L132" t="n">
-        <v>112.63</v>
+        <v>0.02</v>
       </c>
       <c r="M132" t="n">
-        <v>128</v>
+        <v>3</v>
       </c>
       <c r="N132" t="n">
-        <v>71</v>
+        <v>3</v>
       </c>
     </row>
     <row r="133">
@@ -8147,7 +8147,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
@@ -8156,57 +8156,57 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>2026/06/15 18:12:59</t>
+          <t>2026/06/15 16:58:46</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>-32.7834316, -70.8542516</t>
+          <t>-32.7975933, -70.887045</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>-32.78343, -70.85425</t>
+          <t>-32.79759, -70.88705</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/06/15 18:27:41</t>
+          <t>2026/06/15 18:12:44</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>-32.79773, -70.8874249</t>
+          <t>-32.7833433, -70.854065</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>-32.79773, -70.88742</t>
+          <t>-32.78334, -70.85407</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>00:14:42</t>
+          <t>01:13:58</t>
         </is>
       </c>
       <c r="L133" t="n">
-        <v>3.71</v>
+        <v>4.01</v>
       </c>
       <c r="M133" t="n">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="N133" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -8215,57 +8215,57 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2026/06/15 18:27:59</t>
+          <t>2026/06/15 17:40:35</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>-32.797605, -70.8870866</t>
+          <t>-33.36033, -70.8051983</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>-32.79760, -70.88709</t>
+          <t>-33.36033, -70.80520</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/06/15 19:50:54</t>
+          <t>2026/06/15 19:12:40</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>-32.7976599, -70.8873633</t>
+          <t>-33.0873083, -71.3622833</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>-32.79766, -70.88736</t>
+          <t>-33.08731, -71.36228</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>01:22:55</t>
+          <t>01:32:05</t>
         </is>
       </c>
       <c r="L134" t="n">
-        <v>12.97</v>
+        <v>112.63</v>
       </c>
       <c r="M134" t="n">
-        <v>80</v>
+        <v>128</v>
       </c>
       <c r="N134" t="n">
-        <v>22</v>
+        <v>71</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -8274,47 +8274,47 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>2026/06/15 19:13:55</t>
+          <t>2026/06/15 18:12:59</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>-33.0872216, -71.3622716</t>
+          <t>-32.7834316, -70.8542516</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>-33.08722, -71.36227</t>
+          <t>-32.78343, -70.85425</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026/06/16 08:53:03</t>
+          <t>2026/06/15 18:27:41</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>-33.0873283, -71.3622833</t>
+          <t>-32.79773, -70.8874249</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>-33.08733, -71.36228</t>
+          <t>-32.79773, -70.88742</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>13:39:08</t>
+          <t>00:14:42</t>
         </is>
       </c>
       <c r="L135" t="n">
-        <v>0.02</v>
+        <v>3.71</v>
       </c>
       <c r="M135" t="n">
-        <v>8</v>
+        <v>61</v>
       </c>
       <c r="N135" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="136">
@@ -8324,7 +8324,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -8333,53 +8333,53 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>2026/06/15 19:51:11</t>
+          <t>2026/06/15 18:27:59</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>-32.797595, -70.8870983</t>
+          <t>-32.797605, -70.8870866</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>-32.79760, -70.88710</t>
+          <t>-32.79760, -70.88709</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/06/16 08:20:52</t>
+          <t>2026/06/15 19:50:54</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>-33.6327316, -70.8686649</t>
+          <t>-32.7976599, -70.8873633</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>-33.63273, -70.86866</t>
+          <t>-32.79766, -70.88736</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>12:29:41</t>
+          <t>01:22:55</t>
         </is>
       </c>
       <c r="L136" t="n">
-        <v>154.64</v>
+        <v>12.97</v>
       </c>
       <c r="M136" t="n">
-        <v>130</v>
+        <v>80</v>
       </c>
       <c r="N136" t="n">
-        <v>61</v>
+        <v>22</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>LPR20251L02790031-SV</t>
+          <t>SLP20250627045</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -8387,62 +8387,62 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2026/06/16 14:24:41</t>
+          <t>2026/06/15 19:11:20</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>-34.346895, -71.125647</t>
+          <t>-33.38901, -70.617349</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>-34.34690, -71.12565</t>
+          <t>-33.38901, -70.61735</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/06/16 14:49:17</t>
+          <t>2026/06/16 04:49:52</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>-34.346909, -71.125536</t>
+          <t>-33.38851, -70.617518</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>-34.34691, -71.12554</t>
+          <t>-33.38851, -70.61752</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>00:24:36</t>
+          <t>09:38:32</t>
         </is>
       </c>
       <c r="L137" t="n">
-        <v>0.15</v>
+        <v>0.06</v>
       </c>
       <c r="M137" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N137" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>LPR20251L02790031-SV</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -8451,165 +8451,165 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2026/06/16 14:49:31</t>
+          <t>2026/06/15 19:13:55</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>-34.346926, -71.125537</t>
+          <t>-33.0872216, -71.3622716</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>-34.34693, -71.12554</t>
+          <t>-33.08722, -71.36227</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/06/16 15:15:53</t>
+          <t>2026/06/16 08:53:03</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>-34.347368, -71.125768</t>
+          <t>-33.0873283, -71.3622833</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>-34.34737, -71.12577</t>
+          <t>-33.08733, -71.36228</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>00:26:22</t>
+          <t>13:39:08</t>
         </is>
       </c>
       <c r="L138" t="n">
-        <v>0.18</v>
+        <v>0.02</v>
       </c>
       <c r="M138" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N138" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>LPR20251L02790031-SV</t>
+          <t>SLP20250425120</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2026/06/16 15:16:53</t>
+          <t>2026/06/15 19:31:24</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>-34.347169, -71.125764</t>
+          <t>-33.388753, -70.617397</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>-34.34717, -71.12576</t>
+          <t>-33.38875, -70.61740</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>2026/06/16 16:47:57</t>
+          <t>2026/06/16 02:19:45</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>-34.346, -71.125769</t>
+          <t>-33.388201, -70.61719</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>-34.34600, -71.12577</t>
+          <t>-33.38820, -70.61719</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>01:31:04</t>
+          <t>06:48:21</t>
         </is>
       </c>
       <c r="L139" t="n">
-        <v>1.76</v>
+        <v>0.06</v>
       </c>
       <c r="M139" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="N139" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>LPR20251A02800014-DS</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>2026/06/16 16:30:10</t>
+          <t>2026/06/15 19:51:11</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>-34.205426, -70.677296</t>
+          <t>-32.797595, -70.8870983</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>-34.20543, -70.67730</t>
+          <t>-32.79760, -70.88710</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/06/17 23:27:45</t>
+          <t>2026/06/16 08:20:52</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>-34.205436, -70.677309</t>
+          <t>-33.6327316, -70.8686649</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>-34.20544, -70.67731</t>
+          <t>-33.63273, -70.86866</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>30:57:35</t>
+          <t>12:29:41</t>
         </is>
       </c>
       <c r="L140" t="n">
-        <v>0</v>
+        <v>154.64</v>
       </c>
       <c r="M140" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="N140" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
     </row>
     <row r="141">
@@ -8619,7 +8619,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D141" t="inlineStr">
         <is>
@@ -8628,41 +8628,41 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2026/06/16 16:48:53</t>
+          <t>2026/06/16 14:24:41</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>-34.346001, -71.125795</t>
+          <t>-34.346895, -71.125647</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>-34.34600, -71.12579</t>
+          <t>-34.34690, -71.12565</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026/06/17 09:45:58</t>
+          <t>2026/06/16 14:49:17</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>-34.34638, -71.125155</t>
+          <t>-34.346909, -71.125536</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>-34.34638, -71.12516</t>
+          <t>-34.34691, -71.12554</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>16:57:05</t>
+          <t>00:24:36</t>
         </is>
       </c>
       <c r="L141" t="n">
-        <v>0.22</v>
+        <v>0.15</v>
       </c>
       <c r="M141" t="n">
         <v>4</v>
@@ -8674,11 +8674,11 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>JAC X200 SJTJ-50</t>
+          <t>LPR20251L02790031-SV</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D142" t="inlineStr">
         <is>
@@ -8687,57 +8687,57 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2026/06/16 16:51:18</t>
+          <t>2026/06/16 14:49:31</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>-33.3595416, -70.8088316</t>
+          <t>-34.346926, -71.125537</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>-33.35954, -70.80883</t>
+          <t>-34.34693, -71.12554</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/06/16 17:13:18</t>
+          <t>2026/06/16 15:15:53</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>-33.359995, -70.807095</t>
+          <t>-34.347368, -71.125768</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>-33.35999, -70.80710</t>
+          <t>-34.34737, -71.12577</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>00:22:00</t>
+          <t>00:26:22</t>
         </is>
       </c>
       <c r="L142" t="n">
-        <v>0.28</v>
+        <v>0.18</v>
       </c>
       <c r="M142" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="N142" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>JAC X200 SJTJ-50</t>
+          <t>LPR20251L02790031-SV</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -8746,116 +8746,116 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>2026/06/16 17:13:19</t>
+          <t>2026/06/16 15:16:53</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>-33.359995, -70.807095</t>
+          <t>-34.347169, -71.125764</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>-33.35999, -70.80710</t>
+          <t>-34.34717, -71.12576</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/06/16 19:02:32</t>
+          <t>2026/06/16 16:47:57</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>-32.7431433, -70.7330466</t>
+          <t>-34.346, -71.125769</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>-32.74314, -70.73305</t>
+          <t>-34.34600, -71.12577</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>01:49:13</t>
+          <t>01:31:04</t>
         </is>
       </c>
       <c r="L143" t="n">
-        <v>90.31999999999999</v>
+        <v>1.76</v>
       </c>
       <c r="M143" t="n">
-        <v>122</v>
+        <v>7</v>
       </c>
       <c r="N143" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>JAC X200 SJTJ-50</t>
+          <t>LPR20251A02800014-DS</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2026/06/16 19:02:42</t>
+          <t>2026/06/16 16:30:10</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>-32.7432649, -70.7327716</t>
+          <t>-34.205426, -70.677296</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>-32.74326, -70.73277</t>
+          <t>-34.20543, -70.67730</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>2026/06/16 19:19:22</t>
+          <t>2026/06/17 23:27:45</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>-32.7431533, -70.7296483</t>
+          <t>-34.205436, -70.677309</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>-32.74315, -70.72965</t>
+          <t>-34.20544, -70.67731</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>00:16:40</t>
+          <t>30:57:35</t>
         </is>
       </c>
       <c r="L144" t="n">
-        <v>0.37</v>
+        <v>0</v>
       </c>
       <c r="M144" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="N144" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>JAC X200 SJTJ-50</t>
+          <t>LPR20251L02790031-SV</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -8864,293 +8864,293 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2026/06/16 19:20:37</t>
+          <t>2026/06/16 16:48:53</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>-32.74312, -70.72972</t>
+          <t>-34.346001, -71.125795</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>-32.74312, -70.72972</t>
+          <t>-34.34600, -71.12579</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/06/17 08:22:56</t>
+          <t>2026/06/17 09:45:58</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>-33.3599599, -70.8071483</t>
+          <t>-34.34638, -71.125155</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>-33.35996, -70.80715</t>
+          <t>-34.34638, -71.12516</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>13:02:19</t>
+          <t>16:57:05</t>
         </is>
       </c>
       <c r="L145" t="n">
-        <v>90.22</v>
+        <v>0.22</v>
       </c>
       <c r="M145" t="n">
-        <v>118</v>
+        <v>4</v>
       </c>
       <c r="N145" t="n">
-        <v>57</v>
+        <v>3</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>LPR20251P02790030-ALD</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>2026/06/17 15:17:42</t>
+          <t>2026/06/16 16:51:18</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>-34.57966, -70.961408</t>
+          <t>-33.3595416, -70.8088316</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>-34.57966, -70.96141</t>
+          <t>-33.35954, -70.80883</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/06/17 23:19:18</t>
+          <t>2026/06/16 17:13:18</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>-34.57966, -70.961408</t>
+          <t>-33.359995, -70.807095</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>-34.57966, -70.96141</t>
+          <t>-33.35999, -70.80710</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>08:01:36</t>
+          <t>00:22:00</t>
         </is>
       </c>
       <c r="L146" t="n">
-        <v>0</v>
+        <v>0.28</v>
       </c>
       <c r="M146" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="N146" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>LPR20251L02790031-SV</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2026/06/17 16:36:14</t>
+          <t>2026/06/16 17:13:19</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>-34.345978, -71.125749</t>
+          <t>-33.359995, -70.807095</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>-34.34598, -71.12575</t>
+          <t>-33.35999, -70.80710</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/06/17 23:37:59</t>
+          <t>2026/06/16 19:02:32</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>-34.345978, -71.125749</t>
+          <t>-32.7431433, -70.7330466</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>-34.34598, -71.12575</t>
+          <t>-32.74314, -70.73305</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>07:01:45</t>
+          <t>01:49:13</t>
         </is>
       </c>
       <c r="L147" t="n">
-        <v>0</v>
+        <v>90.31999999999999</v>
       </c>
       <c r="M147" t="n">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="N147" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2026/06/17 17:42:05</t>
+          <t>2026/06/16 19:02:42</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>-33.0873166, -71.36232</t>
+          <t>-32.7432649, -70.7327716</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>-33.08732, -71.36232</t>
+          <t>-32.74326, -70.73277</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2026/06/17 23:53:19</t>
+          <t>2026/06/16 19:19:22</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>-33.0872466, -71.36224</t>
+          <t>-32.7431533, -70.7296483</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>-33.08725, -71.36224</t>
+          <t>-32.74315, -70.72965</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>06:11:14</t>
+          <t>00:16:40</t>
         </is>
       </c>
       <c r="L148" t="n">
-        <v>0.01</v>
+        <v>0.37</v>
       </c>
       <c r="M148" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="N148" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2026/06/17 18:35:03</t>
+          <t>2026/06/16 19:20:37</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>-32.7976083, -70.8870916</t>
+          <t>-32.74312, -70.72972</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>-32.79761, -70.88709</t>
+          <t>-32.74312, -70.72972</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>2026/06/17 23:12:37</t>
+          <t>2026/06/17 08:22:56</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>-32.7976083, -70.8870916</t>
+          <t>-33.3599599, -70.8071483</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>-32.79761, -70.88709</t>
+          <t>-33.35996, -70.80715</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>04:37:34</t>
+          <t>13:02:19</t>
         </is>
       </c>
       <c r="L149" t="n">
-        <v>0</v>
+        <v>90.22</v>
       </c>
       <c r="M149" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="N149" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>JAC X200 SJTJ-50</t>
+          <t>LPR20251P02790030-ALD</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D150" t="inlineStr">
         <is>
@@ -9159,37 +9159,37 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>2026/06/17 19:42:38</t>
+          <t>2026/06/17 15:17:42</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>-32.74302, -70.7297716</t>
+          <t>-34.57966, -70.961408</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>-32.74302, -70.72977</t>
+          <t>-34.57966, -70.96141</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026/06/17 23:42:44</t>
+          <t>2026/06/17 23:19:18</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>-32.74302, -70.7297716</t>
+          <t>-34.57966, -70.961408</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>-32.74302, -70.72977</t>
+          <t>-34.57966, -70.96141</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>04:00:06</t>
+          <t>08:01:36</t>
         </is>
       </c>
       <c r="L150" t="n">
@@ -9205,11 +9205,11 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>LPR20251L02790031-SV</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D151" t="inlineStr">
         <is>
@@ -9218,37 +9218,37 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>2026/06/17 19:44:02</t>
+          <t>2026/06/17 16:36:14</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>-33.47617, -70.6984266</t>
+          <t>-34.345978, -71.125749</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>-33.47617, -70.69843</t>
+          <t>-34.34598, -71.12575</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2026/06/17 23:44:12</t>
+          <t>2026/06/17 23:37:59</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>-33.47617, -70.6984266</t>
+          <t>-34.345978, -71.125749</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>-33.47617, -70.69843</t>
+          <t>-34.34598, -71.12575</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>04:00:10</t>
+          <t>07:01:45</t>
         </is>
       </c>
       <c r="L151" t="n">
@@ -9264,11 +9264,11 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -9277,41 +9277,41 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>2026/06/17 21:24:40</t>
+          <t>2026/06/17 17:42:05</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>-33.4370583, -70.6293866</t>
+          <t>-33.0873166, -71.36232</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>-33.43706, -70.62939</t>
+          <t>-33.08732, -71.36232</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>2026/06/17 23:26:45</t>
+          <t>2026/06/17 23:53:19</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>-33.4370583, -70.6293866</t>
+          <t>-33.0872466, -71.36224</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>-33.43706, -70.62939</t>
+          <t>-33.08725, -71.36224</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>02:02:05</t>
+          <t>06:11:14</t>
         </is>
       </c>
       <c r="L152" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="M152" t="n">
         <v>0</v>
@@ -9323,11 +9323,11 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -9336,37 +9336,37 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2026/06/17 22:16:58</t>
+          <t>2026/06/17 18:35:03</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>-32.841647, -70.93681</t>
+          <t>-32.7976083, -70.8870916</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>-32.84165, -70.93681</t>
+          <t>-32.79761, -70.88709</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/06/17 23:20:00</t>
+          <t>2026/06/17 23:12:37</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>-32.841647, -70.93681</t>
+          <t>-32.7976083, -70.8870916</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>-32.84165, -70.93681</t>
+          <t>-32.79761, -70.88709</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>01:03:02</t>
+          <t>04:37:34</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -9376,6 +9376,242 @@
         <v>0</v>
       </c>
       <c r="N153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>13</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2026/06/17 19:42:38</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>-32.74302, -70.7297716</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>-32.74302, -70.72977</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>2026/06/17 23:42:44</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>-32.74302, -70.7297716</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>-32.74302, -70.72977</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>04:00:06</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>9</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2026/06/17 19:44:02</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.6984266</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69843</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>2026/06/17 23:44:12</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.6984266</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69843</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>04:00:10</t>
+        </is>
+      </c>
+      <c r="L155" t="n">
+        <v>0</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0</v>
+      </c>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>11</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>2026/06/17 21:24:40</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>-33.4370583, -70.6293866</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>-33.43706, -70.62939</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>2026/06/17 23:26:45</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>-33.4370583, -70.6293866</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>-33.43706, -70.62939</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>02:02:05</t>
+        </is>
+      </c>
+      <c r="L156" t="n">
+        <v>0</v>
+      </c>
+      <c r="M156" t="n">
+        <v>0</v>
+      </c>
+      <c r="N156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>8</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>2026/06/17 22:16:58</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>-32.841647, -70.93681</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>-32.84165, -70.93681</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>2026/06/17 23:20:00</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>-32.841647, -70.93681</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>-32.84165, -70.93681</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>01:03:02</t>
+        </is>
+      </c>
+      <c r="L157" t="n">
+        <v>0</v>
+      </c>
+      <c r="M157" t="n">
+        <v>0</v>
+      </c>
+      <c r="N157" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9390,7 +9626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9689,38 +9925,76 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>SLP20250425120</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>656.04</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>138</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>SLP20250627045</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>656.04</v>
+      </c>
+      <c r="C18" t="n">
+        <v>62</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>VOLKSWAGEN AMAROK KPDV-13</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B19" t="n">
         <v>907.61</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C19" t="n">
         <v>51</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D19" t="n">
         <v>1</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E19" t="n">
         <v>143</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-20T07:49Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/06/19 22:53:32</t>
+          <t>2026/06/19 23:53:32</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:57:24</t>
+          <t>166:57:24</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/06/19 22:57:45</t>
+          <t>2026/06/19 23:57:37</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>165:58:37</t>
+          <t>166:58:29</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/06/19 22:34:42</t>
+          <t>2026/06/19 23:34:40</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>29:37:41</t>
+          <t>30:37:39</t>
         </is>
       </c>
       <c r="L145" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/06/19 22:52:29</t>
+          <t>2026/06/19 23:52:29</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>07:01:01</t>
+          <t>08:01:01</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/06/19 21:53:59</t>
+          <t>2026/06/19 23:53:59</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026/06/19 22:59:21</t>
+          <t>2026/06/19 23:59:20</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>01:57:30</t>
+          <t>02:57:29</t>
         </is>
       </c>
       <c r="L167" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-23T07:48Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/06/22 22:56:10</t>
+          <t>2026/06/22 23:56:10</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/06/22 22:57:39</t>
+          <t>2026/06/22 23:57:15</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>166:00:07</t>
+          <t>166:59:43</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>2026/06/22 22:45:44</t>
+          <t>2026/06/22 23:45:43</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>08:01:04</t>
+          <t>09:01:03</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -10236,7 +10236,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>2026/06/22 22:49:05</t>
+          <t>2026/06/22 23:49:05</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>06:01:37</t>
+          <t>07:01:37</t>
         </is>
       </c>
       <c r="L168" t="n">
@@ -10295,7 +10295,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>2026/06/22 22:37:26</t>
+          <t>2026/06/22 23:37:26</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>05:03:21</t>
+          <t>06:03:21</t>
         </is>
       </c>
       <c r="L169" t="n">
@@ -10472,7 +10472,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>2026/06/22 21:54:15</t>
+          <t>2026/06/22 23:54:15</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L172" t="n">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>2026/06/22 22:41:17</t>
+          <t>2026/06/22 23:41:17</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>01:57:29</t>
+          <t>02:57:29</t>
         </is>
       </c>
       <c r="L175" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-24T07:39Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/06/23 22:56:12</t>
+          <t>2026/06/23 23:56:12</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/06/23 22:57:21</t>
+          <t>2026/06/23 23:57:21</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:58:13</t>
+          <t>166:58:13</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026/06/23 22:31:38</t>
+          <t>2026/06/23 23:31:38</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>164:00:00</t>
+          <t>165:00:00</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -10354,7 +10354,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>2026/06/23 21:59:44</t>
+          <t>2026/06/23 23:59:44</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>02:00:17</t>
+          <t>04:00:17</t>
         </is>
       </c>
       <c r="L170" t="n">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>2026/06/23 22:42:56</t>
+          <t>2026/06/23 23:42:57</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>01:57:35</t>
+          <t>02:57:36</t>
         </is>
       </c>
       <c r="L175" t="n">
@@ -10885,26 +10885,26 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>2026/06/23 23:28:28</t>
+          <t>2026/06/23 23:57:08</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>-32.845465, -70.6048249</t>
+          <t>-32.84549, -70.6047049</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>-32.84546, -70.60482</t>
+          <t>-32.84549, -70.60470</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>00:46:38</t>
+          <t>01:15:18</t>
         </is>
       </c>
       <c r="L179" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="M179" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-25T07:41Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N181"/>
+  <dimension ref="A1:N182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/06/24 22:31:21</t>
+          <t>2026/06/24 23:31:38</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>165:59:43</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/06/24 22:56:12</t>
+          <t>2026/06/24 23:56:12</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>166:00:02</t>
+          <t>167:00:02</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/06/24 22:57:21</t>
+          <t>2026/06/24 23:57:37</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>165:59:58</t>
+          <t>167:00:14</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -10236,7 +10236,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>2026/06/24 22:40:54</t>
+          <t>2026/06/24 23:40:54</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>09:04:34</t>
+          <t>10:04:34</t>
         </is>
       </c>
       <c r="L168" t="n">
@@ -10295,7 +10295,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>2026/06/24 21:54:20</t>
+          <t>2026/06/24 23:54:20</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>08:01:43</t>
+          <t>10:01:43</t>
         </is>
       </c>
       <c r="L169" t="n">
@@ -10413,7 +10413,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>2026/06/24 21:44:27</t>
+          <t>2026/06/24 23:44:27</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>06:10:39</t>
+          <t>08:10:39</t>
         </is>
       </c>
       <c r="L171" t="n">
@@ -10590,7 +10590,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>2026/06/24 22:43:50</t>
+          <t>2026/06/24 23:43:50</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -10605,7 +10605,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>06:01:31</t>
+          <t>07:01:31</t>
         </is>
       </c>
       <c r="L174" t="n">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>2026/06/24 22:45:55</t>
+          <t>2026/06/24 23:45:55</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>06:01:00</t>
+          <t>07:01:00</t>
         </is>
       </c>
       <c r="L175" t="n">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>2026/06/24 22:34:19</t>
+          <t>2026/06/24 23:34:19</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -10841,7 +10841,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>04:03:04</t>
+          <t>05:03:04</t>
         </is>
       </c>
       <c r="L178" t="n">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>2026/06/24 21:49:21</t>
+          <t>2026/06/24 23:49:21</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L180" t="n">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026/06/24 21:51:19</t>
+          <t>2026/06/24 23:51:19</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L181" t="n">
@@ -11028,6 +11028,65 @@
         <v>0</v>
       </c>
       <c r="N181" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>13</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>2026/06/24 21:39:56</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>-32.838389, -70.955509</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>-32.83839, -70.95551</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>2026/06/24 23:38:30</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>-32.838389, -70.955509</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>-32.83839, -70.95551</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>01:58:34</t>
+        </is>
+      </c>
+      <c r="L182" t="n">
+        <v>0</v>
+      </c>
+      <c r="M182" t="n">
+        <v>0</v>
+      </c>
+      <c r="N182" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11098,13 +11157,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1317.27</v>
+        <v>1317.21</v>
       </c>
       <c r="C3" t="n">
         <v>61</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>141</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-26T07:51Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N182"/>
+  <dimension ref="A1:N183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/06/25 22:53:35</t>
+          <t>2026/06/25 23:53:35</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>166:00:03</t>
+          <t>167:00:03</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/06/25 22:57:15</t>
+          <t>2026/06/25 23:57:40</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:58:03</t>
+          <t>166:58:28</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -10354,22 +10354,22 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>2026/06/25 22:48:10</t>
+          <t>2026/06/25 23:48:10</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>-33.36004, -70.807126</t>
+          <t>-33.36003, -70.807123</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>-33.36004, -70.80713</t>
+          <t>-33.36003, -70.80712</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>06:01:00</t>
+          <t>07:01:00</t>
         </is>
       </c>
       <c r="L170" t="n">
@@ -10885,7 +10885,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>2026/06/25 21:40:26</t>
+          <t>2026/06/25 23:40:26</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -10900,7 +10900,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>02:11:51</t>
+          <t>04:11:51</t>
         </is>
       </c>
       <c r="L179" t="n">
@@ -11003,26 +11003,26 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026/06/25 21:51:01</t>
+          <t>2026/06/25 21:50:46</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>-32.7430566, -70.729785</t>
+          <t>-32.7430883, -70.7297366</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>-32.74306, -70.72979</t>
+          <t>-32.74309, -70.72974</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>00:33:58</t>
+          <t>00:33:43</t>
         </is>
       </c>
       <c r="L181" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="M181" t="n">
         <v>15</v>
@@ -11087,6 +11087,65 @@
         <v>0</v>
       </c>
       <c r="N182" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>20</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>2026/06/25 21:51:01</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>-32.7430566, -70.729785</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>-32.74306, -70.72979</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>2026/06/25 23:51:01</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>-32.7430566, -70.729785</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>-32.74306, -70.72979</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L183" t="n">
+        <v>0</v>
+      </c>
+      <c r="M183" t="n">
+        <v>0</v>
+      </c>
+      <c r="N183" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11195,13 +11254,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1012.33</v>
+        <v>1012.32</v>
       </c>
       <c r="C5" t="n">
         <v>75</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>139</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-27T06:51Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N178"/>
+  <dimension ref="A1:N180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/06/26 22:53:35</t>
+          <t>2026/06/26 23:53:35</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>166:00:03</t>
+          <t>167:00:03</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026/06/26 21:57:14</t>
+          <t>2026/06/26 23:57:17</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>164:59:53</t>
+          <t>166:59:56</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/06/26 22:40:42</t>
+          <t>2026/06/26 23:40:42</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>67:00:33</t>
+          <t>68:00:33</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/06/26 22:13:05</t>
+          <t>2026/06/26 23:13:24</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>53:30:46</t>
+          <t>54:31:05</t>
         </is>
       </c>
       <c r="L145" t="n">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>2026/06/26 21:18:29</t>
+          <t>2026/06/26 23:18:29</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -10546,7 +10546,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>05:41:02</t>
+          <t>07:41:02</t>
         </is>
       </c>
       <c r="L173" t="n">
@@ -10590,7 +10590,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>2026/06/26 22:14:15</t>
+          <t>2026/06/26 23:13:51</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -10605,7 +10605,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>05:00:26</t>
+          <t>06:00:02</t>
         </is>
       </c>
       <c r="L174" t="n">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>2026/06/26 21:34:24</t>
+          <t>2026/06/26 23:34:24</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L175" t="n">
@@ -10767,7 +10767,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>2026/06/26 21:51:17</t>
+          <t>2026/06/26 23:51:17</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L177" t="n">
@@ -10798,11 +10798,11 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>JAC X200 SJTJ-50</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
@@ -10811,46 +10811,164 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>2026/06/26 21:53:47</t>
+          <t>2026/06/26 21:13:03</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>-32.743075, -70.7297933</t>
+          <t>-33.4761283, -70.6985433</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>-32.74307, -70.72979</t>
+          <t>-33.47613, -70.69854</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>2026/06/26 22:01:41</t>
+          <t>2026/06/26 23:13:33</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>-32.7430083, -70.7298233</t>
+          <t>-33.4761283, -70.6985433</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>-32.74301, -70.72982</t>
+          <t>-33.47613, -70.69854</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>00:07:54</t>
+          <t>02:00:30</t>
         </is>
       </c>
       <c r="L178" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="M178" t="n">
         <v>0</v>
       </c>
       <c r="N178" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>13</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>2026/06/26 21:53:47</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>-32.743075, -70.7297933</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>-32.74307, -70.72979</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>2026/06/26 22:01:41</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>-32.7430083, -70.7298233</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>-32.74301, -70.72982</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>00:07:54</t>
+        </is>
+      </c>
+      <c r="L179" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M179" t="n">
+        <v>0</v>
+      </c>
+      <c r="N179" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>9</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>2026/06/26 22:31:15</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>-33.399197, -70.795128</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>-33.39920, -70.79513</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>2026/06/26 23:35:15</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>-33.399197, -70.795128</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>-33.39920, -70.79513</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>01:04:00</t>
+        </is>
+      </c>
+      <c r="L180" t="n">
+        <v>0</v>
+      </c>
+      <c r="M180" t="n">
+        <v>0</v>
+      </c>
+      <c r="N180" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10921,10 +11039,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>818.65</v>
+        <v>819.58</v>
       </c>
       <c r="C3" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -11130,13 +11248,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1564.21</v>
+        <v>1564.18</v>
       </c>
       <c r="C14" t="n">
         <v>75</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>131</v>
@@ -11244,13 +11362,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>635.54</v>
+        <v>635.47</v>
       </c>
       <c r="C20" t="n">
         <v>57</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>147</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-28T07:50Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N181"/>
+  <dimension ref="A1:N182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/06/27 22:53:35</t>
+          <t>2026/06/27 23:53:35</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>166:00:03</t>
+          <t>167:00:03</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026/06/27 22:57:46</t>
+          <t>2026/06/27 23:57:45</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>165:58:39</t>
+          <t>166:58:38</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/06/27 22:40:42</t>
+          <t>2026/06/27 23:40:42</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>91:00:33</t>
+          <t>92:00:33</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>2026/06/27 21:54:08</t>
+          <t>2026/06/27 23:54:08</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L180" t="n">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026/06/27 22:48:54</t>
+          <t>2026/06/27 23:48:54</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>01:02:59</t>
+          <t>02:02:59</t>
         </is>
       </c>
       <c r="L181" t="n">
@@ -11028,6 +11028,65 @@
         <v>0</v>
       </c>
       <c r="N181" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>8</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>2026/06/27 21:48:29</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>-32.780847, -70.98129</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>-32.78085, -70.98129</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>2026/06/27 23:45:58</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>-32.780847, -70.98129</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>-32.78085, -70.98129</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>01:57:29</t>
+        </is>
+      </c>
+      <c r="L182" t="n">
+        <v>0</v>
+      </c>
+      <c r="M182" t="n">
+        <v>0</v>
+      </c>
+      <c r="N182" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11104,7 +11163,7 @@
         <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>140</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-29T08:58Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N185"/>
+  <dimension ref="A1:N186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026/06/28 22:56:10</t>
+          <t>2026/06/28 23:56:10</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026/06/28 22:57:45</t>
+          <t>2026/06/28 23:57:47</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>166:00:08</t>
+          <t>167:00:10</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -11211,11 +11211,11 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+          <t>MITSUBISHI L200 PHZF-89</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
@@ -11224,37 +11224,37 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>2026/06/28 21:51:51</t>
+          <t>2026/06/28 21:51:21</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>-32.841725, -70.93688</t>
+          <t>-33.4362983, -70.6294</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>-32.84172, -70.93688</t>
+          <t>-33.43630, -70.62940</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>2026/06/28 22:54:50</t>
+          <t>2026/06/28 23:51:21</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>-32.841725, -70.93688</t>
+          <t>-33.4362983, -70.6294</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>-32.84172, -70.93688</t>
+          <t>-33.43630, -70.62940</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>01:02:59</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="L185" t="n">
@@ -11264,6 +11264,65 @@
         <v>0</v>
       </c>
       <c r="N185" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>7</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>2026/06/28 21:51:51</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>-32.841725, -70.93688</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>-32.84172, -70.93688</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>2026/06/28 23:54:50</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>-32.841725, -70.93688</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>-32.84172, -70.93688</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>02:02:59</t>
+        </is>
+      </c>
+      <c r="L186" t="n">
+        <v>0</v>
+      </c>
+      <c r="M186" t="n">
+        <v>0</v>
+      </c>
+      <c r="N186" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11568,7 +11627,7 @@
         <v>34</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>144</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-06-30T07:52Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/06/29 22:56:10</t>
+          <t>2026/06/29 23:56:10</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/06/29 22:57:38</t>
+          <t>2026/06/29 23:57:15</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>165:58:27</t>
+          <t>166:58:04</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/06/29 21:44:31</t>
+          <t>2026/06/29 23:44:31</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>99:36:24</t>
+          <t>101:36:24</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>2026/06/29 22:46:40</t>
+          <t>2026/06/29 23:46:16</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -10546,7 +10546,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>77:32:51</t>
+          <t>78:32:27</t>
         </is>
       </c>
       <c r="L173" t="n">
@@ -11180,7 +11180,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>2026/06/29 22:47:44</t>
+          <t>2026/06/29 23:47:47</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -11195,7 +11195,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>01:02:55</t>
+          <t>02:02:58</t>
         </is>
       </c>
       <c r="L184" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-01T08:11Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1563,7 +1563,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026/06/30 22:56:08</t>
+          <t>2026/06/30 23:56:08</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>165:59:56</t>
+          <t>166:59:56</t>
         </is>
       </c>
       <c r="L21" t="n">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026/06/30 22:57:21</t>
+          <t>2026/06/30 23:57:17</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>165:59:44</t>
+          <t>166:59:40</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>2026/06/30 21:44:31</t>
+          <t>2026/06/30 23:44:31</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>123:36:24</t>
+          <t>125:36:24</t>
         </is>
       </c>
       <c r="L144" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-02T07:30Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/07/01 22:56:08</t>
+          <t>2026/07/01 23:56:08</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:59:56</t>
+          <t>166:59:56</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/01 22:57:22</t>
+          <t>2026/07/01 23:57:41</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:58:15</t>
+          <t>166:58:34</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>2026/07/01 21:44:31</t>
+          <t>2026/07/01 23:44:31</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>147:36:24</t>
+          <t>149:36:24</t>
         </is>
       </c>
       <c r="L108" t="n">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>2026/07/01 22:40:46</t>
+          <t>2026/07/01 23:40:46</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9130,7 +9130,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>44:01:19</t>
+          <t>45:01:19</t>
         </is>
       </c>
       <c r="L149" t="n">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>2026/07/01 22:46:14</t>
+          <t>2026/07/01 23:46:14</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>34:51:17</t>
+          <t>35:51:17</t>
         </is>
       </c>
       <c r="L152" t="n">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/07/01 22:42:50</t>
+          <t>2026/07/01 23:42:50</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>29:13:16</t>
+          <t>30:13:16</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>2026/07/01 21:48:02</t>
+          <t>2026/07/01 23:48:02</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>03:06:51</t>
+          <t>05:06:51</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/07/01 21:50:56</t>
+          <t>2026/07/01 23:50:56</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L159" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-02T17:46Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1063,7 +1063,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SLP20250425120</t>
+          <t>SLP20250425120-AC01</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1181,7 +1181,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SLP20250627045</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2597,7 +2597,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SLP20250627045</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -3482,7 +3482,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SLP20250627045</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -3600,7 +3600,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SLP20250627045</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3718,7 +3718,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SLP20250627045</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -6078,7 +6078,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SLP20250627045</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -6137,7 +6137,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SLP20250627045</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -9264,7 +9264,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SLP20250627045</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -10298,7 +10298,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SLP20250425120</t>
+          <t>SLP20250425120-AC01</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -10317,7 +10317,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SLP20250627045</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="B18" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-03T07:19Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N142"/>
+  <dimension ref="A1:N143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/02 22:01:38</t>
+          <t>2026/07/02 23:01:16</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>166:00:17</t>
+          <t>166:59:55</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -619,7 +619,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/07/02 21:44:31</t>
+          <t>2026/07/02 23:44:31</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>165:36:22</t>
+          <t>167:36:22</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/07/02 22:13:15</t>
+          <t>2026/07/02 23:13:36</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>165:59:52</t>
+          <t>167:00:13</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/02 21:56:12</t>
+          <t>2026/07/02 23:56:12</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>165:02:37</t>
+          <t>167:02:37</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/02 21:57:15</t>
+          <t>2026/07/02 23:57:21</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>164:59:38</t>
+          <t>166:59:44</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026/07/02 22:41:12</t>
+          <t>2026/07/02 23:41:12</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>68:01:45</t>
+          <t>69:01:45</t>
         </is>
       </c>
       <c r="L115" t="n">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/07/02 22:11:24</t>
+          <t>2026/07/02 23:11:22</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>52:41:50</t>
+          <t>53:41:48</t>
         </is>
       </c>
       <c r="L119" t="n">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/07/02 21:53:23</t>
+          <t>2026/07/02 23:53:17</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>06:15:11</t>
+          <t>08:15:05</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/07/02 22:04:58</t>
+          <t>2026/07/02 23:04:58</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>04:03:05</t>
+          <t>05:03:05</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/07/02 21:08:56</t>
+          <t>2026/07/02 23:08:56</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>02:00:43</t>
+          <t>04:00:43</t>
         </is>
       </c>
       <c r="L134" t="n">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/07/02 21:48:16</t>
+          <t>2026/07/02 23:48:17</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>01:57:29</t>
+          <t>03:57:30</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -8728,6 +8728,65 @@
       </c>
       <c r="N142" t="n">
         <v>23</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>9</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>2026/07/02 21:57:31</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>-33.4760816, -70.6985116</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>-33.47608, -70.69851</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>2026/07/02 23:57:43</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>-33.4760816, -70.6985116</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>-33.47608, -70.69851</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>02:00:12</t>
+        </is>
+      </c>
+      <c r="L143" t="n">
+        <v>0</v>
+      </c>
+      <c r="M143" t="n">
+        <v>0</v>
+      </c>
+      <c r="N143" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -9006,13 +9065,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1025.93</v>
+        <v>1025.91</v>
       </c>
       <c r="C14" t="n">
         <v>69</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>131</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-04T06:46Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -619,7 +619,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/07/03 22:01:26</t>
+          <t>2026/07/03 23:01:37</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>165:59:47</t>
+          <t>166:59:58</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/07/03 22:13:14</t>
+          <t>2026/07/03 23:13:24</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>166:00:04</t>
+          <t>167:00:14</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/03 21:56:12</t>
+          <t>2026/07/03 23:56:12</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:02:37</t>
+          <t>167:02:37</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/07/03 21:57:29</t>
+          <t>2026/07/03 23:57:27</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>164:59:52</t>
+          <t>166:59:50</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>2026/07/03 22:11:17</t>
+          <t>2026/07/03 23:11:36</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5177,7 +5177,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>76:41:43</t>
+          <t>77:42:02</t>
         </is>
       </c>
       <c r="L82" t="n">
@@ -7817,7 +7817,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>2026/07/03 21:49:36</t>
+          <t>2026/07/03 23:49:36</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7832,7 +7832,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>10:00:10</t>
+          <t>12:00:10</t>
         </is>
       </c>
       <c r="L127" t="n">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/07/03 21:38:36</t>
+          <t>2026/07/03 23:38:36</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>03:42:38</t>
+          <t>05:42:38</t>
         </is>
       </c>
       <c r="L134" t="n">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/07/03 21:46:58</t>
+          <t>2026/07/03 23:46:58</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>02:01:02</t>
+          <t>04:01:02</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/07/03 22:06:43</t>
+          <t>2026/07/03 23:06:40</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>00:06:15</t>
+          <t>01:06:12</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -8502,7 +8502,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>662.99</v>
+        <v>663.73</v>
       </c>
       <c r="C3" t="n">
         <v>51</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-05T07:24Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N140"/>
+  <dimension ref="A1:N141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/04 22:01:37</t>
+          <t>2026/07/04 23:01:21</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>166:00:21</t>
+          <t>167:00:05</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/07/04 22:13:16</t>
+          <t>2026/07/04 23:13:36</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:20</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/04 22:56:09</t>
+          <t>2026/07/04 23:56:09</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>166:02:34</t>
+          <t>167:02:34</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/07/04 21:57:38</t>
+          <t>2026/07/04 23:57:21</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>164:59:30</t>
+          <t>166:59:13</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -4749,7 +4749,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>2026/07/04 22:11:47</t>
+          <t>2026/07/04 23:11:32</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>100:42:13</t>
+          <t>101:41:58</t>
         </is>
       </c>
       <c r="L75" t="n">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026/07/04 21:25:06</t>
+          <t>2026/07/04 23:25:06</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>04:01:21</t>
+          <t>06:01:21</t>
         </is>
       </c>
       <c r="L135" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/07/04 22:38:58</t>
+          <t>2026/07/04 23:38:58</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>01:03:03</t>
+          <t>02:03:03</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -8609,6 +8609,65 @@
         <v>0</v>
       </c>
       <c r="N140" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>10</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>2026/07/04 21:52:40</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>-32.780851, -70.981255</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>-32.78085, -70.98126</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>2026/07/04 23:50:10</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>-32.780851, -70.981255</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>-32.78085, -70.98126</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>01:57:30</t>
+        </is>
+      </c>
+      <c r="L141" t="n">
+        <v>0</v>
+      </c>
+      <c r="M141" t="n">
+        <v>0</v>
+      </c>
+      <c r="N141" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8685,7 +8744,7 @@
         <v>53</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>141</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-06T08:19Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/05 22:56:09</t>
+          <t>2026/07/05 23:56:09</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>165:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/05 22:57:39</t>
+          <t>2026/07/05 23:57:26</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:58:31</t>
+          <t>166:58:18</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/07/05 21:43:59</t>
+          <t>2026/07/05 23:43:59</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>02:00:01</t>
+          <t>04:00:01</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026/07/05 22:59:54</t>
+          <t>2026/07/05 23:59:55</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>02:57:31</t>
+          <t>03:57:32</t>
         </is>
       </c>
       <c r="L141" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-07T07:36Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N159"/>
+  <dimension ref="A1:N161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,7 +619,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/07/06 22:01:21</t>
+          <t>2026/07/06 23:01:39</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>165:59:44</t>
+          <t>167:00:02</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/07/06 22:13:30</t>
+          <t>2026/07/06 23:13:37</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>166:00:04</t>
+          <t>167:00:11</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/06 22:56:11</t>
+          <t>2026/07/06 23:56:11</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>166:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/06 21:57:22</t>
+          <t>2026/07/06 23:57:24</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>164:59:44</t>
+          <t>166:59:46</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -4808,7 +4808,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>2026/07/06 22:11:21</t>
+          <t>2026/07/06 23:11:38</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>148:41:47</t>
+          <t>149:42:04</t>
         </is>
       </c>
       <c r="L76" t="n">
@@ -9233,22 +9233,22 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2026/07/06 22:44:08</t>
+          <t>2026/07/06 23:44:07</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>-33.360033, -70.807094</t>
+          <t>-33.360032, -70.807101</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>-33.36003, -70.80709</t>
+          <t>-33.36003, -70.80710</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>06:05:22</t>
+          <t>07:05:21</t>
         </is>
       </c>
       <c r="L151" t="n">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>2026/07/06 22:40:06</t>
+          <t>2026/07/06 23:40:09</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>04:03:45</t>
+          <t>05:03:48</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -9528,7 +9528,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>2026/07/06 21:33:58</t>
+          <t>2026/07/06 23:33:58</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>02:11:43</t>
+          <t>04:11:43</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>2026/07/06 21:23:29</t>
+          <t>2026/07/06 23:23:29</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -9602,7 +9602,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L157" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/07/06 21:45:04</t>
+          <t>2026/07/06 23:45:04</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/07/06 21:57:58</t>
+          <t>2026/07/06 23:57:58</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>02:00:08</t>
+          <t>04:00:08</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -9730,6 +9730,124 @@
         <v>0</v>
       </c>
       <c r="N159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>7</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>2026/07/06 21:08:29</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>-32.838348, -70.955692</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>-32.83835, -70.95569</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>2026/07/06 23:06:48</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>-32.838348, -70.955692</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>-32.83835, -70.95569</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>01:58:19</t>
+        </is>
+      </c>
+      <c r="L160" t="n">
+        <v>0</v>
+      </c>
+      <c r="M160" t="n">
+        <v>0</v>
+      </c>
+      <c r="N160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>10</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>2026/07/06 21:15:50</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>-33.4362633, -70.6293216</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>-33.43626, -70.62932</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>2026/07/06 23:15:50</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>-33.4362633, -70.6293216</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>-33.43626, -70.62932</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L161" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" t="n">
+        <v>0</v>
+      </c>
+      <c r="N161" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9800,13 +9918,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>882.66</v>
+        <v>882.62</v>
       </c>
       <c r="C3" t="n">
         <v>57</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
         <v>141</v>
@@ -10028,13 +10146,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>321</v>
+        <v>320.91</v>
       </c>
       <c r="C15" t="n">
         <v>48</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>126</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-07T14:30Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -9351,26 +9351,26 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/07/06 22:48:07</t>
+          <t>2026/07/06 22:50:17</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>-33.400785, -70.5716966</t>
+          <t>-33.40065, -70.5716883</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>-33.40078, -70.57170</t>
+          <t>-33.40065, -70.57169</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>05:57:54</t>
+          <t>06:00:04</t>
         </is>
       </c>
       <c r="L153" t="n">
-        <v>14.99</v>
+        <v>15</v>
       </c>
       <c r="M153" t="n">
         <v>98</v>
@@ -10165,7 +10165,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>275.26</v>
+        <v>275.28</v>
       </c>
       <c r="C16" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-08T06:27Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N168"/>
+  <dimension ref="A1:N167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/07 22:01:21</t>
+          <t>2026/07/07 23:01:21</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:59:45</t>
+          <t>166:59:45</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/07/07 22:13:21</t>
+          <t>2026/07/07 23:13:40</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>165:59:57</t>
+          <t>167:00:16</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/07/07 22:11:21</t>
+          <t>2026/07/07 23:12:00</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>165:40:46</t>
+          <t>166:41:25</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026/07/07 21:56:11</t>
+          <t>2026/07/07 23:56:11</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>165:00:03</t>
+          <t>167:00:03</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026/07/07 21:31:16</t>
+          <t>2026/07/07 23:31:15</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>157:15:02</t>
+          <t>159:15:01</t>
         </is>
       </c>
       <c r="L27" t="n">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>2026/07/07 21:40:08</t>
+          <t>2026/07/07 23:40:11</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -9838,7 +9838,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>04:03:54</t>
+          <t>06:03:57</t>
         </is>
       </c>
       <c r="L161" t="n">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026/07/07 20:53:09</t>
+          <t>2026/07/07 22:53:09</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>02:00:04</t>
+          <t>04:00:04</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2026/07/07 21:20:49</t>
+          <t>2026/07/07 23:20:49</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L165" t="n">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>2026/07/07 21:24:06</t>
+          <t>2026/07/07 23:24:06</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026/07/07 21:25:38</t>
+          <t>2026/07/07 23:25:38</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>02:00:11</t>
+          <t>04:00:11</t>
         </is>
       </c>
       <c r="L167" t="n">
@@ -10202,65 +10202,6 @@
         <v>0</v>
       </c>
       <c r="N167" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
-        </is>
-      </c>
-      <c r="C168" t="n">
-        <v>1</v>
-      </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>Paradas</t>
-        </is>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>2026/07/07 19:34:40</t>
-        </is>
-      </c>
-      <c r="F168" t="inlineStr">
-        <is>
-          <t>-33.4133183, -70.5978216</t>
-        </is>
-      </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>-33.41332, -70.59782</t>
-        </is>
-      </c>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>2026/07/07 21:37:43</t>
-        </is>
-      </c>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>-33.4132783, -70.5975683</t>
-        </is>
-      </c>
-      <c r="J168" t="inlineStr">
-        <is>
-          <t>-33.41328, -70.59757</t>
-        </is>
-      </c>
-      <c r="K168" t="inlineStr">
-        <is>
-          <t>02:03:03</t>
-        </is>
-      </c>
-      <c r="L168" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="M168" t="n">
-        <v>0</v>
-      </c>
-      <c r="N168" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10331,13 +10272,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1078.76</v>
+        <v>1078.7</v>
       </c>
       <c r="C3" t="n">
         <v>58</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
         <v>141</v>
@@ -10559,13 +10500,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>298.84</v>
+        <v>307.17</v>
       </c>
       <c r="C15" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
         <v>126</v>
@@ -10578,7 +10519,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>329.24</v>
+        <v>335.8</v>
       </c>
       <c r="C16" t="n">
         <v>13</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-09T07:36Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N169"/>
+  <dimension ref="A1:N172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/08 22:01:21</t>
+          <t>2026/07/08 23:01:38</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:17</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/07/08 22:13:38</t>
+          <t>2026/07/08 23:13:21</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>166:00:21</t>
+          <t>167:00:04</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/07/08 22:31:51</t>
+          <t>2026/07/08 23:31:23</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>166:16:27</t>
+          <t>167:15:59</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/07/08 21:56:09</t>
+          <t>2026/07/08 23:56:09</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>2026/07/08 22:49:09</t>
+          <t>2026/07/08 23:49:09</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -9897,7 +9897,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>06:01:01</t>
+          <t>07:01:01</t>
         </is>
       </c>
       <c r="L162" t="n">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026/07/08 21:37:54</t>
+          <t>2026/07/08 23:37:54</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>03:58:22</t>
+          <t>05:58:22</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/07/08 21:37:25</t>
+          <t>2026/07/08 23:37:25</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -10208,11 +10208,11 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCL-70</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
@@ -10221,37 +10221,37 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>2026/07/08 21:39:36</t>
+          <t>2026/07/08 21:12:09</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>-32.838381, -70.955498</t>
+          <t>-32.743035, -70.7297883</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>-32.83838, -70.95550</t>
+          <t>-32.74303, -70.72979</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>2026/07/08 22:38:05</t>
+          <t>2026/07/08 23:12:09</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>-32.838381, -70.955498</t>
+          <t>-32.743035, -70.7297883</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>-32.83838, -70.95550</t>
+          <t>-32.74303, -70.72979</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>00:58:29</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="L168" t="n">
@@ -10267,11 +10267,11 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+          <t>MITSUBISHI L200 PHZF-89</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D169" t="inlineStr">
         <is>
@@ -10280,37 +10280,37 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>2026/07/08 21:43:27</t>
+          <t>2026/07/08 21:14:57</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>-32.841869, -70.9368</t>
+          <t>-33.4374016, -70.6293816</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>-32.84187, -70.93680</t>
+          <t>-33.43740, -70.62938</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>2026/07/08 22:46:39</t>
+          <t>2026/07/08 23:15:05</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>-32.841869, -70.9368</t>
+          <t>-33.4374016, -70.6293816</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>-32.84187, -70.93680</t>
+          <t>-33.43740, -70.62938</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>01:03:12</t>
+          <t>02:00:08</t>
         </is>
       </c>
       <c r="L169" t="n">
@@ -10320,6 +10320,183 @@
         <v>0</v>
       </c>
       <c r="N169" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>10</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>2026/07/08 21:25:13</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>-33.4761066, -70.6985216</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>-33.47611, -70.69852</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>2026/07/08 23:25:37</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>-33.4761066, -70.6985216</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>-33.47611, -70.69852</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>02:00:24</t>
+        </is>
+      </c>
+      <c r="L170" t="n">
+        <v>0</v>
+      </c>
+      <c r="M170" t="n">
+        <v>0</v>
+      </c>
+      <c r="N170" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>12</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>2026/07/08 21:39:36</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>-32.838381, -70.955498</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>-32.83838, -70.95550</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>2026/07/08 23:38:05</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>-32.838381, -70.955498</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>-32.83838, -70.95550</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>01:58:29</t>
+        </is>
+      </c>
+      <c r="L171" t="n">
+        <v>0</v>
+      </c>
+      <c r="M171" t="n">
+        <v>0</v>
+      </c>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>12</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>2026/07/08 21:43:27</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>-32.841869, -70.9368</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>-32.84187, -70.93680</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>2026/07/08 23:46:39</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>-32.841869, -70.9368</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>-32.84187, -70.93680</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>02:03:12</t>
+        </is>
+      </c>
+      <c r="L172" t="n">
+        <v>0</v>
+      </c>
+      <c r="M172" t="n">
+        <v>0</v>
+      </c>
+      <c r="N172" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10428,13 +10605,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1333.79</v>
+        <v>1333.77</v>
       </c>
       <c r="C5" t="n">
         <v>59</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
         <v>134</v>
@@ -10599,13 +10776,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1198.45</v>
+        <v>1198.43</v>
       </c>
       <c r="C14" t="n">
         <v>65</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>122</v>
@@ -10618,13 +10795,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>334.53</v>
+        <v>334.4</v>
       </c>
       <c r="C15" t="n">
         <v>48</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>134</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-10T07:33Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/09 22:23:56</t>
+          <t>2026/07/09 23:23:56</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:27:44</t>
+          <t>166:27:44</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>2026/07/09 21:02:21</t>
+          <t>2026/07/09 23:02:21</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>12:00:00</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>2026/07/09 21:09:50</t>
+          <t>2026/07/09 23:09:50</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -10546,7 +10546,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>04:18:03</t>
+          <t>06:18:03</t>
         </is>
       </c>
       <c r="L173" t="n">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>2026/07/09 22:06:46</t>
+          <t>2026/07/09 23:06:46</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>05:01:00</t>
+          <t>06:01:00</t>
         </is>
       </c>
       <c r="L175" t="n">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>2026/07/09 22:14:38</t>
+          <t>2026/07/09 23:14:22</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -10723,7 +10723,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>05:00:16</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L176" t="n">
@@ -10767,7 +10767,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>2026/07/09 22:20:44</t>
+          <t>2026/07/09 23:21:36</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>05:01:10</t>
+          <t>06:02:02</t>
         </is>
       </c>
       <c r="L177" t="n">
@@ -10826,7 +10826,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>2026/07/09 22:25:55</t>
+          <t>2026/07/09 23:25:54</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -10841,7 +10841,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>05:00:29</t>
+          <t>06:00:28</t>
         </is>
       </c>
       <c r="L178" t="n">
@@ -10885,7 +10885,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>2026/07/09 21:15:28</t>
+          <t>2026/07/09 23:15:28</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -10900,7 +10900,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L179" t="n">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>2026/07/09 22:37:24</t>
+          <t>2026/07/09 23:37:23</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>02:57:32</t>
+          <t>03:57:31</t>
         </is>
       </c>
       <c r="L180" t="n">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>2026/07/09 22:40:50</t>
+          <t>2026/07/09 23:40:50</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -11136,7 +11136,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>02:03:05</t>
+          <t>03:03:05</t>
         </is>
       </c>
       <c r="L183" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-11T06:11Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N177"/>
+  <dimension ref="A1:N181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/07/10 22:23:56</t>
+          <t>2026/07/10 23:23:56</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>165:27:44</t>
+          <t>166:27:44</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>2026/07/10 21:02:21</t>
+          <t>2026/07/10 23:02:21</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>36:00:00</t>
+          <t>38:00:00</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/07/10 22:14:21</t>
+          <t>2026/07/10 23:14:41</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>28:59:59</t>
+          <t>30:00:19</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2026/07/10 22:25:47</t>
+          <t>2026/07/10 23:25:55</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>29:00:21</t>
+          <t>30:00:29</t>
         </is>
       </c>
       <c r="L165" t="n">
@@ -10295,7 +10295,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>2026/07/10 20:48:31</t>
+          <t>2026/07/10 22:48:31</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L169" t="n">
@@ -10472,7 +10472,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>2026/07/10 20:39:24</t>
+          <t>2026/07/10 22:39:24</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>02:25:58</t>
+          <t>04:25:58</t>
         </is>
       </c>
       <c r="L172" t="n">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>2026/07/10 20:33:19</t>
+          <t>2026/07/10 22:33:19</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -10546,7 +10546,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>02:01:50</t>
+          <t>04:01:50</t>
         </is>
       </c>
       <c r="L173" t="n">
@@ -10680,70 +10680,70 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>2026/07/10 21:20:30</t>
+          <t>2026/07/10 20:32:07</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>-33.4551016, -70.6583816</t>
+          <t>-32.7431766, -70.7296583</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>-33.45510, -70.65838</t>
+          <t>-32.74318, -70.72966</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>2026/07/10 21:46:39</t>
+          <t>2026/07/10 22:33:51</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>-33.4763316, -70.6984033</t>
+          <t>-32.7430183, -70.7297866</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>-33.47633, -70.69840</t>
+          <t>-32.74302, -70.72979</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>00:26:09</t>
+          <t>02:01:44</t>
         </is>
       </c>
       <c r="L176" t="n">
-        <v>7.12</v>
+        <v>0.02</v>
       </c>
       <c r="M176" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="N176" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+          <t>SUZUKI CARRY SKDB-52</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
@@ -10752,47 +10752,283 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2026/07/10 21:32:29</t>
+          <t>2026/07/10 20:51:15</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>-33.484898, -70.77242</t>
+          <t>-32.8794316, -70.6088516</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>-33.48490, -70.77242</t>
+          <t>-32.87943, -70.60885</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>2026/07/10 21:44:07</t>
+          <t>2026/07/10 22:52:59</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>-33.484898, -70.77242</t>
+          <t>-32.879205, -70.6088216</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>-33.48490, -70.77242</t>
+          <t>-32.87920, -70.60882</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>00:11:38</t>
+          <t>02:01:44</t>
         </is>
       </c>
       <c r="L177" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="M177" t="n">
         <v>0</v>
       </c>
       <c r="N177" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>16</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>2026/07/10 21:20:30</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>-33.4551016, -70.6583816</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>-33.45510, -70.65838</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>2026/07/10 21:46:26</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>-33.476, -70.6980066</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>-33.47600, -70.69801</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>00:25:56</t>
+        </is>
+      </c>
+      <c r="L178" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="M178" t="n">
+        <v>57</v>
+      </c>
+      <c r="N178" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>8</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>2026/07/10 21:35:16</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>-32.838379, -70.95552</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>-32.83838, -70.95552</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>2026/07/10 23:32:50</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>-32.838379, -70.95552</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>-32.83838, -70.95552</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>01:57:34</t>
+        </is>
+      </c>
+      <c r="L179" t="n">
+        <v>0</v>
+      </c>
+      <c r="M179" t="n">
+        <v>0</v>
+      </c>
+      <c r="N179" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>17</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>2026/07/10 21:46:39</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>-33.4763316, -70.6984033</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>-33.47633, -70.69840</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>2026/07/10 22:53:16</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>-33.49691, -70.7077533</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>-33.49691, -70.70775</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>01:06:37</t>
+        </is>
+      </c>
+      <c r="L180" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M180" t="n">
+        <v>64</v>
+      </c>
+      <c r="N180" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>18</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>2026/07/10 22:53:31</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>-33.497, -70.7076666</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>-33.49700, -70.70767</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>2026/07/10 23:11:43</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>-33.4761216, -70.6985266</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>-33.47612, -70.69853</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>00:18:12</t>
+        </is>
+      </c>
+      <c r="L181" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="M181" t="n">
+        <v>48</v>
+      </c>
+      <c r="N181" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -10862,13 +11098,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1429.13</v>
+        <v>1429.09</v>
       </c>
       <c r="C3" t="n">
         <v>62</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
         <v>145</v>
@@ -10900,13 +11136,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1366.1</v>
+        <v>1366.07</v>
       </c>
       <c r="C5" t="n">
         <v>43</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
         <v>134</v>
@@ -11071,10 +11307,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1030.83</v>
+        <v>1039.87</v>
       </c>
       <c r="C14" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -11166,13 +11402,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1441.48</v>
+        <v>1440.96</v>
       </c>
       <c r="C19" t="n">
         <v>79</v>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
         <v>139</v>
@@ -11185,13 +11421,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>808.5700000000001</v>
+        <v>812.13</v>
       </c>
       <c r="C20" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
         <v>144</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-12T06:31Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N184"/>
+  <dimension ref="A1:N183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026/07/11 22:23:56</t>
+          <t>2026/07/11 23:23:56</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>165:27:47</t>
+          <t>166:27:47</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/07/11 21:02:21</t>
+          <t>2026/07/11 23:02:21</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>60:00:00</t>
+          <t>62:00:00</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026/07/11 22:14:22</t>
+          <t>2026/07/11 23:14:22</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>53:00:00</t>
+          <t>54:00:00</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2026/07/11 22:25:54</t>
+          <t>2026/07/11 23:25:26</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>53:00:28</t>
+          <t>54:00:00</t>
         </is>
       </c>
       <c r="L165" t="n">
@@ -10354,7 +10354,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>2026/07/11 20:48:31</t>
+          <t>2026/07/11 22:48:31</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>28:00:00</t>
+          <t>30:00:00</t>
         </is>
       </c>
       <c r="L170" t="n">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026/07/11 20:47:44</t>
+          <t>2026/07/11 22:47:44</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>02:01:06</t>
+          <t>04:01:06</t>
         </is>
       </c>
       <c r="L181" t="n">
@@ -11034,11 +11034,11 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCL-70</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
@@ -11047,37 +11047,37 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>2026/07/11 18:52:27</t>
+          <t>2026/07/11 19:13:18</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>-32.838398, -70.95549</t>
+          <t>-33.4761183, -70.6984916</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>-32.83840, -70.95549</t>
+          <t>-33.47612, -70.69849</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>2026/07/11 21:49:58</t>
+          <t>2026/07/11 23:13:18</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>-32.838398, -70.95549</t>
+          <t>-33.4761183, -70.6984916</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>-32.83840, -70.95549</t>
+          <t>-33.47612, -70.69849</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>02:57:31</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L182" t="n">
@@ -11093,11 +11093,11 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
@@ -11106,37 +11106,37 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>2026/07/11 19:13:18</t>
+          <t>2026/07/11 21:25:31</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>-33.4761183, -70.6984916</t>
+          <t>-32.841755, -70.936878</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>-33.47612, -70.69849</t>
+          <t>-32.84175, -70.93688</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>2026/07/11 21:13:18</t>
+          <t>2026/07/11 23:28:31</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>-33.4761183, -70.6984916</t>
+          <t>-32.841755, -70.936878</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>-33.47612, -70.69849</t>
+          <t>-32.84175, -70.93688</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>02:03:00</t>
         </is>
       </c>
       <c r="L183" t="n">
@@ -11146,65 +11146,6 @@
         <v>0</v>
       </c>
       <c r="N183" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>VOLKSWAGEN AMAROK KPDV-13</t>
-        </is>
-      </c>
-      <c r="C184" t="n">
-        <v>11</v>
-      </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>Paradas</t>
-        </is>
-      </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>2026/07/11 21:25:31</t>
-        </is>
-      </c>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>-32.841755, -70.936878</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>-32.84175, -70.93688</t>
-        </is>
-      </c>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>2026/07/11 22:28:31</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>-32.841755, -70.936878</t>
-        </is>
-      </c>
-      <c r="J184" t="inlineStr">
-        <is>
-          <t>-32.84175, -70.93688</t>
-        </is>
-      </c>
-      <c r="K184" t="inlineStr">
-        <is>
-          <t>01:03:00</t>
-        </is>
-      </c>
-      <c r="L184" t="n">
-        <v>0</v>
-      </c>
-      <c r="M184" t="n">
-        <v>0</v>
-      </c>
-      <c r="N184" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11275,13 +11216,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1307.7</v>
+        <v>1331.58</v>
       </c>
       <c r="C3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>145</v>
@@ -11579,10 +11520,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1495.03</v>
+        <v>1500.04</v>
       </c>
       <c r="C19" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D19" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-13T06:51Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N184"/>
+  <dimension ref="A1:N185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/12 21:56:10</t>
+          <t>2026/07/12 23:56:10</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/07/12 21:02:21</t>
+          <t>2026/07/12 23:02:21</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>84:00:00</t>
+          <t>86:00:00</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -10354,7 +10354,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>2026/07/12 22:31:40</t>
+          <t>2026/07/12 23:31:39</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>77:06:14</t>
+          <t>78:06:13</t>
         </is>
       </c>
       <c r="L170" t="n">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>2026/07/12 20:48:31</t>
+          <t>2026/07/12 22:48:31</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -10546,7 +10546,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>52:00:00</t>
+          <t>54:00:00</t>
         </is>
       </c>
       <c r="L173" t="n">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026/07/12 20:39:59</t>
+          <t>2026/07/12 22:39:59</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>04:46:47</t>
+          <t>06:46:47</t>
         </is>
       </c>
       <c r="L181" t="n">
@@ -11062,7 +11062,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>2026/07/12 21:09:47</t>
+          <t>2026/07/12 23:09:47</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -11077,7 +11077,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>04:00:06</t>
+          <t>06:00:06</t>
         </is>
       </c>
       <c r="L182" t="n">
@@ -11205,6 +11205,65 @@
         <v>0</v>
       </c>
       <c r="N184" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>6</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>2026/07/12 21:52:01</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>-32.841676, -70.936803</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>-32.84168, -70.93680</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>2026/07/12 23:55:01</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>-32.841676, -70.936803</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>-32.84168, -70.93680</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>02:03:00</t>
+        </is>
+      </c>
+      <c r="L185" t="n">
+        <v>0</v>
+      </c>
+      <c r="M185" t="n">
+        <v>0</v>
+      </c>
+      <c r="N185" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11275,7 +11334,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1530.9</v>
+        <v>1531.1</v>
       </c>
       <c r="C3" t="n">
         <v>56</v>
@@ -11598,13 +11657,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>894.38</v>
+        <v>894.36</v>
       </c>
       <c r="C20" t="n">
         <v>73</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>144</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-14T06:09Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N175"/>
+  <dimension ref="A1:N178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/07/13 21:56:10</t>
+          <t>2026/07/13 23:56:10</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>164:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/07/13 21:34:31</t>
+          <t>2026/07/13 23:34:38</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>139:00:10</t>
+          <t>141:00:17</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -8938,7 +8938,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/07/13 21:02:21</t>
+          <t>2026/07/13 23:02:21</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>108:00:00</t>
+          <t>110:00:00</t>
         </is>
       </c>
       <c r="L146" t="n">
@@ -9528,7 +9528,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>2026/07/13 21:31:38</t>
+          <t>2026/07/13 23:31:18</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>100:06:12</t>
+          <t>102:05:52</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -10413,7 +10413,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>2026/07/13 21:48:19</t>
+          <t>2026/07/13 23:48:22</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>04:03:00</t>
+          <t>06:03:03</t>
         </is>
       </c>
       <c r="L171" t="n">
@@ -10472,7 +10472,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>2026/07/13 21:14:34</t>
+          <t>2026/07/13 23:14:34</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>02:00:23</t>
+          <t>04:00:23</t>
         </is>
       </c>
       <c r="L172" t="n">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>2026/07/13 21:15:19</t>
+          <t>2026/07/13 23:15:19</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -10546,7 +10546,7 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L173" t="n">
@@ -10590,7 +10590,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>2026/07/13 21:55:48</t>
+          <t>2026/07/13 23:55:48</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -10605,7 +10605,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L174" t="n">
@@ -10649,7 +10649,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>2026/07/13 21:59:32</t>
+          <t>2026/07/13 23:59:32</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L175" t="n">
@@ -10674,6 +10674,183 @@
         <v>0</v>
       </c>
       <c r="N175" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>6</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>2026/07/13 20:25:42</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>-32.838362, -70.955504</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95550</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>2026/07/13 23:23:11</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>-32.838362, -70.955504</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95550</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>02:57:29</t>
+        </is>
+      </c>
+      <c r="L176" t="n">
+        <v>0</v>
+      </c>
+      <c r="M176" t="n">
+        <v>0</v>
+      </c>
+      <c r="N176" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCS-53</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>12</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>2026/07/13 20:29:15</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>-33.0873083, -71.3623783</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>-33.08731, -71.36238</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>2026/07/13 22:29:15</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>-33.0873083, -71.3623783</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>-33.08731, -71.36238</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L177" t="n">
+        <v>0</v>
+      </c>
+      <c r="M177" t="n">
+        <v>0</v>
+      </c>
+      <c r="N177" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>7</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>2026/07/13 21:25:42</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>-33.4364766, -70.6295866</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>-33.43648, -70.62959</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>2026/07/13 23:25:42</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>-33.4364766, -70.6295866</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>-33.43648, -70.62959</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L178" t="n">
+        <v>0</v>
+      </c>
+      <c r="M178" t="n">
+        <v>0</v>
+      </c>
+      <c r="N178" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10750,7 +10927,7 @@
         <v>55</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>145</v>
@@ -10763,13 +10940,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1007.38</v>
+        <v>1007.37</v>
       </c>
       <c r="C4" t="n">
         <v>67</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>138</v>
@@ -10972,13 +11149,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>389.52</v>
+        <v>389.49</v>
       </c>
       <c r="C15" t="n">
         <v>27</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>134</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-15T06:12Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N168"/>
+  <dimension ref="A1:N169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/14 21:56:11</t>
+          <t>2026/07/14 23:56:11</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>165:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026/07/14 21:35:26</t>
+          <t>2026/07/14 23:36:40</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>163:01:05</t>
+          <t>165:02:19</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -4013,70 +4013,70 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>SUZUKI CARRY SKDB-52</t>
         </is>
       </c>
       <c r="C63" t="n">
+        <v>9</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026/07/08 12:27:27</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>-34.2050183, -70.678095</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>-34.20502, -70.67809</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2026/07/08 12:41:16</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>-34.2047983, -70.67986</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>-34.20480, -70.67986</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>00:13:49</t>
+        </is>
+      </c>
+      <c r="L63" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="M63" t="n">
+        <v>13</v>
+      </c>
+      <c r="N63" t="n">
         <v>8</v>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Recorridos</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>2026/07/08 12:27:27</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>-33.1345533, -71.5637166</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>-33.13455, -71.56372</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>2026/07/08 13:11:21</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>-33.0873083, -71.3622866</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>-33.08731, -71.36229</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>00:43:54</t>
-        </is>
-      </c>
-      <c r="L63" t="n">
-        <v>43.73</v>
-      </c>
-      <c r="M63" t="n">
-        <v>125</v>
-      </c>
-      <c r="N63" t="n">
-        <v>59</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -4090,42 +4090,42 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>-34.2050183, -70.678095</t>
+          <t>-33.1345533, -71.5637166</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>-34.20502, -70.67809</t>
+          <t>-33.13455, -71.56372</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>2026/07/08 12:41:16</t>
+          <t>2026/07/08 13:11:21</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>-34.2047983, -70.67986</t>
+          <t>-33.0873083, -71.3622866</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>-34.20480, -70.67986</t>
+          <t>-33.08731, -71.36229</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>00:13:49</t>
+          <t>00:43:54</t>
         </is>
       </c>
       <c r="L64" t="n">
-        <v>0.38</v>
+        <v>43.73</v>
       </c>
       <c r="M64" t="n">
-        <v>13</v>
+        <v>125</v>
       </c>
       <c r="N64" t="n">
-        <v>8</v>
+        <v>59</v>
       </c>
     </row>
     <row r="65">
@@ -7817,7 +7817,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>2026/07/14 21:25:48</t>
+          <t>2026/07/14 23:25:22</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7832,7 +7832,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>136:31:55</t>
+          <t>138:31:29</t>
         </is>
       </c>
       <c r="L127" t="n">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026/07/14 21:57:19</t>
+          <t>2026/07/14 23:57:15</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>137:01:46</t>
+          <t>139:01:42</t>
         </is>
       </c>
       <c r="L128" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/07/14 21:02:21</t>
+          <t>2026/07/14 23:02:21</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>132:00:00</t>
+          <t>134:00:00</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8938,7 +8938,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/07/14 21:31:23</t>
+          <t>2026/07/14 23:31:38</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>124:05:57</t>
+          <t>126:06:12</t>
         </is>
       </c>
       <c r="L146" t="n">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026/07/14 20:33:04</t>
+          <t>2026/07/14 22:33:04</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>02:09:54</t>
+          <t>04:09:54</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/07/14 21:51:39</t>
+          <t>2026/07/14 23:51:39</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>03:03:06</t>
+          <t>05:03:06</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2026/07/14 21:28:08</t>
+          <t>2026/07/14 23:28:08</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>02:00:12</t>
+          <t>04:00:12</t>
         </is>
       </c>
       <c r="L165" t="n">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>2026/07/14 21:29:22</t>
+          <t>2026/07/14 23:29:22</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>02:00:06</t>
+          <t>04:00:06</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026/07/14 21:43:30</t>
+          <t>2026/07/14 23:43:30</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L167" t="n">
@@ -10261,6 +10261,65 @@
         <v>0</v>
       </c>
       <c r="N168" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>3</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>2026/07/14 20:50:47</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>-32.838363, -70.95554</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95554</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>2026/07/14 23:48:19</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>-32.838363, -70.95554</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95554</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>02:57:32</t>
+        </is>
+      </c>
+      <c r="L169" t="n">
+        <v>0</v>
+      </c>
+      <c r="M169" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10331,13 +10390,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1381.92</v>
+        <v>1381.91</v>
       </c>
       <c r="C3" t="n">
         <v>52</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>145</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-15T20:58Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -4013,11 +4013,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -4031,101 +4031,101 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>-34.2050183, -70.678095</t>
+          <t>-33.1345533, -71.5637166</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>-34.20502, -70.67809</t>
+          <t>-33.13455, -71.56372</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>2026/07/08 12:41:16</t>
+          <t>2026/07/08 13:11:21</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>-34.2047983, -70.67986</t>
+          <t>-33.0873083, -71.3622866</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>-34.20480, -70.67986</t>
+          <t>-33.08731, -71.36229</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>00:13:49</t>
+          <t>00:43:54</t>
         </is>
       </c>
       <c r="L63" t="n">
-        <v>0.38</v>
+        <v>43.73</v>
       </c>
       <c r="M63" t="n">
-        <v>13</v>
+        <v>125</v>
       </c>
       <c r="N63" t="n">
-        <v>8</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>SUZUKI CARRY SKDB-52</t>
         </is>
       </c>
       <c r="C64" t="n">
+        <v>9</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026/07/08 12:27:27</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>-34.2050183, -70.678095</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>-34.20502, -70.67809</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026/07/08 12:41:16</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>-34.2047983, -70.67986</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>-34.20480, -70.67986</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>00:13:49</t>
+        </is>
+      </c>
+      <c r="L64" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="M64" t="n">
+        <v>13</v>
+      </c>
+      <c r="N64" t="n">
         <v>8</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Recorridos</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>2026/07/08 12:27:27</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>-33.1345533, -71.5637166</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>-33.13455, -71.56372</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>2026/07/08 13:11:21</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>-33.0873083, -71.3622866</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>-33.08731, -71.36229</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>00:43:54</t>
-        </is>
-      </c>
-      <c r="L64" t="n">
-        <v>43.73</v>
-      </c>
-      <c r="M64" t="n">
-        <v>125</v>
-      </c>
-      <c r="N64" t="n">
-        <v>59</v>
       </c>
     </row>
     <row r="65">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-16T06:16Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N161"/>
+  <dimension ref="A1:N165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/07/15 21:56:11</t>
+          <t>2026/07/15 23:56:11</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>162:17:15</t>
+          <t>164:17:15</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/15 21:35:06</t>
+          <t>2026/07/15 23:36:26</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>161:50:11</t>
+          <t>163:51:31</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026/07/15 22:24:46</t>
+          <t>2026/07/15 23:25:59</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>161:30:53</t>
+          <t>162:32:06</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026/07/15 21:57:24</t>
+          <t>2026/07/15 23:57:16</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>161:01:51</t>
+          <t>163:01:43</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>2026/07/15 21:02:21</t>
+          <t>2026/07/15 23:02:21</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>156:00:00</t>
+          <t>158:00:00</t>
         </is>
       </c>
       <c r="L40" t="n">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>2026/07/15 22:13:14</t>
+          <t>2026/07/15 23:13:37</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>148:58:51</t>
+          <t>149:59:14</t>
         </is>
       </c>
       <c r="L108" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>2026/07/15 21:31:21</t>
+          <t>2026/07/15 23:31:21</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>148:05:55</t>
+          <t>150:05:55</t>
         </is>
       </c>
       <c r="L110" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/07/15 21:41:32</t>
+          <t>2026/07/15 23:39:24</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>89:02:14</t>
+          <t>91:00:06</t>
         </is>
       </c>
       <c r="L145" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/07/15 21:12:02</t>
+          <t>2026/07/15 23:12:02</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>02:08:22</t>
+          <t>04:08:22</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/07/15 22:07:57</t>
+          <t>2026/07/15 23:07:57</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>02:57:56</t>
+          <t>03:57:56</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/07/15 21:20:18</t>
+          <t>2026/07/15 23:20:18</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -9823,22 +9823,22 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>2026/07/15 21:35:22</t>
+          <t>2026/07/15 21:31:52</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>-32.841741, -70.936882</t>
+          <t>-32.841759, -70.936896</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>-32.84174, -70.93688</t>
+          <t>-32.84176, -70.93690</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>01:32:41</t>
+          <t>01:29:11</t>
         </is>
       </c>
       <c r="L161" t="n">
@@ -9849,6 +9849,242 @@
       </c>
       <c r="N161" t="n">
         <v>21</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>16</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>2026/07/15 20:51:39</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>-33.4761616, -70.698455</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>-33.47616, -70.69845</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>2026/07/15 22:56:09</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>-33.4761616, -70.698455</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>-33.47616, -70.69845</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>02:04:30</t>
+        </is>
+      </c>
+      <c r="L162" t="n">
+        <v>0</v>
+      </c>
+      <c r="M162" t="n">
+        <v>0</v>
+      </c>
+      <c r="N162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>5</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>2026/07/15 21:16:54</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>-32.743215, -70.7296266</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>-32.74321, -70.72963</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>2026/07/15 23:21:50</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>-32.7430133, -70.72982</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>-32.74301, -70.72982</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>02:04:56</t>
+        </is>
+      </c>
+      <c r="L163" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M163" t="n">
+        <v>0</v>
+      </c>
+      <c r="N163" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>15</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>2026/07/15 21:32:18</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>-32.841741, -70.936882</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>-32.84174, -70.93688</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>2026/07/15 23:35:22</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>-32.841741, -70.936882</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>-32.84174, -70.93688</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>02:03:04</t>
+        </is>
+      </c>
+      <c r="L164" t="n">
+        <v>0</v>
+      </c>
+      <c r="M164" t="n">
+        <v>0</v>
+      </c>
+      <c r="N164" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>6</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>2026/07/15 21:41:29</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>-33.4364349, -70.6291566</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>-33.43643, -70.62916</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>2026/07/15 23:42:00</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>-33.4364349, -70.6291566</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>-33.43643, -70.62916</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>02:00:31</t>
+        </is>
+      </c>
+      <c r="L165" t="n">
+        <v>0</v>
+      </c>
+      <c r="M165" t="n">
+        <v>0</v>
+      </c>
+      <c r="N165" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -9956,13 +10192,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1108.19</v>
+        <v>1108.15</v>
       </c>
       <c r="C5" t="n">
         <v>33</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>134</v>
@@ -10127,13 +10363,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1082.46</v>
+        <v>1082.44</v>
       </c>
       <c r="C14" t="n">
         <v>79</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>128</v>
@@ -10146,13 +10382,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>402.94</v>
+        <v>402.9</v>
       </c>
       <c r="C15" t="n">
         <v>25</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>124</v>
@@ -10241,13 +10477,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>842.54</v>
+        <v>842.53</v>
       </c>
       <c r="C20" t="n">
         <v>74</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>144</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-17T06:13Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/07/16 22:13:16</t>
+          <t>2026/07/16 23:13:38</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>165:58:56</t>
+          <t>166:59:18</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/07/16 21:35:30</t>
+          <t>2026/07/16 23:34:30</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>165:21:07</t>
+          <t>167:20:07</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/07/16 22:24:08</t>
+          <t>2026/07/16 23:23:39</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>166:08:03</t>
+          <t>167:07:34</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/07/16 21:57:55</t>
+          <t>2026/07/16 23:57:29</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>165:41:46</t>
+          <t>167:41:20</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/07/16 21:56:09</t>
+          <t>2026/07/16 23:56:09</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>165:32:13</t>
+          <t>167:32:13</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/07/16 21:31:38</t>
+          <t>2026/07/16 23:31:21</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:06:04</t>
+          <t>167:05:47</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026/07/16 21:02:21</t>
+          <t>2026/07/16 23:02:21</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>164:00:00</t>
+          <t>166:00:00</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/07/16 21:41:06</t>
+          <t>2026/07/16 23:41:06</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>113:01:48</t>
+          <t>115:01:48</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/07/16 21:12:02</t>
+          <t>2026/07/16 23:12:02</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>26:08:22</t>
+          <t>28:08:22</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/07/16 20:56:09</t>
+          <t>2026/07/16 22:56:09</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>24:04:30</t>
+          <t>26:04:30</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/07/16 21:42:00</t>
+          <t>2026/07/16 23:42:00</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>24:00:31</t>
+          <t>26:00:31</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/07/16 21:33:47</t>
+          <t>2026/07/16 23:33:50</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>09:03:08</t>
+          <t>11:03:11</t>
         </is>
       </c>
       <c r="L145" t="n">
@@ -8938,7 +8938,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/07/16 22:21:39</t>
+          <t>2026/07/16 23:21:40</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>01:57:31</t>
+          <t>02:57:32</t>
         </is>
       </c>
       <c r="L146" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-18T06:03Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N132"/>
+  <dimension ref="A1:N133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,7 +619,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/07/17 22:13:37</t>
+          <t>2026/07/17 23:13:21</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>165:59:27</t>
+          <t>166:59:11</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/07/17 21:35:07</t>
+          <t>2026/07/17 23:34:55</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>165:20:52</t>
+          <t>167:20:40</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/07/17 21:24:04</t>
+          <t>2026/07/17 23:23:38</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>165:08:35</t>
+          <t>167:08:09</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/07/17 21:57:27</t>
+          <t>2026/07/17 23:57:30</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>165:41:18</t>
+          <t>167:41:21</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/07/17 21:56:09</t>
+          <t>2026/07/17 23:56:09</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>165:32:13</t>
+          <t>167:32:13</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/07/17 21:31:24</t>
+          <t>2026/07/17 23:31:22</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>165:05:57</t>
+          <t>167:05:55</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026/07/17 21:02:21</t>
+          <t>2026/07/17 23:02:21</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>164:00:00</t>
+          <t>166:00:00</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -4690,7 +4690,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>2026/07/17 21:39:23</t>
+          <t>2026/07/17 23:41:06</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>137:00:05</t>
+          <t>139:01:48</t>
         </is>
       </c>
       <c r="L74" t="n">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>2026/07/17 20:24:22</t>
+          <t>2026/07/17 22:24:22</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>50:00:12</t>
+          <t>52:00:12</t>
         </is>
       </c>
       <c r="L116" t="n">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/07/17 21:12:02</t>
+          <t>2026/07/17 23:12:02</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>50:08:22</t>
+          <t>52:08:22</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/07/17 22:21:15</t>
+          <t>2026/07/17 23:29:49</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>49:04:21</t>
+          <t>50:12:55</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026/07/17 20:50:36</t>
+          <t>2026/07/17 22:50:36</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>08:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="L128" t="n">
@@ -7935,7 +7935,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>2026/07/17 21:40:40</t>
+          <t>2026/07/17 23:40:40</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>06:03:07</t>
+          <t>08:03:07</t>
         </is>
       </c>
       <c r="L129" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/07/17 21:49:25</t>
+          <t>2026/07/17 23:49:25</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/07/17 21:49:36</t>
+          <t>2026/07/17 23:49:37</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>02:57:30</t>
+          <t>04:57:31</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8137,6 +8137,65 @@
         <v>0</v>
       </c>
       <c r="N132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>5</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2026/07/17 21:10:52</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>-33.4761016, -70.6985316</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>-33.47610, -70.69853</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>2026/07/17 23:13:07</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>-33.4761466, -70.6985149</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>-33.47615, -70.69851</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>02:02:15</t>
+        </is>
+      </c>
+      <c r="L133" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M133" t="n">
+        <v>0</v>
+      </c>
+      <c r="N133" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8416,13 +8475,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>888.86</v>
+        <v>888.84</v>
       </c>
       <c r="C14" t="n">
         <v>56</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>128</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-19T06:28Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/07/18 21:34:34</t>
+          <t>2026/07/18 23:34:36</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>165:20:18</t>
+          <t>167:20:20</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/07/18 22:13:24</t>
+          <t>2026/07/18 23:13:38</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>165:59:04</t>
+          <t>166:59:18</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/07/18 22:24:44</t>
+          <t>2026/07/18 23:24:07</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>166:08:17</t>
+          <t>167:07:40</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/07/18 21:57:21</t>
+          <t>2026/07/18 23:57:22</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>165:40:45</t>
+          <t>167:40:46</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/07/18 21:56:11</t>
+          <t>2026/07/18 23:56:11</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>165:32:15</t>
+          <t>167:32:15</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/07/18 22:31:37</t>
+          <t>2026/07/18 23:31:38</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:05:44</t>
+          <t>167:05:45</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026/07/18 22:01:29</t>
+          <t>2026/07/18 23:01:38</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>164:00:01</t>
+          <t>165:00:10</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026/07/18 22:11:21</t>
+          <t>2026/07/18 23:11:22</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>163:59:07</t>
+          <t>164:59:08</t>
         </is>
       </c>
       <c r="L25" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026/07/18 21:40:20</t>
+          <t>2026/07/18 23:40:44</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>161:01:02</t>
+          <t>163:01:26</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -7758,22 +7758,22 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/07/18 22:32:46</t>
+          <t>2026/07/18 23:59:01</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>-32.7429766, -70.7298116</t>
+          <t>-32.7430016, -70.7298083</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>-32.74298, -70.72981</t>
+          <t>-32.74300, -70.72981</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>73:15:52</t>
+          <t>74:42:07</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -7935,7 +7935,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>2026/07/18 21:49:25</t>
+          <t>2026/07/18 23:49:25</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>28:00:00</t>
+          <t>30:00:00</t>
         </is>
       </c>
       <c r="L129" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/07/18 21:42:39</t>
+          <t>2026/07/18 23:42:39</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/07/18 21:10:35</t>
+          <t>2026/07/18 23:10:35</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>08:02:02</t>
+          <t>10:02:02</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/07/18 22:26:36</t>
+          <t>2026/07/18 23:26:36</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>09:03:06</t>
+          <t>10:03:06</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026/07/18 21:04:34</t>
+          <t>2026/07/18 23:04:34</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L135" t="n">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/07/18 21:55:00</t>
+          <t>2026/07/18 23:55:00</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>02:00:02</t>
+          <t>04:00:02</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/07/18 22:16:44</t>
+          <t>2026/07/18 23:16:44</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>01:57:30</t>
+          <t>02:57:30</t>
         </is>
       </c>
       <c r="L137" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-20T06:44Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/07/19 22:23:34</t>
+          <t>2026/07/19 23:23:39</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>166:00:36</t>
+          <t>167:00:41</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/07/19 22:31:37</t>
+          <t>2026/07/19 23:31:38</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>166:00:17</t>
+          <t>167:00:18</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/07/19 22:34:34</t>
+          <t>2026/07/19 23:34:30</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>165:59:49</t>
+          <t>166:59:45</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/07/19 22:40:44</t>
+          <t>2026/07/19 23:40:44</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:01:07</t>
+          <t>167:01:07</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/07/19 22:56:11</t>
+          <t>2026/07/19 23:56:11</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>166:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026/07/19 22:57:38</t>
+          <t>2026/07/19 23:57:22</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>165:59:47</t>
+          <t>166:59:31</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/07/19 21:42:39</t>
+          <t>2026/07/19 23:42:39</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>34:00:00</t>
+          <t>36:00:00</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/07/19 21:55:08</t>
+          <t>2026/07/19 23:55:08</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>06:02:29</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/07/19 21:24:58</t>
+          <t>2026/07/19 23:24:58</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>02:01:43</t>
+          <t>04:01:43</t>
         </is>
       </c>
       <c r="L134" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-21T06:26Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N127"/>
+  <dimension ref="A1:N128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/20 22:01:40</t>
+          <t>2026/07/20 23:01:20</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:59:17</t>
+          <t>166:58:57</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -619,7 +619,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/07/20 22:11:25</t>
+          <t>2026/07/20 23:11:39</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>165:58:59</t>
+          <t>166:59:13</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/07/20 22:13:14</t>
+          <t>2026/07/20 23:13:31</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>165:59:53</t>
+          <t>167:00:10</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/07/20 22:24:57</t>
+          <t>2026/07/20 23:24:01</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>166:01:49</t>
+          <t>167:00:53</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/07/20 21:31:51</t>
+          <t>2026/07/20 23:32:12</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>165:00:13</t>
+          <t>167:00:34</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/07/20 21:34:24</t>
+          <t>2026/07/20 23:34:52</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>164:59:32</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/07/20 21:56:10</t>
+          <t>2026/07/20 23:56:10</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>165:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/07/20 21:57:31</t>
+          <t>2026/07/20 23:57:38</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>164:58:22</t>
+          <t>166:58:29</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026/07/20 21:42:39</t>
+          <t>2026/07/20 23:42:39</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>58:00:00</t>
+          <t>60:00:00</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/07/20 21:39:03</t>
+          <t>2026/07/20 23:39:23</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>18:59:38</t>
+          <t>20:59:58</t>
         </is>
       </c>
       <c r="L119" t="n">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/07/20 21:28:49</t>
+          <t>2026/07/20 23:28:49</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>07:30:49</t>
+          <t>09:30:49</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/07/20 22:00:00</t>
+          <t>2026/07/20 23:00:03</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>05:03:21</t>
+          <t>06:03:24</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/07/20 21:40:29</t>
+          <t>2026/07/20 23:40:29</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>02:00:25</t>
+          <t>04:00:25</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -7842,6 +7842,65 @@
         <v>0</v>
       </c>
       <c r="N127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>5</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2026/07/20 20:35:17</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>-33.4371483, -70.6294466</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>-33.43715, -70.62945</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>2026/07/20 22:36:07</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>-33.43715, -70.629445</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>-33.43715, -70.62945</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>02:00:50</t>
+        </is>
+      </c>
+      <c r="L128" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7912,7 +7971,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>325.5</v>
+        <v>339.69</v>
       </c>
       <c r="C3" t="n">
         <v>34</v>
@@ -8140,13 +8199,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>235.3</v>
+        <v>235.14</v>
       </c>
       <c r="C15" t="n">
         <v>24</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>120</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-22T06:26Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N126"/>
+  <dimension ref="A1:N128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/21 22:01:21</t>
+          <t>2026/07/21 23:01:39</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:59:44</t>
+          <t>167:00:02</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/07/21 22:11:23</t>
+          <t>2026/07/21 23:11:21</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>165:59:55</t>
+          <t>166:59:53</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/07/21 22:13:39</t>
+          <t>2026/07/21 23:13:15</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>166:00:18</t>
+          <t>166:59:54</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/07/21 22:24:37</t>
+          <t>2026/07/21 23:24:09</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>165:58:25</t>
+          <t>166:57:57</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/07/21 21:31:51</t>
+          <t>2026/07/21 23:32:03</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>165:00:30</t>
+          <t>167:00:42</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/07/21 21:34:57</t>
+          <t>2026/07/21 23:34:53</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>164:59:53</t>
+          <t>166:59:49</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/21 21:56:10</t>
+          <t>2026/07/21 23:56:10</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>164:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/21 21:57:22</t>
+          <t>2026/07/21 23:57:20</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>164:59:36</t>
+          <t>166:59:34</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -6755,7 +6755,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>2026/07/21 21:39:00</t>
+          <t>2026/07/21 23:41:19</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>42:59:35</t>
+          <t>45:01:54</t>
         </is>
       </c>
       <c r="L109" t="n">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>2026/07/21 21:52:20</t>
+          <t>2026/07/21 23:52:20</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>31:54:20</t>
+          <t>33:54:20</t>
         </is>
       </c>
       <c r="L111" t="n">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2026/07/21 21:51:23</t>
+          <t>2026/07/21 23:51:23</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>22:57:48</t>
+          <t>24:57:48</t>
         </is>
       </c>
       <c r="L121" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/07/21 21:29:02</t>
+          <t>2026/07/21 23:29:02</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>08:00:57</t>
+          <t>10:00:57</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/07/21 21:11:26</t>
+          <t>2026/07/21 23:11:26</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/07/21 20:55:38</t>
+          <t>2026/07/21 22:55:38</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -7699,7 +7699,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026/07/21 21:09:20</t>
+          <t>2026/07/21 23:09:20</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L125" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/07/21 22:19:28</t>
+          <t>2026/07/21 23:19:28</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>02:03:04</t>
+          <t>03:03:04</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -7783,6 +7783,124 @@
         <v>0</v>
       </c>
       <c r="N126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>16</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>2026/07/21 20:54:58</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>-33.4761583, -70.698465</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>-33.47616, -70.69846</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>2026/07/21 22:54:58</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>-33.4761583, -70.698465</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>-33.47616, -70.69846</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L127" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" t="n">
+        <v>0</v>
+      </c>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>7</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2026/07/21 21:46:46</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>-32.8792099, -70.6088216</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>-32.87921, -70.60882</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>2026/07/21 23:46:46</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>-32.8792099, -70.6088216</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>-32.87921, -70.60882</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L128" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8068,7 +8186,7 @@
         <v>51</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>120</v>
@@ -8157,13 +8275,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>272.36</v>
+        <v>272.35</v>
       </c>
       <c r="C19" t="n">
         <v>24</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-23T06:29Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N113"/>
+  <dimension ref="A1:N114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/22 22:01:28</t>
+          <t>2026/07/22 23:01:23</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:59:36</t>
+          <t>166:59:31</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/07/22 22:13:38</t>
+          <t>2026/07/22 23:13:20</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>166:00:18</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/07/22 22:23:11</t>
+          <t>2026/07/22 23:23:08</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>165:56:09</t>
+          <t>166:56:06</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/07/22 22:31:39</t>
+          <t>2026/07/22 23:31:21</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>166:00:01</t>
+          <t>166:59:43</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/07/22 21:34:38</t>
+          <t>2026/07/22 23:34:57</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>164:59:15</t>
+          <t>166:59:34</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/07/22 21:56:10</t>
+          <t>2026/07/22 23:56:10</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>164:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/22 21:57:38</t>
+          <t>2026/07/22 23:57:21</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>164:58:24</t>
+          <t>166:58:07</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>2026/07/22 21:29:02</t>
+          <t>2026/07/22 23:29:02</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>32:00:57</t>
+          <t>34:00:57</t>
         </is>
       </c>
       <c r="L93" t="n">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>2026/07/22 21:43:00</t>
+          <t>2026/07/22 23:43:03</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>08:40:57</t>
+          <t>10:41:00</t>
         </is>
       </c>
       <c r="L101" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>2026/07/22 21:52:01</t>
+          <t>2026/07/22 23:52:02</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>02:57:49</t>
+          <t>04:57:50</t>
         </is>
       </c>
       <c r="L110" t="n">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>2026/07/22 21:06:29</t>
+          <t>2026/07/22 23:06:29</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L111" t="n">
@@ -6932,7 +6932,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>2026/07/22 21:25:19</t>
+          <t>2026/07/22 23:25:19</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>02:01:10</t>
+          <t>04:01:10</t>
         </is>
       </c>
       <c r="L112" t="n">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026/07/22 21:42:27</t>
+          <t>2026/07/22 23:42:32</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>00:59:33</t>
+          <t>02:59:38</t>
         </is>
       </c>
       <c r="L113" t="n">
@@ -7016,6 +7016,65 @@
         <v>0</v>
       </c>
       <c r="N113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>7</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2026/07/22 21:35:49</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>-33.4358266, -70.62904</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>-33.43583, -70.62904</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>2026/07/22 23:36:00</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>-33.4358266, -70.62904</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>-33.43583, -70.62904</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>02:00:11</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7314,13 +7373,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>209.28</v>
+        <v>209.2</v>
       </c>
       <c r="C15" t="n">
         <v>25</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>133</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-24T06:24Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N123"/>
+  <dimension ref="A1:N127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/23 22:01:38</t>
+          <t>2026/07/23 23:01:38</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:59:02</t>
+          <t>166:59:02</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/07/23 22:23:29</t>
+          <t>2026/07/23 23:22:52</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>165:59:51</t>
+          <t>166:59:14</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/07/23 21:31:21</t>
+          <t>2026/07/23 23:31:21</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>164:59:19</t>
+          <t>166:59:19</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/07/23 21:34:21</t>
+          <t>2026/07/23 23:34:57</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>164:58:53</t>
+          <t>166:59:29</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/23 21:56:10</t>
+          <t>2026/07/23 23:56:10</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:00:01</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/07/23 21:57:20</t>
+          <t>2026/07/23 23:57:29</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>164:59:23</t>
+          <t>166:59:32</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>2026/07/23 21:36:00</t>
+          <t>2026/07/23 23:36:00</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>24:00:11</t>
+          <t>26:00:11</t>
         </is>
       </c>
       <c r="L108" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/07/23 21:26:02</t>
+          <t>2026/07/23 23:26:02</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/07/23 20:55:14</t>
+          <t>2026/07/23 22:55:14</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>02:00:54</t>
+          <t>04:00:54</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/07/23 21:56:08</t>
+          <t>2026/07/23 23:55:50</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>01:00:19</t>
+          <t>03:00:01</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7607,6 +7607,242 @@
       </c>
       <c r="N123" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>3</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2026/07/23 21:30:33</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>-32.838377, -70.95549</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>-32.83838, -70.95549</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2026/07/23 23:28:25</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>-32.838377, -70.95549</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>-32.83838, -70.95549</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>01:57:52</t>
+        </is>
+      </c>
+      <c r="L124" t="n">
+        <v>0</v>
+      </c>
+      <c r="M124" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>5</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2026/07/23 21:51:39</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>-32.841916, -70.936829</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>-32.84192, -70.93683</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>2026/07/23 23:55:15</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>-32.841685, -70.936804</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>-32.84168, -70.93680</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>02:03:36</t>
+        </is>
+      </c>
+      <c r="L125" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M125" t="n">
+        <v>0</v>
+      </c>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>12</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>2026/07/23 21:53:59</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>-32.8792316, -70.6088033</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>-32.87923, -70.60880</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>2026/07/23 23:53:59</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>-32.8792316, -70.6088033</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>-32.87923, -70.60880</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L126" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" t="n">
+        <v>0</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>SLP20250425120-AC01</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>8</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>2026/07/23 22:55:52</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>-33.360006, -70.806995</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>-33.36001, -70.80700</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>2026/07/23 23:55:50</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>-33.360006, -70.806995</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>-33.36001, -70.80700</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>00:59:58</t>
+        </is>
+      </c>
+      <c r="L127" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" t="n">
+        <v>0</v>
+      </c>
+      <c r="N127" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -7676,13 +7912,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>601.37</v>
+        <v>601.3099999999999</v>
       </c>
       <c r="C3" t="n">
         <v>31</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>142</v>
@@ -7948,7 +8184,7 @@
         <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
         <v>9</v>
@@ -7980,13 +8216,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>495.93</v>
+        <v>495.92</v>
       </c>
       <c r="C19" t="n">
         <v>44</v>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
         <v>143</v>
@@ -7999,13 +8235,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>557.5700000000001</v>
+        <v>557.34</v>
       </c>
       <c r="C20" t="n">
         <v>43</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>145</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-24T17:29Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1299,7 +1299,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>LPR20251T02800022</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1317,48 +1317,48 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>-33.4761616, -70.698455</t>
+          <t>-33.367368, -70.696671</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>-33.47616, -70.69845</t>
+          <t>-33.36737, -70.69667</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/17 10:16:04</t>
+          <t>2026/07/23 23:56:10</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>-33.3621016, -70.67012</t>
+          <t>-33.367368, -70.696671</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>-33.36210, -70.67012</t>
+          <t>-33.36737, -70.69667</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>09:19:55</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>18.78</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LPR20251T02800022</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1376,42 +1376,42 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>-33.367368, -70.696671</t>
+          <t>-33.4761616, -70.698455</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-33.36737, -70.69667</t>
+          <t>-33.47616, -70.69845</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/23 23:56:10</t>
+          <t>2026/07/17 10:16:04</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>-33.367368, -70.696671</t>
+          <t>-33.3621016, -70.67012</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>-33.36737, -70.69667</t>
+          <t>-33.36210, -70.67012</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>167:00:01</t>
+          <t>09:19:55</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>18.78</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-24T21:01Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1299,7 +1299,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LPR20251T02800022</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1317,48 +1317,48 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>-33.367368, -70.696671</t>
+          <t>-33.4761616, -70.698455</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>-33.36737, -70.69667</t>
+          <t>-33.47616, -70.69845</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/23 23:56:10</t>
+          <t>2026/07/17 10:16:04</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>-33.367368, -70.696671</t>
+          <t>-33.3621016, -70.67012</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>-33.36737, -70.69667</t>
+          <t>-33.36210, -70.67012</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>167:00:01</t>
+          <t>09:19:55</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>18.78</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>LPR20251T02800022</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1376,42 +1376,42 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>-33.4761616, -70.698455</t>
+          <t>-33.367368, -70.696671</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-33.47616, -70.69845</t>
+          <t>-33.36737, -70.69667</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/17 10:16:04</t>
+          <t>2026/07/23 23:56:10</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>-33.3621016, -70.67012</t>
+          <t>-33.367368, -70.696671</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>-33.36210, -70.67012</t>
+          <t>-33.36737, -70.69667</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>09:19:55</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>18.78</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-25T06:16Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N123"/>
+  <dimension ref="A1:N124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/24 22:01:15</t>
+          <t>2026/07/24 23:01:38</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:59:22</t>
+          <t>166:59:45</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/07/24 22:23:07</t>
+          <t>2026/07/24 23:24:16</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>165:59:45</t>
+          <t>167:00:54</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/07/24 21:31:21</t>
+          <t>2026/07/24 23:31:25</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>164:59:43</t>
+          <t>166:59:47</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/07/24 21:35:20</t>
+          <t>2026/07/24 23:34:53</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>165:00:23</t>
+          <t>166:59:56</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/07/24 21:56:09</t>
+          <t>2026/07/24 23:56:09</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -6637,7 +6637,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>2026/07/24 21:36:00</t>
+          <t>2026/07/24 23:36:00</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>48:00:11</t>
+          <t>50:00:11</t>
         </is>
       </c>
       <c r="L107" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/07/24 22:07:14</t>
+          <t>2026/07/24 23:07:17</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>25:11:25</t>
+          <t>26:11:28</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/07/24 21:56:07</t>
+          <t>2026/07/24 23:55:51</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>23:00:15</t>
+          <t>24:59:59</t>
         </is>
       </c>
       <c r="L119" t="n">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/07/24 21:39:50</t>
+          <t>2026/07/24 23:39:50</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>08:01:12</t>
+          <t>10:01:12</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2026/07/24 22:08:55</t>
+          <t>2026/07/24 23:08:55</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>04:08:00</t>
+          <t>05:08:00</t>
         </is>
       </c>
       <c r="L121" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/07/24 20:50:34</t>
+          <t>2026/07/24 22:50:34</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>02:44:43</t>
+          <t>04:44:43</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/07/24 21:05:47</t>
+          <t>2026/07/24 23:05:47</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -7606,6 +7606,65 @@
         <v>0</v>
       </c>
       <c r="N123" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>7</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2026/07/24 21:19:06</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.955488</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95549</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2026/07/24 23:17:08</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.955488</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95549</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>01:58:02</t>
+        </is>
+      </c>
+      <c r="L124" t="n">
+        <v>0</v>
+      </c>
+      <c r="M124" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7676,13 +7735,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>565.8099999999999</v>
+        <v>565.75</v>
       </c>
       <c r="C3" t="n">
         <v>34</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>142</v>
@@ -7885,10 +7944,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>800.5</v>
+        <v>801.45</v>
       </c>
       <c r="C14" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -7980,13 +8039,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>560.22</v>
+        <v>560.21</v>
       </c>
       <c r="C19" t="n">
         <v>51</v>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
         <v>143</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-26T06:35Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/07/25 22:01:51</t>
+          <t>2026/07/25 23:01:21</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>166:00:26</t>
+          <t>166:59:56</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/07/25 22:22:51</t>
+          <t>2026/07/25 23:22:38</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>165:58:44</t>
+          <t>166:58:31</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/07/25 22:31:25</t>
+          <t>2026/07/25 23:31:38</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>166:00:04</t>
+          <t>167:00:17</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/07/25 22:34:56</t>
+          <t>2026/07/25 23:36:32</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:59:09</t>
+          <t>167:00:45</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/25 21:56:09</t>
+          <t>2026/07/25 23:56:09</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>164:59:58</t>
+          <t>166:59:58</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>2026/07/25 21:36:00</t>
+          <t>2026/07/25 23:36:00</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>72:00:11</t>
+          <t>74:00:11</t>
         </is>
       </c>
       <c r="L101" t="n">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026/07/25 21:46:50</t>
+          <t>2026/07/25 23:46:33</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>48:51:01</t>
+          <t>50:50:44</t>
         </is>
       </c>
       <c r="L115" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/07/25 21:55:53</t>
+          <t>2026/07/25 23:55:51</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>47:00:01</t>
+          <t>48:59:59</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026/07/25 21:56:56</t>
+          <t>2026/07/25 23:56:56</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>08:00:47</t>
+          <t>10:00:47</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/07/25 20:38:20</t>
+          <t>2026/07/25 22:38:20</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="L119" t="n">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/07/25 21:01:31</t>
+          <t>2026/07/25 23:01:31</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2026/07/25 21:25:02</t>
+          <t>2026/07/25 23:25:02</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>02:00:38</t>
+          <t>04:00:38</t>
         </is>
       </c>
       <c r="L121" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/07/25 21:30:47</t>
+          <t>2026/07/25 23:30:47</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/07/25 21:46:44</t>
+          <t>2026/07/25 23:46:41</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>02:12:57</t>
+          <t>04:12:54</t>
         </is>
       </c>
       <c r="L123" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-27T07:29Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N126"/>
+  <dimension ref="A1:N127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/07/26 22:01:45</t>
+          <t>2026/07/26 23:01:52</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>166:00:06</t>
+          <t>167:00:13</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/07/26 22:34:51</t>
+          <t>2026/07/26 23:34:43</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:58:07</t>
+          <t>166:57:59</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/26 21:56:11</t>
+          <t>2026/07/26 23:56:11</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/07/26 22:13:21</t>
+          <t>2026/07/26 23:13:38</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>71:17:29</t>
+          <t>72:17:46</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/07/26 21:25:02</t>
+          <t>2026/07/26 23:25:02</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>26:00:38</t>
+          <t>28:00:38</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/07/26 21:30:47</t>
+          <t>2026/07/26 23:30:47</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>26:00:00</t>
+          <t>28:00:00</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -7699,7 +7699,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026/07/26 22:06:31</t>
+          <t>2026/07/26 23:06:31</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>01:57:35</t>
+          <t>02:57:35</t>
         </is>
       </c>
       <c r="L125" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/07/26 21:54:20</t>
+          <t>2026/07/26 23:54:17</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>00:07:47</t>
+          <t>02:07:44</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -7783,6 +7783,65 @@
         <v>0</v>
       </c>
       <c r="N126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>2</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>2026/07/26 21:46:56</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>-33.4361866, -70.6295933</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>-33.43619, -70.62959</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>2026/07/26 23:46:56</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>-33.4361866, -70.6295933</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>-33.43619, -70.62959</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L127" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" t="n">
+        <v>0</v>
+      </c>
+      <c r="N127" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8087,7 +8146,7 @@
         <v>16</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>133</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-29T06:28Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N131"/>
+  <dimension ref="A1:N134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/07/28 21:56:09</t>
+          <t>2026/07/28 23:56:09</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>164:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>2026/07/28 22:22:39</t>
+          <t>2026/07/28 23:22:25</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>68:00:13</t>
+          <t>68:59:59</t>
         </is>
       </c>
       <c r="L108" t="n">
@@ -6932,7 +6932,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>2026/07/28 21:31:55</t>
+          <t>2026/07/28 23:32:08</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>32:50:38</t>
+          <t>34:50:51</t>
         </is>
       </c>
       <c r="L112" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/07/28 21:01:18</t>
+          <t>2026/07/28 23:01:18</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>24:00:10</t>
+          <t>26:00:10</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/07/28 21:34:58</t>
+          <t>2026/07/28 23:36:06</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>18:59:33</t>
+          <t>21:00:41</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/07/28 21:46:31</t>
+          <t>2026/07/28 23:46:31</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>05:27:45</t>
+          <t>07:27:45</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/07/28 21:32:13</t>
+          <t>2026/07/28 23:32:13</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -8078,6 +8078,183 @@
         <v>0</v>
       </c>
       <c r="N131" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>8</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>2026/07/28 21:08:55</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>-32.7430399, -70.729805</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>-32.74304, -70.72980</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>2026/07/28 23:08:55</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>-32.7430399, -70.729805</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>-32.74304, -70.72980</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L132" t="n">
+        <v>0</v>
+      </c>
+      <c r="M132" t="n">
+        <v>0</v>
+      </c>
+      <c r="N132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>8</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2026/07/28 22:00:48</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>-33.484909, -70.772417</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>-33.48491, -70.77242</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>2026/07/28 23:03:47</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>-33.484909, -70.772417</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>-33.48491, -70.77242</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>01:02:59</t>
+        </is>
+      </c>
+      <c r="L133" t="n">
+        <v>0</v>
+      </c>
+      <c r="M133" t="n">
+        <v>0</v>
+      </c>
+      <c r="N133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>8</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2026/07/28 23:00:34</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>-32.838363, -70.955481</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95548</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>2026/07/28 23:59:47</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>-32.838363, -70.955481</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95548</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>00:59:13</t>
+        </is>
+      </c>
+      <c r="L134" t="n">
+        <v>0</v>
+      </c>
+      <c r="M134" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8148,13 +8325,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1260.69</v>
+        <v>1260.67</v>
       </c>
       <c r="C3" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>144</v>
@@ -8186,13 +8363,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>646.3099999999999</v>
+        <v>646.3</v>
       </c>
       <c r="C5" t="n">
         <v>31</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>132</v>
@@ -8471,13 +8648,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>475.19</v>
+        <v>475.15</v>
       </c>
       <c r="C20" t="n">
         <v>39</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>145</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-30T06:26Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N128"/>
+  <dimension ref="A1:N131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/07/29 21:56:09</t>
+          <t>2026/07/29 23:56:09</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>164:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026/07/29 21:35:31</t>
+          <t>2026/07/29 23:34:29</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>43:00:06</t>
+          <t>44:59:04</t>
         </is>
       </c>
       <c r="L113" t="n">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/07/29 21:45:25</t>
+          <t>2026/07/29 23:45:25</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>11:05:11</t>
+          <t>13:05:11</t>
         </is>
       </c>
       <c r="L119" t="n">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/07/29 21:13:50</t>
+          <t>2026/07/29 23:13:50</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>04:00:17</t>
+          <t>06:00:17</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/07/29 21:42:37</t>
+          <t>2026/07/29 23:42:37</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -7671,11 +7671,11 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -7684,37 +7684,37 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2026/07/29 20:40:14</t>
+          <t>2026/07/29 20:11:30</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>-32.841871, -70.936857</t>
+          <t>-33.4760783, -70.6985216</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>-32.84187, -70.93686</t>
+          <t>-33.47608, -70.69852</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026/07/29 21:43:35</t>
+          <t>2026/07/29 22:11:39</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>-32.841871, -70.936857</t>
+          <t>-33.4760783, -70.6985216</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>-32.84187, -70.93686</t>
+          <t>-33.47608, -70.69852</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>01:03:21</t>
+          <t>02:00:09</t>
         </is>
       </c>
       <c r="L125" t="n">
@@ -7730,70 +7730,70 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCL-70</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2026/07/29 20:54:32</t>
+          <t>2026/07/29 20:17:09</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>-32.840483, -70.959366</t>
+          <t>-32.7976133, -70.88712</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>-32.84048, -70.95937</t>
+          <t>-32.79761, -70.88712</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/07/29 21:15:37</t>
+          <t>2026/07/29 22:17:09</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>-32.838378, -70.955828</t>
+          <t>-32.7976133, -70.88712</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>-32.83838, -70.95583</t>
+          <t>-32.79761, -70.88712</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>00:21:05</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="L126" t="n">
-        <v>1.29</v>
+        <v>0</v>
       </c>
       <c r="M126" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="N126" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -7802,37 +7802,37 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2026/07/29 21:13:22</t>
+          <t>2026/07/29 20:40:14</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>-33.4362033, -70.59588</t>
+          <t>-32.841871, -70.936857</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>-33.43620, -70.59588</t>
+          <t>-32.84187, -70.93686</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>2026/07/29 22:11:10</t>
+          <t>2026/07/29 23:43:38</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>-33.4362033, -70.59588</t>
+          <t>-32.841871, -70.936857</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>-33.43620, -70.59588</t>
+          <t>-32.84187, -70.93686</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>00:57:48</t>
+          <t>03:03:24</t>
         </is>
       </c>
       <c r="L127" t="n">
@@ -7852,55 +7852,232 @@
         </is>
       </c>
       <c r="C128" t="n">
+        <v>11</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>2026/07/29 20:54:32</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>-32.840483, -70.959366</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>-32.84048, -70.95937</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>2026/07/29 21:15:37</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>-32.838378, -70.955828</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>-32.83838, -70.95583</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>00:21:05</t>
+        </is>
+      </c>
+      <c r="L128" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="M128" t="n">
+        <v>33</v>
+      </c>
+      <c r="N128" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>3</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>2026/07/29 21:13:22</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>-33.4362033, -70.59588</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>-33.43620, -70.59588</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>2026/07/29 22:23:15</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>-33.436205, -70.6294716</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>-33.43621, -70.62947</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>01:09:53</t>
+        </is>
+      </c>
+      <c r="L129" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="M129" t="n">
+        <v>48</v>
+      </c>
+      <c r="N129" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
         <v>12</v>
       </c>
-      <c r="D128" t="inlineStr">
+      <c r="D130" t="inlineStr">
         <is>
           <t>Paradas</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr">
+      <c r="E130" t="inlineStr">
         <is>
           <t>2026/07/29 21:15:58</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr">
+      <c r="F130" t="inlineStr">
         <is>
           <t>-32.838366, -70.955903</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr">
+      <c r="G130" t="inlineStr">
         <is>
           <t>-32.83837, -70.95590</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>2026/07/29 21:24:19</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>2026/07/29 23:20:48</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
         <is>
           <t>-32.838366, -70.955903</t>
         </is>
       </c>
-      <c r="J128" t="inlineStr">
+      <c r="J130" t="inlineStr">
         <is>
           <t>-32.83837, -70.95590</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr">
-        <is>
-          <t>00:08:21</t>
-        </is>
-      </c>
-      <c r="L128" t="n">
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>02:04:50</t>
+        </is>
+      </c>
+      <c r="L130" t="n">
         <v>0</v>
       </c>
-      <c r="M128" t="n">
+      <c r="M130" t="n">
         <v>0</v>
       </c>
-      <c r="N128" t="n">
+      <c r="N130" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>4</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>2026/07/29 21:33:36</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>-32.743055, -70.729795</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>-32.74305, -70.72979</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>2026/07/29 23:33:36</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>-32.743055, -70.729795</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>-32.74305, -70.72979</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L131" t="n">
+        <v>0</v>
+      </c>
+      <c r="M131" t="n">
+        <v>0</v>
+      </c>
+      <c r="N131" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7952,13 +8129,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1229.4</v>
+        <v>1229.37</v>
       </c>
       <c r="C2" t="n">
         <v>51</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>151</v>
@@ -8009,13 +8186,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>604.04</v>
+        <v>604.03</v>
       </c>
       <c r="C5" t="n">
         <v>28</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>132</v>
@@ -8180,13 +8357,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1048.52</v>
+        <v>1048.5</v>
       </c>
       <c r="C14" t="n">
         <v>41</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>132</v>
@@ -8199,13 +8376,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>41.98</v>
+        <v>46.26</v>
       </c>
       <c r="C15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
         <v>82</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-07-31T06:42Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N132"/>
+  <dimension ref="A1:N134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/30 21:56:09</t>
+          <t>2026/07/30 23:56:09</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>164:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>2026/07/30 22:12:38</t>
+          <t>2026/07/30 23:13:05</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>82:39:57</t>
+          <t>83:40:24</t>
         </is>
       </c>
       <c r="L79" t="n">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/07/30 22:35:33</t>
+          <t>2026/07/30 23:35:04</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>20:00:44</t>
+          <t>21:00:15</t>
         </is>
       </c>
       <c r="L119" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/07/30 21:52:35</t>
+          <t>2026/07/30 23:52:35</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>10:01:27</t>
+          <t>12:01:27</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -7699,7 +7699,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026/07/30 20:42:34</t>
+          <t>2026/07/30 22:42:34</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L125" t="n">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026/07/30 21:43:47</t>
+          <t>2026/07/30 23:43:47</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>02:00:35</t>
+          <t>04:00:35</t>
         </is>
       </c>
       <c r="L128" t="n">
@@ -7935,7 +7935,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>2026/07/30 22:07:50</t>
+          <t>2026/07/30 23:07:52</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>01:57:40</t>
+          <t>02:57:42</t>
         </is>
       </c>
       <c r="L129" t="n">
@@ -8084,11 +8084,11 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
@@ -8097,37 +8097,37 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2026/07/30 20:55:54</t>
+          <t>2026/07/30 20:53:44</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>-33.482162, -70.764895</t>
+          <t>-33.0872166, -71.3622383</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>-33.48216, -70.76489</t>
+          <t>-33.08722, -71.36224</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/07/30 21:58:55</t>
+          <t>2026/07/30 22:53:44</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>-33.482162, -70.764895</t>
+          <t>-33.0872166, -71.3622383</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>-33.48216, -70.76489</t>
+          <t>-33.08722, -71.36224</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>01:03:01</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8137,6 +8137,124 @@
         <v>0</v>
       </c>
       <c r="N132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>10</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2026/07/30 20:55:54</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>-33.482162, -70.764895</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>-33.48216, -70.76489</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>2026/07/30 23:58:58</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>-33.482162, -70.764895</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>-33.48216, -70.76489</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>03:03:04</t>
+        </is>
+      </c>
+      <c r="L133" t="n">
+        <v>0</v>
+      </c>
+      <c r="M133" t="n">
+        <v>0</v>
+      </c>
+      <c r="N133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>3</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2026/07/30 21:04:35</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>-33.43736, -70.6287583</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>-33.43736, -70.62876</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>2026/07/30 23:04:35</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>-33.43736, -70.6287583</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>-33.43736, -70.62876</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L134" t="n">
+        <v>0</v>
+      </c>
+      <c r="M134" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8232,7 +8350,7 @@
         <v>32</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>132</v>
@@ -8435,13 +8553,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>78.18000000000001</v>
+        <v>78.17</v>
       </c>
       <c r="C15" t="n">
         <v>11</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>125</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-01T06:27Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1358,7 +1358,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LPR20251T02800022</t>
+          <t>SLP20250425120-AC01</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1376,48 +1376,48 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>-33.367368, -70.696671</t>
+          <t>-33.360006, -70.806995</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-33.36737, -70.69667</t>
+          <t>-33.36001, -70.80700</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/31 12:00:34</t>
+          <t>2026/07/27 11:20:55</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>-33.367272, -70.696588</t>
+          <t>-33.360166, -70.807078</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>-33.36727, -70.69659</t>
+          <t>-33.36017, -70.80708</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>155:04:25</t>
+          <t>58:24:46</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>0.51</v>
+        <v>0.03</v>
       </c>
       <c r="M18" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SLP20250425120-AC01</t>
+          <t>LPR20251T02800022</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1435,42 +1435,42 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>-33.360006, -70.806995</t>
+          <t>-33.367368, -70.696671</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-33.36001, -70.80700</t>
+          <t>-33.36737, -70.69667</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/07/27 11:20:55</t>
+          <t>2026/07/31 12:00:34</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-33.360166, -70.807078</t>
+          <t>-33.367272, -70.696588</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>-33.36017, -70.80708</t>
+          <t>-33.36727, -70.69659</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>58:24:46</t>
+          <t>155:04:25</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>0.03</v>
+        <v>0.51</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>2026/07/31 22:02:32</t>
+          <t>2026/07/31 23:02:32</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>106:29:51</t>
+          <t>107:29:51</t>
         </is>
       </c>
       <c r="L68" t="n">
@@ -6755,7 +6755,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>2026/07/31 22:13:37</t>
+          <t>2026/07/31 23:13:22</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -6770,7 +6770,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>66:59:40</t>
+          <t>67:59:25</t>
         </is>
       </c>
       <c r="L109" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/07/31 21:57:37</t>
+          <t>2026/07/31 23:57:34</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>34:06:29</t>
+          <t>36:06:26</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7730,11 +7730,11 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>MITSUBISHI L200 PHZF-89</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -7743,37 +7743,37 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2026/07/30 20:53:44</t>
+          <t>2026/07/30 21:04:35</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>-33.0872166, -71.3622383</t>
+          <t>-33.43736, -70.6287583</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>-33.08722, -71.36224</t>
+          <t>-33.43736, -70.62876</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/07/31 20:53:44</t>
+          <t>2026/07/31 23:04:35</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>-33.0872166, -71.3622383</t>
+          <t>-33.43736, -70.6287583</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>-33.08722, -71.36224</t>
+          <t>-33.43736, -70.62876</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>24:00:00</t>
+          <t>26:00:00</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -7789,60 +7789,60 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>LPR20251E02900022</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2026/07/30 21:04:35</t>
+          <t>2026/07/31 10:41:11</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>-33.43736, -70.6287583</t>
+          <t>-33.367294, -70.696684</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>-33.43736, -70.62876</t>
+          <t>-33.36729, -70.69668</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>2026/07/31 21:04:35</t>
+          <t>2026/07/31 11:47:29</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>-33.43736, -70.6287583</t>
+          <t>-33.367245, -70.696606</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>-33.43736, -70.62876</t>
+          <t>-33.36724, -70.69661</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>24:00:00</t>
+          <t>01:06:18</t>
         </is>
       </c>
       <c r="L127" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="M127" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="N127" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="128">
@@ -7852,66 +7852,66 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>2026/07/31 10:41:11</t>
+          <t>2026/07/31 11:48:27</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>-33.367294, -70.696684</t>
+          <t>-33.367145, -70.696511</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>-33.36729, -70.69668</t>
+          <t>-33.36715, -70.69651</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026/07/31 11:47:29</t>
+          <t>2026/07/31 23:48:30</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>-33.367245, -70.696606</t>
+          <t>-33.36741, -70.696458</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>-33.36724, -70.69661</t>
+          <t>-33.36741, -70.69646</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>01:06:18</t>
+          <t>12:00:03</t>
         </is>
       </c>
       <c r="L128" t="n">
-        <v>0.45</v>
+        <v>0.03</v>
       </c>
       <c r="M128" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="N128" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>LPR20251E02900022</t>
+          <t>LPR20251T02800022</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -7920,41 +7920,41 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2026/07/31 11:48:27</t>
+          <t>2026/07/31 12:23:42</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>-33.367145, -70.696511</t>
+          <t>-33.367244, -70.69677</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>-33.36715, -70.69651</t>
+          <t>-33.36724, -70.69677</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>2026/07/31 21:48:30</t>
+          <t>2026/07/31 23:23:44</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>-33.36741, -70.696458</t>
+          <t>-33.367244, -70.69677</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>-33.36741, -70.69646</t>
+          <t>-33.36724, -70.69677</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>10:00:03</t>
+          <t>11:00:02</t>
         </is>
       </c>
       <c r="L129" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="M129" t="n">
         <v>0</v>
@@ -7966,11 +7966,11 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>LPR20251T02800022</t>
+          <t>SUZUKI CARRY SKDB-52</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -7979,37 +7979,37 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2026/07/31 12:23:42</t>
+          <t>2026/07/31 14:47:36</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>-33.367244, -70.69677</t>
+          <t>-32.8792, -70.6087766</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>-33.36724, -70.69677</t>
+          <t>-32.87920, -70.60878</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/07/31 22:23:44</t>
+          <t>2026/07/31 22:47:36</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>-33.367244, -70.69677</t>
+          <t>-32.8792, -70.6087766</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>-33.36724, -70.69677</t>
+          <t>-32.87920, -70.60878</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>10:00:02</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8025,11 +8025,11 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -8038,37 +8038,37 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2026/07/31 14:47:36</t>
+          <t>2026/07/31 14:54:01</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>-32.8792, -70.6087766</t>
+          <t>-33.367145, -70.6958916</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>-32.87920, -70.60878</t>
+          <t>-33.36715, -70.69589</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/07/31 20:47:36</t>
+          <t>2026/07/31 22:54:16</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>-32.8792, -70.6087766</t>
+          <t>-33.367145, -70.6958916</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>-32.87920, -70.60878</t>
+          <t>-33.36715, -70.69589</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>08:00:15</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8084,11 +8084,11 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
@@ -8097,37 +8097,37 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2026/07/31 14:54:01</t>
+          <t>2026/07/31 17:46:43</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>-33.367145, -70.6958916</t>
+          <t>-32.7976183, -70.8870683</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>-33.36715, -70.69589</t>
+          <t>-32.79762, -70.88707</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/07/31 20:54:16</t>
+          <t>2026/07/31 23:46:43</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>-33.367145, -70.6958916</t>
+          <t>-32.7976183, -70.8870683</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>-33.36715, -70.69589</t>
+          <t>-32.79762, -70.88707</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>06:00:15</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8143,11 +8143,11 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>CHANGAN HUNTER TKCL-70</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
@@ -8156,37 +8156,37 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>2026/07/31 17:46:43</t>
+          <t>2026/07/31 19:05:29</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>-32.7976183, -70.8870683</t>
+          <t>-32.83835, -70.955544</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>-32.79762, -70.88707</t>
+          <t>-32.83835, -70.95554</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/07/31 21:46:43</t>
+          <t>2026/07/31 23:03:01</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>-32.7976183, -70.8870683</t>
+          <t>-32.83835, -70.955544</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>-32.79762, -70.88707</t>
+          <t>-32.83835, -70.95554</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>03:57:32</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -8202,11 +8202,11 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCL-70</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -8215,41 +8215,41 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2026/07/31 19:05:29</t>
+          <t>2026/07/31 20:07:02</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>-32.83835, -70.955544</t>
+          <t>-32.7431883, -70.7296583</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>-32.83835, -70.95554</t>
+          <t>-32.74319, -70.72966</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/07/31 22:03:00</t>
+          <t>2026/07/31 22:41:49</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>-32.83835, -70.955544</t>
+          <t>-32.7430399, -70.729765</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>-32.83835, -70.95554</t>
+          <t>-32.74304, -70.72977</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>02:57:31</t>
+          <t>02:34:47</t>
         </is>
       </c>
       <c r="L134" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="M134" t="n">
         <v>0</v>
@@ -8261,11 +8261,11 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>JAC X200 SJTJ-50</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -8274,41 +8274,41 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>2026/07/31 20:07:02</t>
+          <t>2026/07/31 21:18:54</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>-32.7431883, -70.7296583</t>
+          <t>-33.4761816, -70.6984316</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>-32.74319, -70.72966</t>
+          <t>-33.47618, -70.69843</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026/07/31 20:41:49</t>
+          <t>2026/07/31 23:20:02</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>-32.7430399, -70.729765</t>
+          <t>-33.4761816, -70.6984316</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>-32.74304, -70.72977</t>
+          <t>-33.47618, -70.69843</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>00:34:47</t>
+          <t>02:01:08</t>
         </is>
       </c>
       <c r="L135" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="M135" t="n">
         <v>0</v>
@@ -8403,13 +8403,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>702.64</v>
+        <v>702.65</v>
       </c>
       <c r="C4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>132</v>
@@ -8593,13 +8593,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1138.61</v>
+        <v>1138.6</v>
       </c>
       <c r="C14" t="n">
         <v>44</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>132</v>
@@ -8707,10 +8707,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>732.3200000000001</v>
+        <v>756.0700000000001</v>
       </c>
       <c r="C20" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-01T09:56Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1358,7 +1358,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SLP20250425120-AC01</t>
+          <t>LPR20251T02800022</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1376,48 +1376,48 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>-33.360006, -70.806995</t>
+          <t>-33.367368, -70.696671</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-33.36001, -70.80700</t>
+          <t>-33.36737, -70.69667</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/07/27 11:20:55</t>
+          <t>2026/07/31 12:00:34</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>-33.360166, -70.807078</t>
+          <t>-33.367272, -70.696588</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>-33.36017, -70.80708</t>
+          <t>-33.36727, -70.69659</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>58:24:46</t>
+          <t>155:04:25</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>0.03</v>
+        <v>0.51</v>
       </c>
       <c r="M18" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LPR20251T02800022</t>
+          <t>SLP20250425120-AC01</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1435,42 +1435,42 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>-33.367368, -70.696671</t>
+          <t>-33.360006, -70.806995</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-33.36737, -70.69667</t>
+          <t>-33.36001, -70.80700</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/07/31 12:00:34</t>
+          <t>2026/07/27 11:20:55</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-33.367272, -70.696588</t>
+          <t>-33.360166, -70.807078</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>-33.36727, -70.69659</t>
+          <t>-33.36017, -70.80708</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>155:04:25</t>
+          <t>58:24:46</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>0.51</v>
+        <v>0.03</v>
       </c>
       <c r="M19" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-02T06:32Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -3392,7 +3392,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>2026/08/01 21:46:37</t>
+          <t>2026/08/01 23:46:21</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>130:13:56</t>
+          <t>132:13:40</t>
         </is>
       </c>
       <c r="L52" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/08/01 21:57:37</t>
+          <t>2026/08/01 23:57:26</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>58:06:29</t>
+          <t>60:06:18</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -7935,7 +7935,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>2026/08/01 21:41:33</t>
+          <t>2026/08/01 23:41:33</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>33:53:06</t>
+          <t>35:53:06</t>
         </is>
       </c>
       <c r="L129" t="n">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/08/01 21:55:28</t>
+          <t>2026/08/01 23:55:28</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>33:31:46</t>
+          <t>35:31:46</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/08/01 20:54:16</t>
+          <t>2026/08/01 22:54:16</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>30:00:15</t>
+          <t>32:00:15</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/08/01 21:12:03</t>
+          <t>2026/08/01 23:12:22</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>21:05:26</t>
+          <t>23:05:45</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/08/01 21:44:45</t>
+          <t>2026/08/01 23:44:45</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>05:15:30</t>
+          <t>07:15:30</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/08/01 21:36:42</t>
+          <t>2026/08/01 23:36:42</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L134" t="n">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026/08/01 21:47:39</t>
+          <t>2026/08/01 23:47:39</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>04:00:43</t>
+          <t>06:00:43</t>
         </is>
       </c>
       <c r="L135" t="n">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/08/01 21:53:43</t>
+          <t>2026/08/01 23:53:43</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>04:00:02</t>
+          <t>06:00:02</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/08/01 20:49:02</t>
+          <t>2026/08/01 22:49:02</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/08/01 22:09:19</t>
+          <t>2026/08/01 23:09:20</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>02:57:29</t>
+          <t>03:57:30</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>2026/08/01 21:23:28</t>
+          <t>2026/08/01 23:23:28</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L139" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-03T06:57Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/08/02 21:57:21</t>
+          <t>2026/08/02 23:57:38</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>82:06:13</t>
+          <t>84:06:30</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/08/02 21:41:33</t>
+          <t>2026/08/02 23:41:33</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>57:53:06</t>
+          <t>59:53:06</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/08/02 21:55:28</t>
+          <t>2026/08/02 23:55:28</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>57:31:46</t>
+          <t>59:31:46</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/08/02 20:54:16</t>
+          <t>2026/08/02 22:54:16</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>54:00:15</t>
+          <t>56:00:15</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -8584,26 +8584,26 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/08/02 22:26:09</t>
+          <t>2026/08/02 23:12:29</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>-33.359907, -70.807324</t>
+          <t>-33.359953, -70.807159</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>-33.35991, -70.80732</t>
+          <t>-33.35995, -70.80716</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>13:00:06</t>
+          <t>13:46:26</t>
         </is>
       </c>
       <c r="L140" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="M140" t="n">
         <v>0</v>
@@ -8733,11 +8733,11 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>LPR20251P02790030-ALD</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D143" t="inlineStr">
         <is>
@@ -8746,37 +8746,37 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>2026/08/02 13:13:18</t>
+          <t>2026/08/02 13:35:58</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>-33.08734, -71.3623133</t>
+          <t>-34.579659, -70.961355</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>-33.08734, -71.36231</t>
+          <t>-34.57966, -70.96135</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/08/02 21:13:18</t>
+          <t>2026/08/02 23:36:26</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>-33.08734, -71.3623133</t>
+          <t>-34.579659, -70.961355</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>-33.08734, -71.36231</t>
+          <t>-34.57966, -70.96135</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>08:00:00</t>
+          <t>10:00:28</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -8792,11 +8792,11 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>LPR20251P02790030-ALD</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D144" t="inlineStr">
         <is>
@@ -8805,37 +8805,37 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2026/08/02 13:35:58</t>
+          <t>2026/08/02 18:41:43</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>-34.579659, -70.961355</t>
+          <t>-32.7976166, -70.8871216</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>-34.57966, -70.96135</t>
+          <t>-32.79762, -70.88712</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>2026/08/02 22:36:45</t>
+          <t>2026/08/02 22:41:43</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>-34.579659, -70.961355</t>
+          <t>-32.7976166, -70.8871216</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>-34.57966, -70.96135</t>
+          <t>-32.79762, -70.88712</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>09:00:47</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L144" t="n">
@@ -8851,11 +8851,11 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>SUZUKI CARRY SKDB-52</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D145" t="inlineStr">
         <is>
@@ -8864,32 +8864,32 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2026/08/02 18:41:43</t>
+          <t>2026/08/02 20:23:54</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>-32.7976166, -70.8871216</t>
+          <t>-32.87919, -70.608815</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>-32.79762, -70.88712</t>
+          <t>-32.87919, -70.60882</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/08/02 20:41:43</t>
+          <t>2026/08/02 22:23:54</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>-32.7976166, -70.8871216</t>
+          <t>-32.87919, -70.608815</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>-32.79762, -70.88712</t>
+          <t>-32.87919, -70.60882</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -8910,7 +8910,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>MITSUBISHI L200 PHZF-89</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -8918,111 +8918,111 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>2026/08/02 20:23:54</t>
+          <t>2026/08/02 20:42:57</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>-32.87919, -70.608815</t>
+          <t>-33.4362883, -70.6294366</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>-32.87919, -70.60882</t>
+          <t>-33.43629, -70.62944</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/08/02 22:23:54</t>
+          <t>2026/08/02 22:07:50</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>-32.87919, -70.608815</t>
+          <t>-33.4362749, -70.62938</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>-32.87919, -70.60882</t>
+          <t>-33.43627, -70.62938</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>01:24:53</t>
         </is>
       </c>
       <c r="L146" t="n">
-        <v>0</v>
+        <v>18.82</v>
       </c>
       <c r="M146" t="n">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="N146" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>CHANGAN HUNTER TKCL-70</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2026/08/02 20:42:57</t>
+          <t>2026/08/02 20:51:36</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>-33.4362883, -70.6294366</t>
+          <t>-32.838378, -70.955503</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>-33.43629, -70.62944</t>
+          <t>-32.83838, -70.95550</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/08/02 22:07:50</t>
+          <t>2026/08/02 23:49:51</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>-33.4362749, -70.62938</t>
+          <t>-32.838378, -70.955503</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>-33.43627, -70.62938</t>
+          <t>-32.83838, -70.95550</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>01:24:53</t>
+          <t>02:58:15</t>
         </is>
       </c>
       <c r="L147" t="n">
-        <v>18.82</v>
+        <v>0</v>
       </c>
       <c r="M147" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="N147" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148">
@@ -9056,7 +9056,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2026/08/02 22:27:32</t>
+          <t>2026/08/02 23:27:32</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>01:03:27</t>
+          <t>02:03:27</t>
         </is>
       </c>
       <c r="L148" t="n">
@@ -9151,13 +9151,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1388.99</v>
+        <v>1388.93</v>
       </c>
       <c r="C3" t="n">
         <v>44</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>143</v>
@@ -9170,13 +9170,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1001.72</v>
+        <v>1001.74</v>
       </c>
       <c r="C4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>145</v>
@@ -9189,10 +9189,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1248.98</v>
+        <v>1249.61</v>
       </c>
       <c r="C5" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -9360,10 +9360,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1265.72</v>
+        <v>1268.91</v>
       </c>
       <c r="C14" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-04T06:26Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N144"/>
+  <dimension ref="A1:N147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>2026/08/03 21:57:21</t>
+          <t>2026/08/03 23:57:37</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>106:06:13</t>
+          <t>108:06:29</t>
         </is>
       </c>
       <c r="L110" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/08/03 21:41:59</t>
+          <t>2026/08/03 23:41:59</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>81:53:32</t>
+          <t>83:53:32</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -7699,7 +7699,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026/08/03 21:56:11</t>
+          <t>2026/08/03 23:56:11</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>81:32:29</t>
+          <t>83:32:29</t>
         </is>
       </c>
       <c r="L125" t="n">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/08/03 21:30:46</t>
+          <t>2026/08/03 23:30:38</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>36:04:43</t>
+          <t>38:04:35</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/08/03 21:59:34</t>
+          <t>2026/08/03 23:59:37</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>09:01:34</t>
+          <t>11:01:37</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/08/03 21:27:12</t>
+          <t>2026/08/03 23:27:12</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -8584,32 +8584,32 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/08/03 21:06:33</t>
+          <t>2026/08/03 22:57:58</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>-33.0873183, -71.3623116</t>
+          <t>-33.087165, -71.3621583</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>-33.08732, -71.36231</t>
+          <t>-33.08716, -71.36216</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>05:51:25</t>
         </is>
       </c>
       <c r="L140" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="M140" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N140" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="141">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/08/03 22:22:14</t>
+          <t>2026/08/03 23:22:14</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>03:04:06</t>
+          <t>04:04:06</t>
         </is>
       </c>
       <c r="L142" t="n">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>2026/08/03 21:43:19</t>
+          <t>2026/08/03 23:43:19</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>02:05:47</t>
+          <t>04:05:47</t>
         </is>
       </c>
       <c r="L144" t="n">
@@ -8845,6 +8845,183 @@
         <v>0</v>
       </c>
       <c r="N144" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>9</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>2026/08/03 20:49:06</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>-33.4761666, -70.698435</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69844</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>2026/08/03 22:49:21</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>-33.4761666, -70.698435</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69844</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>02:00:15</t>
+        </is>
+      </c>
+      <c r="L145" t="n">
+        <v>0</v>
+      </c>
+      <c r="M145" t="n">
+        <v>0</v>
+      </c>
+      <c r="N145" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>6</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>2026/08/03 21:14:15</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>-33.4362033, -70.6295249</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>-33.43620, -70.62952</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>2026/08/03 23:15:24</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>-33.4362033, -70.6295249</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>-33.43620, -70.62952</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>02:01:09</t>
+        </is>
+      </c>
+      <c r="L146" t="n">
+        <v>0</v>
+      </c>
+      <c r="M146" t="n">
+        <v>0</v>
+      </c>
+      <c r="N146" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>5</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>2026/08/03 21:53:26</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>-32.838347, -70.955562</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>-32.83835, -70.95556</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>2026/08/03 23:50:57</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>-32.838347, -70.955562</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>-32.83835, -70.95556</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>01:57:31</t>
+        </is>
+      </c>
+      <c r="L147" t="n">
+        <v>0</v>
+      </c>
+      <c r="M147" t="n">
+        <v>0</v>
+      </c>
+      <c r="N147" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8915,13 +9092,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1404.49</v>
+        <v>1404.44</v>
       </c>
       <c r="C3" t="n">
         <v>40</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>143</v>
@@ -8934,13 +9111,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>786.87</v>
+        <v>786.89</v>
       </c>
       <c r="C4" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>145</v>
@@ -9124,13 +9301,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1499.39</v>
+        <v>1499.38</v>
       </c>
       <c r="C14" t="n">
         <v>58</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>140</v>
@@ -9143,13 +9320,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>210.52</v>
+        <v>210.46</v>
       </c>
       <c r="C15" t="n">
         <v>23</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>125</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-05T06:26Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N157"/>
+  <dimension ref="A1:N161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>2026/08/04 21:57:37</t>
+          <t>2026/08/04 23:57:31</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>130:06:29</t>
+          <t>132:06:23</t>
         </is>
       </c>
       <c r="L105" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/08/04 21:41:59</t>
+          <t>2026/08/04 23:41:59</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>105:53:32</t>
+          <t>107:53:32</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -7699,7 +7699,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026/08/04 21:56:11</t>
+          <t>2026/08/04 23:56:11</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>105:32:29</t>
+          <t>107:32:29</t>
         </is>
       </c>
       <c r="L125" t="n">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/08/04 21:02:20</t>
+          <t>2026/08/04 23:02:20</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>08:01:07</t>
+          <t>10:01:07</t>
         </is>
       </c>
       <c r="L142" t="n">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/08/04 22:13:30</t>
+          <t>2026/08/04 23:13:30</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>08:01:03</t>
+          <t>09:01:03</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -8997,26 +8997,26 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/08/04 21:49:43</t>
+          <t>2026/08/04 21:49:26</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>-33.0872116, -71.3622166</t>
+          <t>-33.0872883, -71.3623</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>-33.08721, -71.36222</t>
+          <t>-33.08729, -71.36230</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>03:28:24</t>
+          <t>03:28:07</t>
         </is>
       </c>
       <c r="L147" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="M147" t="n">
         <v>3</v>
@@ -9115,7 +9115,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>2026/08/04 21:35:18</t>
+          <t>2026/08/04 23:35:18</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9130,7 +9130,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>03:01:02</t>
+          <t>05:01:02</t>
         </is>
       </c>
       <c r="L149" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026/08/04 21:44:37</t>
+          <t>2026/08/04 23:44:40</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>03:03:45</t>
+          <t>05:03:48</t>
         </is>
       </c>
       <c r="L150" t="n">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>2026/08/04 21:08:56</t>
+          <t>2026/08/04 23:08:56</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L152" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/08/04 21:42:27</t>
+          <t>2026/08/04 23:42:27</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -9559,60 +9559,296 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>11</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>2026/08/04 21:44:50</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>-32.79758, -70.8870816</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>-32.79758, -70.88708</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>2026/08/04 23:44:50</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>-32.79758, -70.8870816</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>-32.79758, -70.88708</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L157" t="n">
+        <v>0</v>
+      </c>
+      <c r="M157" t="n">
+        <v>0</v>
+      </c>
+      <c r="N157" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCS-53</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>8</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>2026/08/04 21:49:43</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>-33.0872116, -71.3622166</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>-33.08721, -71.36222</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>2026/08/04 23:49:43</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>-33.0872116, -71.3622166</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>-33.08721, -71.36222</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L158" t="n">
+        <v>0</v>
+      </c>
+      <c r="M158" t="n">
+        <v>0</v>
+      </c>
+      <c r="N158" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
           <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
-      <c r="C157" t="n">
+      <c r="C159" t="n">
         <v>20</v>
       </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>Recorridos</t>
-        </is>
-      </c>
-      <c r="E157" t="inlineStr">
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
         <is>
           <t>2026/08/04 21:54:08</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr">
+      <c r="F159" t="inlineStr">
         <is>
           <t>-32.7440749, -70.7328199</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr">
+      <c r="G159" t="inlineStr">
         <is>
           <t>-32.74407, -70.73282</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr">
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>2026/08/04 22:16:28</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>-32.7417916, -70.7364716</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>-32.74179, -70.73647</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>00:22:20</t>
+        </is>
+      </c>
+      <c r="L159" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="M159" t="n">
+        <v>28</v>
+      </c>
+      <c r="N159" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>8</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>2026/08/04 21:59:28</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>-32.838363, -70.955523</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95552</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>2026/08/04 23:57:18</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>-32.838363, -70.955523</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>-32.83836, -70.95552</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>01:57:50</t>
+        </is>
+      </c>
+      <c r="L160" t="n">
+        <v>0</v>
+      </c>
+      <c r="M160" t="n">
+        <v>0</v>
+      </c>
+      <c r="N160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>21</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
         <is>
           <t>2026/08/04 22:16:35</t>
         </is>
       </c>
-      <c r="I157" t="inlineStr">
+      <c r="F161" t="inlineStr">
         <is>
           <t>-32.7416816, -70.7364883</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr">
+      <c r="G161" t="inlineStr">
         <is>
           <t>-32.74168, -70.73649</t>
         </is>
       </c>
-      <c r="K157" t="inlineStr">
-        <is>
-          <t>00:22:27</t>
-        </is>
-      </c>
-      <c r="L157" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="M157" t="n">
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>2026/08/04 22:27:27</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>-32.7440616, -70.732775</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>-32.74406, -70.73278</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>00:10:52</t>
+        </is>
+      </c>
+      <c r="L161" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="M161" t="n">
         <v>28</v>
       </c>
-      <c r="N157" t="n">
-        <v>17</v>
+      <c r="N161" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -9688,7 +9924,7 @@
         <v>40</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>143</v>
@@ -9707,7 +9943,7 @@
         <v>40</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
         <v>145</v>
@@ -9720,10 +9956,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1252.73</v>
+        <v>1253.49</v>
       </c>
       <c r="C5" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -9986,13 +10222,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2367.09</v>
+        <v>2367.06</v>
       </c>
       <c r="C19" t="n">
         <v>76</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-06T06:28Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N165"/>
+  <dimension ref="A1:N167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026/08/05 22:01:31</t>
+          <t>2026/08/05 23:01:59</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>164:00:10</t>
+          <t>165:00:38</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>2026/08/05 21:57:38</t>
+          <t>2026/08/05 23:57:45</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>154:06:30</t>
+          <t>156:06:37</t>
         </is>
       </c>
       <c r="L58" t="n">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026/08/05 21:41:53</t>
+          <t>2026/08/05 23:41:53</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>129:53:26</t>
+          <t>131:53:26</t>
         </is>
       </c>
       <c r="L115" t="n">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>2026/08/05 21:56:10</t>
+          <t>2026/08/05 23:56:10</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>129:32:28</t>
+          <t>131:32:28</t>
         </is>
       </c>
       <c r="L116" t="n">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026/08/05 22:15:36</t>
+          <t>2026/08/05 23:15:35</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>32:03:09</t>
+          <t>33:03:08</t>
         </is>
       </c>
       <c r="L135" t="n">
@@ -9528,7 +9528,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>2026/08/05 22:25:08</t>
+          <t>2026/08/05 23:25:08</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>05:01:01</t>
+          <t>06:01:01</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/08/05 21:23:07</t>
+          <t>2026/08/05 23:23:07</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>02:10:37</t>
+          <t>04:10:37</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026/08/05 22:09:15</t>
+          <t>2026/08/05 23:09:16</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>01:57:31</t>
+          <t>02:57:32</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -10085,6 +10085,124 @@
       </c>
       <c r="N165" t="n">
         <v>43</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>6</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>2026/08/05 21:32:50</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>-33.436355, -70.629265</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>-33.43635, -70.62927</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>2026/08/05 23:32:53</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>-33.436355, -70.629265</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>-33.43635, -70.62927</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>02:00:03</t>
+        </is>
+      </c>
+      <c r="L166" t="n">
+        <v>0</v>
+      </c>
+      <c r="M166" t="n">
+        <v>0</v>
+      </c>
+      <c r="N166" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>12</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>2026/08/05 21:43:14</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>-32.841907, -70.936853</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>-32.84191, -70.93685</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>2026/08/05 23:47:02</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>-32.841907, -70.936853</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>-32.84191, -70.93685</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>02:03:48</t>
+        </is>
+      </c>
+      <c r="L167" t="n">
+        <v>0</v>
+      </c>
+      <c r="M167" t="n">
+        <v>0</v>
+      </c>
+      <c r="N167" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -10382,13 +10500,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>270.03</v>
+        <v>269.97</v>
       </c>
       <c r="C15" t="n">
         <v>28</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>127</v>
@@ -10477,13 +10595,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>863.29</v>
+        <v>863.11</v>
       </c>
       <c r="C20" t="n">
         <v>58</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>137</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-07T05:39Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N167"/>
+  <dimension ref="A1:N173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/08/06 20:01:21</t>
+          <t>2026/08/06 23:01:39</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>163:59:42</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/06 19:57:21</t>
+          <t>2026/08/06 23:57:38</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>163:04:46</t>
+          <t>167:05:03</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2026/08/06 20:41:53</t>
+          <t>2026/08/06 23:41:53</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>152:53:26</t>
+          <t>155:53:26</t>
         </is>
       </c>
       <c r="L41" t="n">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>2026/08/06 19:56:10</t>
+          <t>2026/08/06 23:56:10</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>151:32:28</t>
+          <t>155:32:28</t>
         </is>
       </c>
       <c r="L44" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>2026/08/06 20:22:24</t>
+          <t>2026/08/06 23:22:21</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>80:08:24</t>
+          <t>83:08:21</t>
         </is>
       </c>
       <c r="L99" t="n">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/08/06 20:02:31</t>
+          <t>2026/08/06 22:02:31</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>28:00:00</t>
+          <t>30:00:00</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026/08/06 19:32:53</t>
+          <t>2026/08/06 23:32:53</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>22:00:03</t>
+          <t>26:00:03</t>
         </is>
       </c>
       <c r="L150" t="n">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>2026/08/06 20:18:56</t>
+          <t>2026/08/06 23:18:58</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -9602,7 +9602,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>05:01:02</t>
+          <t>08:01:04</t>
         </is>
       </c>
       <c r="L157" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/08/06 20:49:43</t>
+          <t>2026/08/06 23:49:43</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>05:01:01</t>
+          <t>08:01:01</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -9941,26 +9941,26 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026/08/06 20:29:42</t>
+          <t>2026/08/06 20:27:58</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>-33.3621833, -70.6701533</t>
+          <t>-33.3623416, -70.6701416</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>-33.36218, -70.67015</t>
+          <t>-33.36234, -70.67014</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>02:23:13</t>
+          <t>02:21:29</t>
         </is>
       </c>
       <c r="L163" t="n">
-        <v>36.73</v>
+        <v>36.72</v>
       </c>
       <c r="M163" t="n">
         <v>95</v>
@@ -10000,26 +10000,26 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/08/06 20:09:56</t>
+          <t>2026/08/06 22:11:22</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>-33.0873366, -71.3623333</t>
+          <t>-33.0871766, -71.3622</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>-33.08734, -71.36233</t>
+          <t>-33.08718, -71.36220</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:01:26</t>
         </is>
       </c>
       <c r="L164" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="M164" t="n">
         <v>0</v>
@@ -10177,7 +10177,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026/08/06 20:08:08</t>
+          <t>2026/08/06 23:08:11</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>01:04:28</t>
+          <t>04:04:31</t>
         </is>
       </c>
       <c r="L167" t="n">
@@ -10202,6 +10202,360 @@
         <v>0</v>
       </c>
       <c r="N167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>13</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>2026/08/06 19:07:53</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>-32.8792133, -70.608815</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>-32.87921, -70.60882</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>2026/08/06 23:10:33</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>-32.8792133, -70.608815</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>-32.87921, -70.60882</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>04:02:40</t>
+        </is>
+      </c>
+      <c r="L168" t="n">
+        <v>0</v>
+      </c>
+      <c r="M168" t="n">
+        <v>0</v>
+      </c>
+      <c r="N168" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>9</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>2026/08/06 19:41:25</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>-32.743035, -70.7297983</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>-32.74303, -70.72980</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>2026/08/06 23:41:25</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>-32.743035, -70.7297983</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>-32.74303, -70.72980</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>04:00:00</t>
+        </is>
+      </c>
+      <c r="L169" t="n">
+        <v>0</v>
+      </c>
+      <c r="M169" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>13</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>2026/08/06 20:29:13</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>-33.3621833, -70.6701533</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>-33.36218, -70.67015</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>2026/08/06 21:52:41</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>-33.476235, -70.6982433</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>-33.47624, -70.69824</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>01:23:28</t>
+        </is>
+      </c>
+      <c r="L170" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="M170" t="n">
+        <v>98</v>
+      </c>
+      <c r="N170" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>9</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>2026/08/06 20:30:25</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>-32.838372, -70.955502</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>-32.83837, -70.95550</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>2026/08/06 23:28:26</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>-32.838372, -70.955502</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>-32.83837, -70.95550</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>02:58:01</t>
+        </is>
+      </c>
+      <c r="L171" t="n">
+        <v>0</v>
+      </c>
+      <c r="M171" t="n">
+        <v>0</v>
+      </c>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>OPEL COMBO</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>11</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>2026/08/06 21:41:04</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>-32.7975549, -70.8870483</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>-32.79755, -70.88705</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>2026/08/06 23:41:43</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>-32.7975549, -70.8870483</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>-32.79755, -70.88705</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>02:00:39</t>
+        </is>
+      </c>
+      <c r="L172" t="n">
+        <v>0</v>
+      </c>
+      <c r="M172" t="n">
+        <v>0</v>
+      </c>
+      <c r="N172" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>14</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>2026/08/06 21:53:56</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>-33.4761583, -70.69843</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>-33.47616, -70.69843</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>2026/08/06 23:56:15</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>-33.4761583, -70.69843</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>-33.47616, -70.69843</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>02:02:19</t>
+        </is>
+      </c>
+      <c r="L173" t="n">
+        <v>0</v>
+      </c>
+      <c r="M173" t="n">
+        <v>0</v>
+      </c>
+      <c r="N173" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10272,13 +10626,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1107.06</v>
+        <v>1107.01</v>
       </c>
       <c r="C3" t="n">
         <v>42</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>138</v>
@@ -10310,13 +10664,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1093.23</v>
+        <v>1093.21</v>
       </c>
       <c r="C5" t="n">
         <v>82</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>133</v>
@@ -10481,13 +10835,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1245.88</v>
+        <v>1266.29</v>
       </c>
       <c r="C14" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>140</v>
@@ -10519,13 +10873,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>339.1</v>
+        <v>357.28</v>
       </c>
       <c r="C16" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
         <v>122</v>
@@ -10576,13 +10930,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1777.89</v>
+        <v>1777.88</v>
       </c>
       <c r="C19" t="n">
         <v>69</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-08T04:54Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N164"/>
+  <dimension ref="A1:N166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/08/07 21:01:39</t>
+          <t>2026/08/07 23:01:38</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:00:12</t>
+          <t>167:00:11</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/08/07 20:56:10</t>
+          <t>2026/08/07 23:56:10</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>164:32:26</t>
+          <t>167:32:26</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/07 20:43:00</t>
+          <t>2026/08/07 23:43:00</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>163:54:30</t>
+          <t>166:54:30</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/08/07 20:57:45</t>
+          <t>2026/08/07 23:57:43</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>163:58:38</t>
+          <t>166:58:36</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/08/07 20:02:31</t>
+          <t>2026/08/07 22:02:31</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>52:00:00</t>
+          <t>54:00:00</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026/08/07 21:15:47</t>
+          <t>2026/08/07 23:15:52</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>29:57:53</t>
+          <t>31:57:58</t>
         </is>
       </c>
       <c r="L150" t="n">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/08/07 20:46:39</t>
+          <t>2026/08/07 23:46:31</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>28:57:57</t>
+          <t>31:57:49</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>2026/08/07 20:26:01</t>
+          <t>2026/08/07 22:26:01</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -9897,7 +9897,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L162" t="n">
@@ -9913,11 +9913,11 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -9926,37 +9926,37 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>2026/08/07 18:47:36</t>
+          <t>2026/08/07 19:14:25</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>-32.8791883, -70.6088133</t>
+          <t>-32.7975866, -70.8871233</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>-32.87919, -70.60881</t>
+          <t>-32.79759, -70.88712</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>2026/08/07 20:49:11</t>
+          <t>2026/08/07 23:23:53</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>-32.8791883, -70.6088133</t>
+          <t>-32.7975866, -70.8871233</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>-32.87919, -70.60881</t>
+          <t>-32.79759, -70.88712</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>02:01:35</t>
+          <t>04:09:28</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -9972,11 +9972,11 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D164" t="inlineStr">
         <is>
@@ -9985,37 +9985,37 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>2026/08/07 19:14:25</t>
+          <t>2026/08/07 20:35:22</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>-32.7975866, -70.8871233</t>
+          <t>-32.7430399, -70.7298066</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>-32.79759, -70.88712</t>
+          <t>-32.74304, -70.72981</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/08/07 21:23:53</t>
+          <t>2026/08/07 22:35:22</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>-32.7975866, -70.8871233</t>
+          <t>-32.7430399, -70.7298066</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>-32.79759, -70.88712</t>
+          <t>-32.74304, -70.72981</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>02:09:28</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -10025,6 +10025,124 @@
         <v>0</v>
       </c>
       <c r="N164" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>9</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>2026/08/07 21:09:04</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>-32.841921, -70.936836</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>-32.84192, -70.93684</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>2026/08/07 23:12:46</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>-32.841683, -70.936821</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>-32.84168, -70.93682</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>02:03:42</t>
+        </is>
+      </c>
+      <c r="L165" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M165" t="n">
+        <v>0</v>
+      </c>
+      <c r="N165" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>9</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>2026/08/07 21:23:35</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>-33.4762083, -70.6984066</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>-33.47621, -70.69841</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>2026/08/07 23:25:07</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>-33.4762083, -70.6984066</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>-33.47621, -70.69841</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>02:01:32</t>
+        </is>
+      </c>
+      <c r="L166" t="n">
+        <v>0</v>
+      </c>
+      <c r="M166" t="n">
+        <v>0</v>
+      </c>
+      <c r="N166" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10095,7 +10213,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1242.77</v>
+        <v>1242.81</v>
       </c>
       <c r="C3" t="n">
         <v>43</v>
@@ -10114,13 +10232,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1300.56</v>
+        <v>1300.55</v>
       </c>
       <c r="C4" t="n">
         <v>59</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
         <v>145</v>
@@ -10133,13 +10251,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1104.5</v>
+        <v>1104.49</v>
       </c>
       <c r="C5" t="n">
         <v>90</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>133</v>
@@ -10304,13 +10422,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1701.44</v>
+        <v>1701.37</v>
       </c>
       <c r="C14" t="n">
         <v>57</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>144</v>
@@ -10399,13 +10517,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1624.2</v>
+        <v>1626.81</v>
       </c>
       <c r="C19" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
         <v>137</v>
@@ -10418,13 +10536,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>876.5</v>
+        <v>876.46</v>
       </c>
       <c r="C20" t="n">
         <v>64</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>143</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-09T05:02Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N167"/>
+  <dimension ref="A1:N170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/08/08 21:01:21</t>
+          <t>2026/08/08 23:02:27</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>164:59:59</t>
+          <t>167:01:05</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/08/08 20:43:00</t>
+          <t>2026/08/08 23:43:00</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>164:01:27</t>
+          <t>167:01:27</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/08/08 20:56:10</t>
+          <t>2026/08/08 23:56:10</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>164:00:42</t>
+          <t>167:00:42</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/08 20:57:43</t>
+          <t>2026/08/08 23:57:38</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>164:00:06</t>
+          <t>167:00:01</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026/08/08 21:13:22</t>
+          <t>2026/08/08 23:13:39</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>161:59:37</t>
+          <t>163:59:54</t>
         </is>
       </c>
       <c r="L26" t="n">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/08/08 20:02:31</t>
+          <t>2026/08/08 22:02:31</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>76:00:00</t>
+          <t>78:00:00</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -9233,7 +9233,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2026/08/08 21:15:27</t>
+          <t>2026/08/08 23:15:47</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>53:57:33</t>
+          <t>55:57:53</t>
         </is>
       </c>
       <c r="L151" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/08/08 20:46:39</t>
+          <t>2026/08/08 23:46:40</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>52:57:57</t>
+          <t>55:57:58</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>2026/08/08 20:28:23</t>
+          <t>2026/08/08 22:28:23</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>02:00:20</t>
+          <t>04:00:20</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2026/08/08 20:32:55</t>
+          <t>2026/08/08 22:32:55</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L165" t="n">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>2026/08/08 21:24:32</t>
+          <t>2026/08/08 23:24:32</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -10149,11 +10149,11 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCL-70</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D167" t="inlineStr">
         <is>
@@ -10162,37 +10162,37 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>2026/08/08 19:56:55</t>
+          <t>2026/08/08 20:19:13</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>-32.791603, -71.19195</t>
+          <t>-32.7430149, -70.7298233</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>-32.79160, -71.19195</t>
+          <t>-32.74301, -70.72982</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026/08/08 20:01:56</t>
+          <t>2026/08/08 22:19:13</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>-32.791603, -71.19195</t>
+          <t>-32.7430149, -70.7298233</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>-32.79160, -71.19195</t>
+          <t>-32.74301, -70.72982</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>00:05:01</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="L167" t="n">
@@ -10202,6 +10202,183 @@
         <v>0</v>
       </c>
       <c r="N167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>2</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>2026/08/08 20:33:40</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>-33.4362383, -70.629435</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>-33.43624, -70.62944</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>2026/08/08 22:33:40</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>-33.4362383, -70.629435</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>-33.43624, -70.62944</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L168" t="n">
+        <v>0</v>
+      </c>
+      <c r="M168" t="n">
+        <v>0</v>
+      </c>
+      <c r="N168" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>5</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>2026/08/08 21:03:56</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>-33.4762183, -70.6984383</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>-33.47622, -70.69844</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>2026/08/08 23:04:02</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>-33.4762183, -70.6984383</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>-33.47622, -70.69844</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>02:00:06</t>
+        </is>
+      </c>
+      <c r="L169" t="n">
+        <v>0</v>
+      </c>
+      <c r="M169" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>2</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>2026/08/08 21:28:43</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>-32.841679, -70.936837</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>-32.84168, -70.93684</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>2026/08/08 23:29:44</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>-32.841679, -70.936837</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>-32.84168, -70.93684</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>02:01:01</t>
+        </is>
+      </c>
+      <c r="L170" t="n">
+        <v>0</v>
+      </c>
+      <c r="M170" t="n">
+        <v>0</v>
+      </c>
+      <c r="N170" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10272,13 +10449,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1196.28</v>
+        <v>1196.38</v>
       </c>
       <c r="C3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>138</v>
@@ -10310,13 +10487,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1055.65</v>
+        <v>1055.64</v>
       </c>
       <c r="C5" t="n">
         <v>85</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>133</v>
@@ -10487,7 +10664,7 @@
         <v>54</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>144</v>
@@ -10500,13 +10677,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>254.43</v>
+        <v>254.38</v>
       </c>
       <c r="C15" t="n">
         <v>29</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>127</v>
@@ -10601,7 +10778,7 @@
         <v>65</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>143</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-10T05:25Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N169"/>
+  <dimension ref="A1:N172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/08/09 21:01:38</t>
+          <t>2026/08/09 23:01:22</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:00:14</t>
+          <t>166:59:58</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/08/09 21:13:38</t>
+          <t>2026/08/09 23:13:38</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>164:59:30</t>
+          <t>166:59:30</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/08/09 20:41:36</t>
+          <t>2026/08/09 23:41:36</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>164:00:03</t>
+          <t>167:00:03</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/08/09 20:56:09</t>
+          <t>2026/08/09 23:56:09</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>164:00:41</t>
+          <t>167:00:41</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2026/08/09 21:22:27</t>
+          <t>2026/08/09 23:24:43</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3171,7 +3171,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>153:08:27</t>
+          <t>155:10:43</t>
         </is>
       </c>
       <c r="L48" t="n">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>2026/08/09 20:02:31</t>
+          <t>2026/08/09 22:02:31</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>100:00:00</t>
+          <t>102:00:00</t>
         </is>
       </c>
       <c r="L139" t="n">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>2026/08/09 21:30:09</t>
+          <t>2026/08/09 23:30:18</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>78:12:15</t>
+          <t>80:12:24</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>2026/08/09 20:33:40</t>
+          <t>2026/08/09 22:33:40</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>24:00:00</t>
+          <t>26:00:00</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026/08/09 21:04:02</t>
+          <t>2026/08/09 23:04:02</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>24:00:06</t>
+          <t>26:00:06</t>
         </is>
       </c>
       <c r="L167" t="n">
@@ -10236,7 +10236,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>2026/08/09 20:02:51</t>
+          <t>2026/08/09 22:02:51</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L168" t="n">
@@ -10295,7 +10295,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>2026/08/09 20:06:11</t>
+          <t>2026/08/09 22:06:11</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>02:01:27</t>
+          <t>04:01:27</t>
         </is>
       </c>
       <c r="L169" t="n">
@@ -10320,6 +10320,183 @@
         <v>0</v>
       </c>
       <c r="N169" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>6</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>2026/08/09 19:48:44</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>-32.8791983, -70.6088283</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>-32.87920, -70.60883</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>2026/08/09 23:48:44</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>-32.8791983, -70.6088283</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>-32.87920, -70.60883</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>04:00:00</t>
+        </is>
+      </c>
+      <c r="L170" t="n">
+        <v>0</v>
+      </c>
+      <c r="M170" t="n">
+        <v>0</v>
+      </c>
+      <c r="N170" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCS-53</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>14</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>2026/08/09 20:21:04</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>-33.087275, -71.3622883</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>-33.08727, -71.36229</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>2026/08/09 22:21:04</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>-33.087275, -71.3622883</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>-33.08727, -71.36229</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L171" t="n">
+        <v>0</v>
+      </c>
+      <c r="M171" t="n">
+        <v>0</v>
+      </c>
+      <c r="N171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>7</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>2026/08/09 21:31:12</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>-32.841651, -70.936805</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>-32.84165, -70.93681</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>2026/08/09 23:34:11</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>-32.841651, -70.936805</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>-32.84165, -70.93681</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>02:02:59</t>
+        </is>
+      </c>
+      <c r="L172" t="n">
+        <v>0</v>
+      </c>
+      <c r="M172" t="n">
+        <v>0</v>
+      </c>
+      <c r="N172" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10409,13 +10586,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1014.46</v>
+        <v>1014.45</v>
       </c>
       <c r="C4" t="n">
         <v>63</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
         <v>132</v>
@@ -10694,13 +10871,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1554.6</v>
+        <v>1554.58</v>
       </c>
       <c r="C19" t="n">
         <v>80</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>137</v>
@@ -10713,13 +10890,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>883.61</v>
+        <v>883.42</v>
       </c>
       <c r="C20" t="n">
         <v>66</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>143</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-11T05:06Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N160"/>
+  <dimension ref="A1:N163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/08/10 21:01:22</t>
+          <t>2026/08/10 23:02:07</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>164:59:44</t>
+          <t>167:00:29</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/08/10 21:13:22</t>
+          <t>2026/08/10 23:13:38</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>165:00:01</t>
+          <t>167:00:17</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/08/10 21:23:38</t>
+          <t>2026/08/10 23:23:19</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>165:08:14</t>
+          <t>167:07:55</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/08/10 20:41:36</t>
+          <t>2026/08/10 23:41:36</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>163:59:37</t>
+          <t>166:59:37</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/08/10 20:56:09</t>
+          <t>2026/08/10 23:56:09</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>163:59:58</t>
+          <t>166:59:58</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026/08/10 20:02:31</t>
+          <t>2026/08/10 22:02:31</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>124:00:00</t>
+          <t>126:00:00</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/08/10 21:30:39</t>
+          <t>2026/08/10 23:30:09</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>102:12:45</t>
+          <t>104:12:15</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -9646,7 +9646,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>2026/08/10 20:58:44</t>
+          <t>2026/08/10 22:58:44</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>04:02:34</t>
+          <t>06:02:34</t>
         </is>
       </c>
       <c r="L158" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>2026/08/10 20:30:50</t>
+          <t>2026/08/10 22:30:50</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L159" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>2026/08/10 21:21:19</t>
+          <t>2026/08/10 23:21:22</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>02:04:37</t>
+          <t>04:04:40</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -9789,6 +9789,183 @@
         <v>0</v>
       </c>
       <c r="N160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>8</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>2026/08/10 21:08:46</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>-33.4761449, -70.69843</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>-33.47614, -70.69843</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>2026/08/10 23:08:46</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>-33.4761449, -70.69843</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>-33.47614, -70.69843</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L161" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" t="n">
+        <v>0</v>
+      </c>
+      <c r="N161" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>7</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>2026/08/10 21:15:06</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>-33.4368166, -70.6288133</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>-33.43682, -70.62881</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>2026/08/10 23:15:06</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>-33.4368166, -70.6288133</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>-33.43682, -70.62881</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L162" t="n">
+        <v>0</v>
+      </c>
+      <c r="M162" t="n">
+        <v>0</v>
+      </c>
+      <c r="N162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>14</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>2026/08/10 21:41:03</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>-32.7431366, -70.729665</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>-32.74314, -70.72966</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>2026/08/10 23:41:35</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>-32.7430399, -70.7297549</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>-32.74304, -70.72975</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>02:00:32</t>
+        </is>
+      </c>
+      <c r="L163" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M163" t="n">
+        <v>0</v>
+      </c>
+      <c r="N163" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9897,13 +10074,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1214.61</v>
+        <v>1215.15</v>
       </c>
       <c r="C5" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>133</v>
@@ -10068,13 +10245,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1489.34</v>
+        <v>1489.33</v>
       </c>
       <c r="C14" t="n">
         <v>46</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>144</v>
@@ -10087,13 +10264,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>171.26</v>
+        <v>171.21</v>
       </c>
       <c r="C15" t="n">
         <v>24</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>137</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-12T05:36Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N154"/>
+  <dimension ref="A1:N155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/08/11 21:01:39</t>
+          <t>2026/08/11 23:01:58</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>165:00:18</t>
+          <t>167:00:37</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -678,7 +678,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/08/11 21:13:38</t>
+          <t>2026/08/11 23:13:21</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>165:00:17</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L6" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/08/11 21:22:28</t>
+          <t>2026/08/11 23:23:04</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>164:59:49</t>
+          <t>167:00:25</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/08/11 21:42:01</t>
+          <t>2026/08/11 23:42:01</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>165:00:02</t>
+          <t>167:00:02</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/08/11 20:56:03</t>
+          <t>2026/08/11 23:56:03</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>163:59:52</t>
+          <t>166:59:52</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/08/11 21:30:24</t>
+          <t>2026/08/11 23:30:24</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>126:12:30</t>
+          <t>128:12:30</t>
         </is>
       </c>
       <c r="L126" t="n">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/08/11 21:34:39</t>
+          <t>2026/08/11 23:34:21</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>66:59:30</t>
+          <t>68:59:12</t>
         </is>
       </c>
       <c r="L147" t="n">
@@ -9056,7 +9056,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2026/08/11 20:20:29</t>
+          <t>2026/08/11 22:20:29</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>06:25:47</t>
+          <t>08:25:47</t>
         </is>
       </c>
       <c r="L148" t="n">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>2026/08/11 20:00:31</t>
+          <t>2026/08/11 22:00:31</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9130,7 +9130,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L149" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026/08/11 21:11:42</t>
+          <t>2026/08/11 23:11:42</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>03:11:03</t>
+          <t>05:11:03</t>
         </is>
       </c>
       <c r="L150" t="n">
@@ -9233,7 +9233,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2026/08/11 20:03:18</t>
+          <t>2026/08/11 22:03:18</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L151" t="n">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>2026/08/11 20:30:04</t>
+          <t>2026/08/11 22:30:04</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L152" t="n">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/08/11 20:52:11</t>
+          <t>2026/08/11 22:52:11</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>02:11:35</t>
+          <t>04:11:35</t>
         </is>
       </c>
       <c r="L153" t="n">
@@ -9410,7 +9410,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/08/11 21:38:31</t>
+          <t>2026/08/11 23:38:31</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -9435,6 +9435,65 @@
         <v>0</v>
       </c>
       <c r="N154" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>12</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2026/08/11 20:12:51</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.6984516</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69845</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>2026/08/11 22:12:51</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.6984516</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69845</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L155" t="n">
+        <v>0</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0</v>
+      </c>
+      <c r="N155" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9505,7 +9564,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1601.72</v>
+        <v>1605.96</v>
       </c>
       <c r="C3" t="n">
         <v>28</v>
@@ -9714,13 +9773,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1695.56</v>
+        <v>1695.55</v>
       </c>
       <c r="C14" t="n">
         <v>53</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>144</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-13T05:38Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N151"/>
+  <dimension ref="A1:N154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/08/12 21:13:21</t>
+          <t>2026/08/12 23:13:38</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>165:00:06</t>
+          <t>167:00:23</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/08/12 21:23:22</t>
+          <t>2026/08/12 23:24:22</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>164:59:58</t>
+          <t>167:00:58</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/12 21:42:01</t>
+          <t>2026/08/12 23:42:01</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>165:00:08</t>
+          <t>167:00:08</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/08/12 20:56:03</t>
+          <t>2026/08/12 23:56:03</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>163:59:53</t>
+          <t>166:59:53</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/08/12 21:46:18</t>
+          <t>2026/08/12 23:46:25</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>17:59:39</t>
+          <t>19:59:46</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026/08/12 21:38:08</t>
+          <t>2026/08/12 23:38:08</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>10:34:00</t>
+          <t>12:34:00</t>
         </is>
       </c>
       <c r="L141" t="n">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/08/12 21:40:56</t>
+          <t>2026/08/12 23:40:39</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>08:57:50</t>
+          <t>10:57:33</t>
         </is>
       </c>
       <c r="L142" t="n">
@@ -8938,7 +8938,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/08/12 21:32:28</t>
+          <t>2026/08/12 23:32:28</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>05:01:09</t>
+          <t>07:01:09</t>
         </is>
       </c>
       <c r="L146" t="n">
@@ -9056,7 +9056,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2026/08/12 21:27:06</t>
+          <t>2026/08/12 22:09:13</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>04:42:07</t>
         </is>
       </c>
       <c r="L148" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026/08/12 20:50:21</t>
+          <t>2026/08/12 22:50:21</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L150" t="n">
@@ -9233,7 +9233,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2026/08/12 21:27:55</t>
+          <t>2026/08/12 23:27:55</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>02:00:17</t>
+          <t>04:00:17</t>
         </is>
       </c>
       <c r="L151" t="n">
@@ -9258,6 +9258,183 @@
         <v>0</v>
       </c>
       <c r="N151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>11</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>2026/08/12 20:43:17</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>-32.8792183, -70.6088016</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>-32.87922, -70.60880</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>2026/08/12 22:43:17</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>-32.8792183, -70.6088016</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>-32.87922, -70.60880</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L152" t="n">
+        <v>0</v>
+      </c>
+      <c r="M152" t="n">
+        <v>0</v>
+      </c>
+      <c r="N152" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>JAC X200 SJTJ-50</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>10</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>2026/08/12 21:07:09</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>-32.7430766, -70.7297583</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>-32.74308, -70.72976</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>2026/08/12 23:07:10</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>-32.7430766, -70.7297583</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>-32.74308, -70.72976</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>02:00:01</t>
+        </is>
+      </c>
+      <c r="L153" t="n">
+        <v>0</v>
+      </c>
+      <c r="M153" t="n">
+        <v>0</v>
+      </c>
+      <c r="N153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>5</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2026/08/12 21:45:37</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>-33.4371533, -70.6287916</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>-33.43715, -70.62879</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>2026/08/12 23:45:37</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>-33.4371533, -70.6287916</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>-33.43715, -70.62879</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9328,7 +9505,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1466.28</v>
+        <v>1470.48</v>
       </c>
       <c r="C3" t="n">
         <v>18</v>
@@ -9366,13 +9543,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1262.57</v>
+        <v>1262.56</v>
       </c>
       <c r="C5" t="n">
         <v>64</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>133</v>
@@ -9556,13 +9733,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>157.86</v>
+        <v>157.81</v>
       </c>
       <c r="C15" t="n">
         <v>23</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>137</v>
@@ -9632,13 +9809,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>433.62</v>
+        <v>433.6</v>
       </c>
       <c r="C19" t="n">
         <v>66</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>129</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-13T16:54Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N154"/>
+  <dimension ref="A1:N155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9323,11 +9323,11 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>JAC X200 SJTJ-50</t>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -9336,41 +9336,41 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2026/08/12 21:07:09</t>
+          <t>2026/08/12 21:04:21</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>-32.7430766, -70.7297583</t>
+          <t>-32.841977, -70.936819</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>-32.74308, -70.72976</t>
+          <t>-32.84198, -70.93682</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/08/12 23:07:10</t>
+          <t>2026/08/12 23:40:26</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>-32.7430766, -70.7297583</t>
+          <t>-32.841671, -70.936791</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>-32.74308, -70.72976</t>
+          <t>-32.84167, -70.93679</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>02:00:01</t>
+          <t>02:36:05</t>
         </is>
       </c>
       <c r="L153" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="M153" t="n">
         <v>0</v>
@@ -9382,11 +9382,11 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -9395,37 +9395,37 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>2026/08/12 21:45:37</t>
+          <t>2026/08/12 21:07:09</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>-33.4371533, -70.6287916</t>
+          <t>-32.7430766, -70.7297583</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>-33.43715, -70.62879</t>
+          <t>-32.74308, -70.72976</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>2026/08/12 23:45:37</t>
+          <t>2026/08/12 23:07:10</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>-33.4371533, -70.6287916</t>
+          <t>-32.7430766, -70.7297583</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>-33.43715, -70.62879</t>
+          <t>-32.74308, -70.72976</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>02:00:01</t>
         </is>
       </c>
       <c r="L154" t="n">
@@ -9435,6 +9435,65 @@
         <v>0</v>
       </c>
       <c r="N154" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>5</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2026/08/12 21:45:37</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>-33.4371533, -70.6287916</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>-33.43715, -70.62879</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>2026/08/12 23:45:37</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>-33.4371533, -70.6287916</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>-33.43715, -70.62879</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L155" t="n">
+        <v>0</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0</v>
+      </c>
+      <c r="N155" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9828,13 +9887,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1023.15</v>
+        <v>1050</v>
       </c>
       <c r="C20" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>143</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-14T05:36Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N133"/>
+  <dimension ref="A1:N135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/08/13 21:13:38</t>
+          <t>2026/08/13 23:13:21</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>165:00:24</t>
+          <t>167:00:07</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/08/13 21:23:21</t>
+          <t>2026/08/13 23:23:02</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>164:59:40</t>
+          <t>166:59:21</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/08/13 21:42:27</t>
+          <t>2026/08/13 23:42:27</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>165:00:34</t>
+          <t>167:00:34</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/08/13 20:56:50</t>
+          <t>2026/08/13 23:56:50</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>164:00:40</t>
+          <t>167:00:40</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/08/13 21:40:39</t>
+          <t>2026/08/13 23:40:41</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>32:57:33</t>
+          <t>34:57:35</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2026/08/13 21:34:43</t>
+          <t>2026/08/13 23:34:15</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>29:03:24</t>
+          <t>31:02:56</t>
         </is>
       </c>
       <c r="L121" t="n">
@@ -7817,7 +7817,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>2026/08/13 21:12:53</t>
+          <t>2026/08/13 23:12:53</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7832,7 +7832,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="L127" t="n">
@@ -7935,7 +7935,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>2026/08/13 21:06:54</t>
+          <t>2026/08/13 23:06:54</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L129" t="n">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/08/13 20:40:55</t>
+          <t>2026/08/13 22:40:55</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>03:30:41</t>
+          <t>05:30:41</t>
         </is>
       </c>
       <c r="L130" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/08/13 21:43:02</t>
+          <t>2026/08/13 23:43:02</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>04:23:32</t>
+          <t>06:23:32</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/08/13 21:10:22</t>
+          <t>2026/08/13 23:10:22</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/08/13 21:15:00</t>
+          <t>2026/08/13 23:15:00</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>02:00:34</t>
+          <t>04:00:34</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -8196,6 +8196,124 @@
         <v>0</v>
       </c>
       <c r="N133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>OPEL COMBO</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>5</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2026/08/13 20:10:12</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>-32.7432133, -70.72965</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>-32.74321, -70.72965</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>2026/08/13 22:13:21</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>-32.7431399, -70.7297183</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>-32.74314, -70.72972</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>02:03:09</t>
+        </is>
+      </c>
+      <c r="L134" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M134" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>11</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2026/08/13 20:59:47</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>-33.482167, -70.764903</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>-33.48217, -70.76490</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>2026/08/13 23:03:47</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>-33.482167, -70.764903</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>-33.48217, -70.76490</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>02:04:00</t>
+        </is>
+      </c>
+      <c r="L135" t="n">
+        <v>0</v>
+      </c>
+      <c r="M135" t="n">
+        <v>0</v>
+      </c>
+      <c r="N135" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8513,13 +8631,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>745.85</v>
+        <v>745.84</v>
       </c>
       <c r="C16" t="n">
         <v>44</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
         <v>142</v>
@@ -8589,13 +8707,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1142.83</v>
+        <v>1142.79</v>
       </c>
       <c r="C20" t="n">
         <v>58</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>140</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-15T04:28Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N120"/>
+  <dimension ref="A1:N122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/08/14 20:13:26</t>
+          <t>2026/08/14 23:13:38</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>164:00:11</t>
+          <t>167:00:23</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/08/14 20:23:20</t>
+          <t>2026/08/14 23:22:48</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>164:00:42</t>
+          <t>167:00:10</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/08/14 20:42:27</t>
+          <t>2026/08/14 23:42:27</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>163:59:27</t>
+          <t>166:59:27</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/08/14 20:56:50</t>
+          <t>2026/08/14 23:56:50</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>164:00:40</t>
+          <t>167:00:40</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>2026/08/14 21:01:22</t>
+          <t>2026/08/14 23:02:07</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>56:18:16</t>
+          <t>58:19:01</t>
         </is>
       </c>
       <c r="L99" t="n">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>2026/08/14 20:34:53</t>
+          <t>2026/08/14 23:34:36</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>52:03:34</t>
+          <t>55:03:17</t>
         </is>
       </c>
       <c r="L103" t="n">
@@ -6932,22 +6932,22 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>2026/08/14 20:32:33</t>
+          <t>2026/08/14 23:13:53</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>-33.360003, -70.807248</t>
+          <t>-33.360021, -70.807295</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>-33.36000, -70.80725</t>
+          <t>-33.36002, -70.80729</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>29:32:55</t>
+          <t>32:14:15</t>
         </is>
       </c>
       <c r="L112" t="n">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026/08/14 19:43:02</t>
+          <t>2026/08/14 23:43:02</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>26:23:32</t>
+          <t>30:23:32</t>
         </is>
       </c>
       <c r="L115" t="n">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>2026/08/14 20:35:38</t>
+          <t>2026/08/14 22:35:38</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>06:20:00</t>
+          <t>08:20:00</t>
         </is>
       </c>
       <c r="L116" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/08/14 19:39:31</t>
+          <t>2026/08/14 23:39:31</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -7286,22 +7286,22 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026/08/14 19:51:36</t>
+          <t>2026/08/14 23:08:12</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>-33.0873266, -71.3623383</t>
+          <t>-33.0873066, -71.3623283</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>-33.08733, -71.36234</t>
+          <t>-33.08731, -71.36233</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>02:00:02</t>
+          <t>05:16:38</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -7376,11 +7376,11 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -7389,37 +7389,37 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>2026/08/14 18:36:51</t>
+          <t>2026/08/14 19:32:31</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>-32.7433466, -70.7325849</t>
+          <t>-32.7975733, -70.8870516</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>-32.74335, -70.73258</t>
+          <t>-32.79757, -70.88705</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/08/14 20:39:18</t>
+          <t>2026/08/14 23:33:01</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>-32.7433466, -70.7325849</t>
+          <t>-32.7975733, -70.8870516</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>-32.74335, -70.73258</t>
+          <t>-32.79757, -70.88705</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>02:02:27</t>
+          <t>04:00:30</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -7429,6 +7429,124 @@
         <v>0</v>
       </c>
       <c r="N120" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>11</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2026/08/14 21:01:30</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>-33.476315, -70.6983766</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>-33.47631, -70.69838</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>2026/08/14 23:03:21</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>-33.47618, -70.6984266</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>-33.47618, -70.69843</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>02:01:51</t>
+        </is>
+      </c>
+      <c r="L121" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M121" t="n">
+        <v>0</v>
+      </c>
+      <c r="N121" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>OPEL COMBO</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>3</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2026/08/14 22:27:34</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>-32.7432366, -70.7296983</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>-32.74324, -70.72970</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2026/08/14 22:33:48</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>-32.7430716, -70.7297316</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>-32.74307, -70.72973</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>00:06:14</t>
+        </is>
+      </c>
+      <c r="L122" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M122" t="n">
+        <v>0</v>
+      </c>
+      <c r="N122" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7480,13 +7598,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>524.0599999999999</v>
+        <v>524.02</v>
       </c>
       <c r="C2" t="n">
         <v>27</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>157</v>
@@ -7708,13 +7826,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1194.32</v>
+        <v>1194.3</v>
       </c>
       <c r="C14" t="n">
         <v>46</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>127</v>
@@ -7746,10 +7864,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>812.03</v>
+        <v>812.71</v>
       </c>
       <c r="C16" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -7822,10 +7940,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1079.94</v>
+        <v>1151.02</v>
       </c>
       <c r="C20" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-15T20:20Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N122"/>
+  <dimension ref="A1:N123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7547,6 +7547,65 @@
         <v>0</v>
       </c>
       <c r="N122" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>13</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2026/08/14 23:06:22</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>-32.841915, -70.936789</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>-32.84192, -70.93679</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2026/08/14 23:59:56</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>-32.841668, -70.936825</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>-32.84167, -70.93682</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>00:53:34</t>
+        </is>
+      </c>
+      <c r="L123" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M123" t="n">
+        <v>0</v>
+      </c>
+      <c r="N123" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7940,13 +7999,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1151.02</v>
+        <v>1174.05</v>
       </c>
       <c r="C20" t="n">
         <v>62</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>140</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-16T04:33Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N124"/>
+  <dimension ref="A1:N125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/08/15 20:13:14</t>
+          <t>2026/08/15 23:13:21</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>163:59:53</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/08/15 20:22:48</t>
+          <t>2026/08/15 23:22:40</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>163:59:11</t>
+          <t>166:59:03</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/15 20:42:52</t>
+          <t>2026/08/15 23:42:52</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>163:59:52</t>
+          <t>166:59:52</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/08/15 20:57:15</t>
+          <t>2026/08/15 23:57:15</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>164:01:05</t>
+          <t>167:01:05</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026/08/15 20:57:40</t>
+          <t>2026/08/15 23:57:21</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>163:00:11</t>
+          <t>165:59:52</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>2026/08/15 20:34:38</t>
+          <t>2026/08/15 23:34:25</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>76:03:19</t>
+          <t>79:03:06</t>
         </is>
       </c>
       <c r="L103" t="n">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026/08/15 20:13:39</t>
+          <t>2026/08/15 23:13:40</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>53:14:01</t>
+          <t>56:14:02</t>
         </is>
       </c>
       <c r="L113" t="n">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>2026/08/15 19:43:02</t>
+          <t>2026/08/15 23:43:02</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>50:23:32</t>
+          <t>54:23:32</t>
         </is>
       </c>
       <c r="L116" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/08/15 19:39:31</t>
+          <t>2026/08/15 23:39:31</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>28:00:00</t>
+          <t>32:00:00</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -7345,26 +7345,26 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/08/15 18:40:38</t>
+          <t>2026/08/15 23:19:02</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>-32.780822, -70.981241</t>
+          <t>-32.780854, -70.981269</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>-32.78082, -70.98124</t>
+          <t>-32.78085, -70.98127</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>24:28:38</t>
+          <t>29:07:02</t>
         </is>
       </c>
       <c r="L119" t="n">
-        <v>7.88</v>
+        <v>10.33</v>
       </c>
       <c r="M119" t="n">
         <v>0</v>
@@ -7404,7 +7404,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/08/15 20:33:48</t>
+          <t>2026/08/15 22:33:48</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>22:06:14</t>
+          <t>24:06:14</t>
         </is>
       </c>
       <c r="L120" t="n">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/08/15 19:55:52</t>
+          <t>2026/08/15 23:55:52</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>08:01:06</t>
+          <t>12:01:06</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7581,7 +7581,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/08/15 20:15:02</t>
+          <t>2026/08/15 22:15:02</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>02:01:06</t>
+          <t>04:01:06</t>
         </is>
       </c>
       <c r="L123" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/08/15 20:41:19</t>
+          <t>2026/08/15 22:41:19</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -7665,6 +7665,65 @@
         <v>0</v>
       </c>
       <c r="N124" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>4</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2026/08/15 20:30:16</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>-32.8792166, -70.6088099</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>-32.87922, -70.60881</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>2026/08/15 22:32:53</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>-32.8792166, -70.6088099</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>-32.87922, -70.60881</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>02:02:37</t>
+        </is>
+      </c>
+      <c r="L125" t="n">
+        <v>0</v>
+      </c>
+      <c r="M125" t="n">
+        <v>0</v>
+      </c>
+      <c r="N125" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7735,7 +7794,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1469.55</v>
+        <v>1472</v>
       </c>
       <c r="C3" t="n">
         <v>7</v>
@@ -8039,13 +8098,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>467.83</v>
+        <v>467.82</v>
       </c>
       <c r="C19" t="n">
         <v>46</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>129</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-16T16:22Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N125"/>
+  <dimension ref="A1:N126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7724,6 +7724,65 @@
         <v>0</v>
       </c>
       <c r="N125" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>8</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>2026/08/15 21:23:01</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>-32.841689, -70.936801</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>-32.84169, -70.93680</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>2026/08/15 23:58:15</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>-32.84158, -70.93677</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>-32.84158, -70.93677</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>02:35:14</t>
+        </is>
+      </c>
+      <c r="L126" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M126" t="n">
+        <v>0</v>
+      </c>
+      <c r="N126" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8117,13 +8176,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1207.82</v>
+        <v>1221.86</v>
       </c>
       <c r="C20" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>140</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-17T04:39Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N123"/>
+  <dimension ref="A1:N122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/08/16 20:13:38</t>
+          <t>2026/08/16 23:13:38</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>164:00:17</t>
+          <t>167:00:17</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026/08/16 20:24:44</t>
+          <t>2026/08/16 23:22:25</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>164:02:06</t>
+          <t>166:59:47</t>
         </is>
       </c>
       <c r="L11" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/16 20:42:52</t>
+          <t>2026/08/16 23:42:52</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>164:01:16</t>
+          <t>167:01:16</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/08/16 20:57:15</t>
+          <t>2026/08/16 23:57:15</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>164:01:06</t>
+          <t>167:01:06</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/08/16 20:57:37</t>
+          <t>2026/08/16 23:57:15</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>163:59:46</t>
+          <t>166:59:24</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>2026/08/16 21:02:05</t>
+          <t>2026/08/16 23:01:52</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6121,7 +6121,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>104:18:59</t>
+          <t>106:18:46</t>
         </is>
       </c>
       <c r="L98" t="n">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>2026/08/16 20:34:38</t>
+          <t>2026/08/16 23:34:40</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>100:03:19</t>
+          <t>103:03:21</t>
         </is>
       </c>
       <c r="L102" t="n">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>2026/08/16 20:13:47</t>
+          <t>2026/08/16 23:13:53</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>77:14:09</t>
+          <t>80:14:15</t>
         </is>
       </c>
       <c r="L111" t="n">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>2026/08/16 19:43:02</t>
+          <t>2026/08/16 23:43:02</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>74:23:32</t>
+          <t>78:23:32</t>
         </is>
       </c>
       <c r="L114" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/08/16 20:02:27</t>
+          <t>2026/08/16 22:02:27</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>45:34:53</t>
+          <t>47:34:53</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/08/16 20:55:26</t>
+          <t>2026/08/16 22:55:26</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>04:38:45</t>
+          <t>06:38:45</t>
         </is>
       </c>
       <c r="L119" t="n">
@@ -7376,11 +7376,11 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>SUZUKI CARRY SKDB-52</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -7389,41 +7389,41 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>2026/08/16 16:23:57</t>
+          <t>2026/08/16 16:31:04</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>-33.4518433, -70.6709383</t>
+          <t>-32.87922, -70.6087983</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>-33.45184, -70.67094</t>
+          <t>-32.87922, -70.60880</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/08/16 20:27:44</t>
+          <t>2026/08/16 22:31:04</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>-33.4517733, -70.671</t>
+          <t>-32.87922, -70.6087983</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>-33.45177, -70.67100</t>
+          <t>-32.87922, -70.60880</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>04:03:47</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L120" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="M120" t="n">
         <v>0</v>
@@ -7435,11 +7435,11 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -7448,37 +7448,37 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>2026/08/16 16:31:04</t>
+          <t>2026/08/16 16:36:02</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>-32.87922, -70.6087983</t>
+          <t>-32.7976316, -70.88709</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>-32.87922, -70.60880</t>
+          <t>-32.79763, -70.88709</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2026/08/16 20:31:04</t>
+          <t>2026/08/16 22:36:22</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>-32.87922, -70.6087983</t>
+          <t>-32.7976233, -70.8870599</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>-32.87922, -70.60880</t>
+          <t>-32.79762, -70.88706</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:20</t>
         </is>
       </c>
       <c r="L121" t="n">
@@ -7494,11 +7494,11 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -7507,37 +7507,37 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>2026/08/16 16:36:02</t>
+          <t>2026/08/16 17:20:29</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>-32.7976316, -70.88709</t>
+          <t>-33.476165, -70.698405</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>-32.79763, -70.88709</t>
+          <t>-33.47617, -70.69840</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>2026/08/16 20:36:22</t>
+          <t>2026/08/16 23:20:58</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>-32.7976233, -70.8870599</t>
+          <t>-33.476165, -70.698405</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>-32.79762, -70.88706</t>
+          <t>-33.47617, -70.69840</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>04:00:20</t>
+          <t>06:00:29</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -7547,65 +7547,6 @@
         <v>0</v>
       </c>
       <c r="N122" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
-        </is>
-      </c>
-      <c r="C123" t="n">
-        <v>3</v>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>Paradas</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>2026/08/16 17:20:29</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>-33.476165, -70.698405</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>-33.47617, -70.69840</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>2026/08/16 19:20:58</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>-33.476165, -70.698405</t>
-        </is>
-      </c>
-      <c r="J123" t="inlineStr">
-        <is>
-          <t>-33.47617, -70.69840</t>
-        </is>
-      </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>02:00:29</t>
-        </is>
-      </c>
-      <c r="L123" t="n">
-        <v>0</v>
-      </c>
-      <c r="M123" t="n">
-        <v>0</v>
-      </c>
-      <c r="N123" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7904,13 +7845,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>178.4</v>
+        <v>184.25</v>
       </c>
       <c r="C15" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
         <v>137</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-17T12:39Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -3069,11 +3069,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3087,52 +3087,52 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>-33.3688266, -70.6980799</t>
+          <t>-34.207225, -70.675975</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>-33.36883, -70.69808</t>
+          <t>-34.20723, -70.67597</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>2026/08/10 13:26:41</t>
+          <t>2026/08/10 12:38:07</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>-32.8831716, -70.6124633</t>
+          <t>-34.2042833, -70.6790466</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>-32.88317, -70.61246</t>
+          <t>-34.20428, -70.67905</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>00:56:01</t>
+          <t>00:07:27</t>
         </is>
       </c>
       <c r="L47" t="n">
-        <v>65.29000000000001</v>
+        <v>0.49</v>
       </c>
       <c r="M47" t="n">
-        <v>119</v>
+        <v>14</v>
       </c>
       <c r="N47" t="n">
-        <v>69</v>
+        <v>12</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3146,42 +3146,42 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>-34.207225, -70.675975</t>
+          <t>-33.3688266, -70.6980799</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>-34.20723, -70.67597</t>
+          <t>-33.36883, -70.69808</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2026/08/10 12:38:07</t>
+          <t>2026/08/10 13:26:41</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>-34.2042833, -70.6790466</t>
+          <t>-32.8831716, -70.6124633</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>-34.20428, -70.67905</t>
+          <t>-32.88317, -70.61246</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>00:07:27</t>
+          <t>00:56:01</t>
         </is>
       </c>
       <c r="L48" t="n">
-        <v>0.49</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="M48" t="n">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="N48" t="n">
-        <v>12</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-17T16:25Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N122"/>
+  <dimension ref="A1:N123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3069,11 +3069,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3087,52 +3087,52 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>-34.207225, -70.675975</t>
+          <t>-33.3688266, -70.6980799</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>-34.20723, -70.67597</t>
+          <t>-33.36883, -70.69808</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>2026/08/10 12:38:07</t>
+          <t>2026/08/10 13:26:41</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>-34.2042833, -70.6790466</t>
+          <t>-32.8831716, -70.6124633</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>-34.20428, -70.67905</t>
+          <t>-32.88317, -70.61246</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>00:07:27</t>
+          <t>00:56:01</t>
         </is>
       </c>
       <c r="L47" t="n">
-        <v>0.49</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="M47" t="n">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="N47" t="n">
-        <v>12</v>
+        <v>69</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3146,42 +3146,42 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>-33.3688266, -70.6980799</t>
+          <t>-34.207225, -70.675975</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>-33.36883, -70.69808</t>
+          <t>-34.20723, -70.67597</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2026/08/10 13:26:41</t>
+          <t>2026/08/10 12:38:07</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>-32.8831716, -70.6124633</t>
+          <t>-34.2042833, -70.6790466</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>-32.88317, -70.61246</t>
+          <t>-34.20428, -70.67905</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>00:56:01</t>
+          <t>00:07:27</t>
         </is>
       </c>
       <c r="L48" t="n">
-        <v>65.29000000000001</v>
+        <v>0.49</v>
       </c>
       <c r="M48" t="n">
-        <v>119</v>
+        <v>14</v>
       </c>
       <c r="N48" t="n">
-        <v>69</v>
+        <v>12</v>
       </c>
     </row>
     <row r="49">
@@ -7547,6 +7547,65 @@
         <v>0</v>
       </c>
       <c r="N122" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>5</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2026/08/16 23:38:27</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>-32.841659, -70.936845</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>-32.84166, -70.93685</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2026/08/16 23:55:20</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>-32.841627, -70.936888</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>-32.84163, -70.93689</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>00:16:53</t>
+        </is>
+      </c>
+      <c r="L123" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M123" t="n">
+        <v>0</v>
+      </c>
+      <c r="N123" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7940,13 +7999,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1281.5</v>
+        <v>1299.14</v>
       </c>
       <c r="C20" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>140</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-17T20:23Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -3069,11 +3069,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3087,52 +3087,52 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>-33.3688266, -70.6980799</t>
+          <t>-34.207225, -70.675975</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>-33.36883, -70.69808</t>
+          <t>-34.20723, -70.67597</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>2026/08/10 13:26:41</t>
+          <t>2026/08/10 12:38:07</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>-32.8831716, -70.6124633</t>
+          <t>-34.2042833, -70.6790466</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>-32.88317, -70.61246</t>
+          <t>-34.20428, -70.67905</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>00:56:01</t>
+          <t>00:07:27</t>
         </is>
       </c>
       <c r="L47" t="n">
-        <v>65.29000000000001</v>
+        <v>0.49</v>
       </c>
       <c r="M47" t="n">
-        <v>119</v>
+        <v>14</v>
       </c>
       <c r="N47" t="n">
-        <v>69</v>
+        <v>12</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3146,42 +3146,42 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>-34.207225, -70.675975</t>
+          <t>-33.3688266, -70.6980799</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>-34.20723, -70.67597</t>
+          <t>-33.36883, -70.69808</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2026/08/10 12:38:07</t>
+          <t>2026/08/10 13:26:41</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>-34.2042833, -70.6790466</t>
+          <t>-32.8831716, -70.6124633</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>-34.20428, -70.67905</t>
+          <t>-32.88317, -70.61246</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>00:07:27</t>
+          <t>00:56:01</t>
         </is>
       </c>
       <c r="L48" t="n">
-        <v>0.49</v>
+        <v>65.29000000000001</v>
       </c>
       <c r="M48" t="n">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="N48" t="n">
-        <v>12</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-18T04:33Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N118"/>
+  <dimension ref="A1:N119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/08/17 20:24:43</t>
+          <t>2026/08/17 23:24:37</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>164:01:51</t>
+          <t>167:01:45</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/08/17 20:43:01</t>
+          <t>2026/08/17 23:43:01</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>164:01:25</t>
+          <t>167:01:25</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/08/17 20:55:51</t>
+          <t>2026/08/17 23:55:51</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>163:59:42</t>
+          <t>166:59:42</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/08/17 20:58:07</t>
+          <t>2026/08/17 23:57:15</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>163:58:57</t>
+          <t>166:58:05</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>2026/08/17 20:46:38</t>
+          <t>2026/08/17 23:46:16</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6062,7 +6062,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>101:47:00</t>
+          <t>104:46:38</t>
         </is>
       </c>
       <c r="L97" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>2026/08/17 20:34:25</t>
+          <t>2026/08/17 23:34:24</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>18:00:09</t>
+          <t>21:00:08</t>
         </is>
       </c>
       <c r="L105" t="n">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>2026/08/17 20:27:12</t>
+          <t>2026/08/17 22:27:12</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="L106" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>2026/08/17 20:19:00</t>
+          <t>2026/08/17 22:19:00</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -6829,7 +6829,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L110" t="n">
@@ -6873,7 +6873,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>2026/08/17 20:26:34</t>
+          <t>2026/08/17 22:26:34</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>04:01:22</t>
+          <t>06:01:22</t>
         </is>
       </c>
       <c r="L111" t="n">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026/08/17 19:27:27</t>
+          <t>2026/08/17 23:27:27</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7006,7 +7006,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>02:03:19</t>
+          <t>06:03:19</t>
         </is>
       </c>
       <c r="L113" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/08/17 20:50:51</t>
+          <t>2026/08/17 22:50:51</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>02:09:59</t>
+          <t>04:09:59</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026/08/17 21:03:58</t>
+          <t>2026/08/17 23:03:58</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -7311,6 +7311,65 @@
         <v>0</v>
       </c>
       <c r="N118" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>8</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2026/08/17 21:36:05</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>-33.4372716, -70.6287483</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>-33.43727, -70.62875</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>2026/08/17 23:36:05</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>-33.4372716, -70.6287483</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>-33.43727, -70.62875</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L119" t="n">
+        <v>0</v>
+      </c>
+      <c r="M119" t="n">
+        <v>0</v>
+      </c>
+      <c r="N119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7609,13 +7668,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>241.12</v>
+        <v>246.78</v>
       </c>
       <c r="C15" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>132</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-18T20:20Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N119"/>
+  <dimension ref="A1:N120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7317,11 +7317,11 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -7330,46 +7330,105 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2026/08/17 21:36:05</t>
+          <t>2026/08/17 21:02:17</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>-33.4372716, -70.6287483</t>
+          <t>-34.179645, -70.707433</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>-33.43727, -70.62875</t>
+          <t>-34.17965, -70.70743</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/08/17 23:36:05</t>
+          <t>2026/08/17 23:57:04</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>-33.4372716, -70.6287483</t>
+          <t>-34.179679, -70.707259</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>-33.43727, -70.62875</t>
+          <t>-34.17968, -70.70726</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>02:54:47</t>
         </is>
       </c>
       <c r="L119" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="M119" t="n">
         <v>0</v>
       </c>
       <c r="N119" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>8</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2026/08/17 21:36:05</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>-33.4372716, -70.6287483</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>-33.43727, -70.62875</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>2026/08/17 23:36:05</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>-33.4372716, -70.6287483</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>-33.43727, -70.62875</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120" t="n">
+        <v>0</v>
+      </c>
+      <c r="N120" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7763,13 +7822,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1180.14</v>
+        <v>1180.47</v>
       </c>
       <c r="C20" t="n">
         <v>70</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-19T04:34Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N119"/>
+  <dimension ref="A1:N123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/08/18 20:23:01</t>
+          <t>2026/08/18 23:22:34</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>164:00:09</t>
+          <t>166:59:42</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/18 20:43:01</t>
+          <t>2026/08/18 23:43:01</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>164:01:00</t>
+          <t>167:01:00</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/08/18 20:55:51</t>
+          <t>2026/08/18 23:55:51</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>163:59:48</t>
+          <t>166:59:48</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026/08/18 20:57:38</t>
+          <t>2026/08/18 23:57:22</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>163:59:59</t>
+          <t>166:59:43</t>
         </is>
       </c>
       <c r="L20" t="n">
@@ -5811,26 +5811,26 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>2026/08/18 20:46:30</t>
+          <t>2026/08/18 23:20:54</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>-33.359954, -70.807205</t>
+          <t>-33.36002, -70.807226</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>-33.35995, -70.80720</t>
+          <t>-33.36002, -70.80723</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>125:46:52</t>
+          <t>128:21:16</t>
         </is>
       </c>
       <c r="L93" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="M93" t="n">
         <v>0</v>
@@ -6460,7 +6460,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>2026/08/18 20:34:52</t>
+          <t>2026/08/18 23:34:37</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>42:00:36</t>
+          <t>45:00:21</t>
         </is>
       </c>
       <c r="L104" t="n">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026/08/18 20:34:58</t>
+          <t>2026/08/18 22:34:58</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>12:00:00</t>
         </is>
       </c>
       <c r="L115" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/08/18 19:55:09</t>
+          <t>2026/08/18 23:55:09</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026/08/18 20:02:49</t>
+          <t>2026/08/18 22:02:49</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>02:01:51</t>
+          <t>04:01:51</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -7345,32 +7345,268 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/08/18 19:25:50</t>
+          <t>2026/08/18 19:23:58</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>-33.4761899, -70.6984266</t>
+          <t>-33.476855, -70.6988616</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>-33.47619, -70.69843</t>
+          <t>-33.47686, -70.69886</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>00:46:01</t>
+          <t>00:44:09</t>
         </is>
       </c>
       <c r="L119" t="n">
-        <v>11.12</v>
+        <v>11.04</v>
       </c>
       <c r="M119" t="n">
         <v>51</v>
       </c>
       <c r="N119" t="n">
         <v>22</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>OPEL COMBO</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>5</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2026/08/18 19:22:33</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>-34.1798066, -70.70728</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>-34.17981, -70.70728</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>2026/08/18 23:26:26</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>-34.1796933, -70.7072383</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>-34.17969, -70.70724</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>04:03:53</t>
+        </is>
+      </c>
+      <c r="L120" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M120" t="n">
+        <v>0</v>
+      </c>
+      <c r="N120" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>5</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2026/08/18 19:23:50</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>-33.43624, -70.6295133</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>-33.43624, -70.62951</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>2026/08/18 23:23:50</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>-33.43624, -70.6295133</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>-33.43624, -70.62951</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>04:00:00</t>
+        </is>
+      </c>
+      <c r="L121" t="n">
+        <v>0</v>
+      </c>
+      <c r="M121" t="n">
+        <v>0</v>
+      </c>
+      <c r="N121" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>13</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2026/08/18 19:25:13</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>-33.4761899, -70.6984266</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>-33.47619, -70.69843</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2026/08/18 23:25:50</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>-33.4761899, -70.6984266</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>-33.47619, -70.69843</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>04:00:37</t>
+        </is>
+      </c>
+      <c r="L122" t="n">
+        <v>0</v>
+      </c>
+      <c r="M122" t="n">
+        <v>0</v>
+      </c>
+      <c r="N122" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCS-53</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>10</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2026/08/18 20:04:32</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>-34.1678533, -70.7329733</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>-34.16785, -70.73297</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>2026/08/18 22:04:32</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>-34.1678533, -70.7329733</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>-34.16785, -70.73297</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L123" t="n">
+        <v>0</v>
+      </c>
+      <c r="M123" t="n">
+        <v>0</v>
+      </c>
+      <c r="N123" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -7440,7 +7676,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>932.9</v>
+        <v>933.04</v>
       </c>
       <c r="C3" t="n">
         <v>9</v>
@@ -7465,7 +7701,7 @@
         <v>51</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>133</v>
@@ -7649,13 +7885,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1146.51</v>
+        <v>1146.43</v>
       </c>
       <c r="C14" t="n">
         <v>44</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>127</v>
@@ -7668,13 +7904,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>315.02</v>
+        <v>315.01</v>
       </c>
       <c r="C15" t="n">
         <v>31</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>156</v>
@@ -7687,13 +7923,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>644.1799999999999</v>
+        <v>644.0599999999999</v>
       </c>
       <c r="C16" t="n">
         <v>28</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
         <v>142</v>
@@ -7725,7 +7961,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-19T16:29Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N123"/>
+  <dimension ref="A1:N124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7606,6 +7606,65 @@
         <v>0</v>
       </c>
       <c r="N123" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>13</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2026/08/18 20:28:39</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>-34.179779, -70.707289</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>-34.17978, -70.70729</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2026/08/18 23:59:09</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>-34.17971, -70.707255</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>-34.17971, -70.70726</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>03:30:30</t>
+        </is>
+      </c>
+      <c r="L124" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M124" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7999,13 +8058,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1090.42</v>
+        <v>1096.41</v>
       </c>
       <c r="C20" t="n">
         <v>74</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-20T04:35Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N111"/>
+  <dimension ref="A1:N116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/08/19 20:24:11</t>
+          <t>2026/08/19 23:22:33</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>164:00:49</t>
+          <t>166:59:11</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/08/19 20:43:28</t>
+          <t>2026/08/19 23:43:28</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>164:01:27</t>
+          <t>167:01:27</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/08/19 20:57:28</t>
+          <t>2026/08/19 23:57:28</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>164:01:25</t>
+          <t>167:01:25</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/19 20:47:09</t>
+          <t>2026/08/19 23:46:59</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>163:48:00</t>
+          <t>166:47:50</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>2026/08/19 20:21:04</t>
+          <t>2026/08/19 23:20:52</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3820,7 +3820,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>149:21:26</t>
+          <t>152:21:14</t>
         </is>
       </c>
       <c r="L59" t="n">
@@ -5575,7 +5575,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>2026/08/19 21:02:07</t>
+          <t>2026/08/19 23:01:45</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>54:50:39</t>
+          <t>56:50:17</t>
         </is>
       </c>
       <c r="L89" t="n">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>2026/08/19 20:34:58</t>
+          <t>2026/08/19 22:34:58</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>34:00:00</t>
+          <t>36:00:00</t>
         </is>
       </c>
       <c r="L104" t="n">
@@ -6755,26 +6755,26 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>2026/08/19 20:45:51</t>
+          <t>2026/08/19 20:43:33</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>-32.7976233, -70.8870833</t>
+          <t>-32.7977, -70.8874083</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>-32.79762, -70.88708</t>
+          <t>-32.79770, -70.88741</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>03:56:53</t>
+          <t>03:54:35</t>
         </is>
       </c>
       <c r="L109" t="n">
-        <v>206.15</v>
+        <v>206.12</v>
       </c>
       <c r="M109" t="n">
         <v>133</v>
@@ -6814,26 +6814,26 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>2026/08/19 19:30:06</t>
+          <t>2026/08/19 19:28:36</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>-34.16784, -70.7330183</t>
+          <t>-34.1678933, -70.7330466</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>-34.16784, -70.73302</t>
+          <t>-34.16789, -70.73305</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>01:09:23</t>
+          <t>01:07:53</t>
         </is>
       </c>
       <c r="L110" t="n">
-        <v>4.09</v>
+        <v>4.08</v>
       </c>
       <c r="M110" t="n">
         <v>70</v>
@@ -6845,11 +6845,11 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -6858,7 +6858,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2026/08/19 19:34:09</t>
+          <t>2026/08/19 19:29:51</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -6873,31 +6873,326 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>2026/08/19 21:07:05</t>
+          <t>2026/08/19 23:30:06</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>-34.1678566, -70.732985</t>
+          <t>-34.16784, -70.7330183</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>-34.16786, -70.73298</t>
+          <t>-34.16784, -70.73302</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>01:32:56</t>
+          <t>04:00:15</t>
         </is>
       </c>
       <c r="L111" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="M111" t="n">
         <v>0</v>
       </c>
       <c r="N111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>OPEL COMBO</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>8</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>2026/08/19 19:34:09</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>-34.16784, -70.7330183</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>-34.16784, -70.73302</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>2026/08/19 23:07:17</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>-34.1678566, -70.732985</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>-34.16786, -70.73298</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>03:33:08</t>
+        </is>
+      </c>
+      <c r="L112" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M112" t="n">
+        <v>0</v>
+      </c>
+      <c r="N112" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>12</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>2026/08/19 19:51:49</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>-33.4761833, -70.6984316</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>-33.47618, -70.69843</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>2026/08/19 23:52:11</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>-33.4761833, -70.6984316</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>-33.47618, -70.69843</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>04:00:22</t>
+        </is>
+      </c>
+      <c r="L113" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" t="n">
+        <v>0</v>
+      </c>
+      <c r="N113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TGPS-77</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>13</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>2026/08/19 20:44:48</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>-32.7976233, -70.8870833</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>-32.79762, -70.88708</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>2026/08/19 22:45:51</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>-32.7976233, -70.8870833</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>-32.79762, -70.88708</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>02:01:03</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>2</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2026/08/19 21:03:13</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>-32.8792033, -70.6087666</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>-32.87920, -70.60877</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>2026/08/19 23:03:13</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>-32.8792033, -70.6087666</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>-32.87920, -70.60877</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L115" t="n">
+        <v>0</v>
+      </c>
+      <c r="M115" t="n">
+        <v>0</v>
+      </c>
+      <c r="N115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>7</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>2026/08/19 21:49:37</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>-33.43791, -70.6292216</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>-33.43791, -70.62922</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>2026/08/19 23:50:15</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>-33.43791, -70.6292216</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>-33.43791, -70.62922</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>02:00:38</t>
+        </is>
+      </c>
+      <c r="L116" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" t="n">
+        <v>0</v>
+      </c>
+      <c r="N116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6949,13 +7244,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1623.53</v>
+        <v>1623.5</v>
       </c>
       <c r="C2" t="n">
         <v>51</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>157</v>
@@ -6968,10 +7263,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1009.66</v>
+        <v>1009.8</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -6987,13 +7282,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1174.14</v>
+        <v>1174.13</v>
       </c>
       <c r="C4" t="n">
         <v>54</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>131</v>
@@ -7177,13 +7472,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1379.9</v>
+        <v>1379.88</v>
       </c>
       <c r="C14" t="n">
         <v>54</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>127</v>
@@ -7196,13 +7491,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>327.52</v>
+        <v>335.36</v>
       </c>
       <c r="C15" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>156</v>
@@ -7272,13 +7567,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>709.92</v>
+        <v>709.91</v>
       </c>
       <c r="C19" t="n">
         <v>43</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>137</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-20T16:32Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N116"/>
+  <dimension ref="A1:N117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6904,11 +6904,11 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -6917,41 +6917,41 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>2026/08/19 19:34:09</t>
+          <t>2026/08/19 19:31:51</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>-34.16784, -70.7330183</t>
+          <t>-34.167893, -70.733015</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>-34.16784, -70.73302</t>
+          <t>-34.16789, -70.73301</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>2026/08/19 23:07:17</t>
+          <t>2026/08/19 23:28:58</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>-34.1678566, -70.732985</t>
+          <t>-34.16775, -70.733029</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>-34.16786, -70.73298</t>
+          <t>-34.16775, -70.73303</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>03:33:08</t>
+          <t>03:57:07</t>
         </is>
       </c>
       <c r="L112" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="M112" t="n">
         <v>0</v>
@@ -6963,11 +6963,11 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -6976,41 +6976,41 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2026/08/19 19:51:49</t>
+          <t>2026/08/19 19:34:09</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>-33.4761833, -70.6984316</t>
+          <t>-34.16784, -70.7330183</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>-33.47618, -70.69843</t>
+          <t>-34.16784, -70.73302</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026/08/19 23:52:11</t>
+          <t>2026/08/19 23:07:17</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>-33.4761833, -70.6984316</t>
+          <t>-34.1678566, -70.732985</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>-33.47618, -70.69843</t>
+          <t>-34.16786, -70.73298</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>04:00:22</t>
+          <t>03:33:08</t>
         </is>
       </c>
       <c r="L113" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="M113" t="n">
         <v>0</v>
@@ -7022,11 +7022,11 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -7035,37 +7035,37 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2026/08/19 20:44:48</t>
+          <t>2026/08/19 19:51:49</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>-32.7976233, -70.8870833</t>
+          <t>-33.4761833, -70.6984316</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>-32.79762, -70.88708</t>
+          <t>-33.47618, -70.69843</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>2026/08/19 22:45:51</t>
+          <t>2026/08/19 23:52:11</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>-32.7976233, -70.8870833</t>
+          <t>-33.4761833, -70.6984316</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>-32.79762, -70.88708</t>
+          <t>-33.47618, -70.69843</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>02:01:03</t>
+          <t>04:00:22</t>
         </is>
       </c>
       <c r="L114" t="n">
@@ -7081,11 +7081,11 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -7094,37 +7094,37 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2026/08/19 21:03:13</t>
+          <t>2026/08/19 20:44:48</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>-32.8792033, -70.6087666</t>
+          <t>-32.7976233, -70.8870833</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>-32.87920, -70.60877</t>
+          <t>-32.79762, -70.88708</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026/08/19 23:03:13</t>
+          <t>2026/08/19 22:45:51</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>-32.8792033, -70.6087666</t>
+          <t>-32.7976233, -70.8870833</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>-32.87920, -70.60877</t>
+          <t>-32.79762, -70.88708</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>02:01:03</t>
         </is>
       </c>
       <c r="L115" t="n">
@@ -7140,11 +7140,11 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>SUZUKI CARRY SKDB-52</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -7153,37 +7153,37 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2026/08/19 21:49:37</t>
+          <t>2026/08/19 21:03:13</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>-33.43791, -70.6292216</t>
+          <t>-32.8792033, -70.6087666</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>-33.43791, -70.62922</t>
+          <t>-32.87920, -70.60877</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>2026/08/19 23:50:15</t>
+          <t>2026/08/19 23:03:13</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>-33.43791, -70.6292216</t>
+          <t>-32.8792033, -70.6087666</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>-33.43791, -70.62922</t>
+          <t>-32.87920, -70.60877</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>02:00:38</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="L116" t="n">
@@ -7193,6 +7193,65 @@
         <v>0</v>
       </c>
       <c r="N116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>7</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>2026/08/19 21:49:37</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>-33.43791, -70.6292216</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>-33.43791, -70.62922</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>2026/08/19 23:50:15</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>-33.43791, -70.6292216</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>-33.43791, -70.62922</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>02:00:38</t>
+        </is>
+      </c>
+      <c r="L117" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" t="n">
+        <v>0</v>
+      </c>
+      <c r="N117" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7586,13 +7645,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>897.09</v>
+        <v>901.01</v>
       </c>
       <c r="C20" t="n">
         <v>73</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-20T20:25Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -6932,22 +6932,22 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>2026/08/19 23:28:58</t>
+          <t>2026/08/19 23:59:22</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>-34.16775, -70.733029</t>
+          <t>-34.167769, -70.733032</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>-34.16775, -70.73303</t>
+          <t>-34.16777, -70.73303</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>03:57:07</t>
+          <t>04:27:31</t>
         </is>
       </c>
       <c r="L112" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-21T04:35Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N133"/>
+  <dimension ref="A1:N138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/08/20 20:24:18</t>
+          <t>2026/08/20 23:23:46</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>164:00:55</t>
+          <t>167:00:23</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/08/20 20:43:28</t>
+          <t>2026/08/20 23:43:28</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>164:01:01</t>
+          <t>167:01:01</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/08/20 20:20:47</t>
+          <t>2026/08/20 23:21:03</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>163:24:19</t>
+          <t>166:24:35</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/08/20 20:57:28</t>
+          <t>2026/08/20 23:57:28</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>164:00:38</t>
+          <t>167:00:38</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/08/20 20:47:07</t>
+          <t>2026/08/20 23:47:08</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>163:49:26</t>
+          <t>166:49:27</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>2026/08/20 20:31:20</t>
+          <t>2026/08/20 23:31:37</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5295,7 +5295,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>113:59:43</t>
+          <t>117:00:00</t>
         </is>
       </c>
       <c r="L84" t="n">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>2026/08/20 21:01:38</t>
+          <t>2026/08/20 23:01:33</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -5472,7 +5472,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>78:50:10</t>
+          <t>80:50:05</t>
         </is>
       </c>
       <c r="L87" t="n">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>2026/08/20 20:34:58</t>
+          <t>2026/08/20 22:34:58</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>58:00:00</t>
+          <t>60:00:00</t>
         </is>
       </c>
       <c r="L101" t="n">
@@ -6904,11 +6904,11 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>SLP20250425120-AC01</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -6917,47 +6917,47 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>2026/08/20 11:20:09</t>
+          <t>2026/08/20 11:38:36</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>-33.3672483, -70.695835</t>
+          <t>-33.360431, -70.806826</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>-33.36725, -70.69584</t>
+          <t>-33.36043, -70.80683</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>2026/08/20 19:20:09</t>
+          <t>2026/08/20 11:50:38</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>-33.3672483, -70.695835</t>
+          <t>-33.360653, -70.806874</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>-33.36725, -70.69584</t>
+          <t>-33.36065, -70.80687</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>08:00:00</t>
+          <t>00:12:02</t>
         </is>
       </c>
       <c r="L112" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="M112" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N112" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="113">
@@ -6967,56 +6967,56 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2026/08/20 11:38:36</t>
+          <t>2026/08/20 11:51:38</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>-33.360431, -70.806826</t>
+          <t>-33.360659, -70.806827</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>-33.36043, -70.80683</t>
+          <t>-33.36066, -70.80683</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>2026/08/20 11:50:38</t>
+          <t>2026/08/20 12:02:06</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>-33.360653, -70.806874</t>
+          <t>-33.360694, -70.806797</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>-33.36065, -70.80687</t>
+          <t>-33.36069, -70.80680</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>00:12:02</t>
+          <t>00:10:28</t>
         </is>
       </c>
       <c r="L113" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="M113" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N113" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="114">
@@ -7026,56 +7026,56 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2026/08/20 11:51:38</t>
+          <t>2026/08/20 12:02:40</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>-33.360659, -70.806827</t>
+          <t>-33.360688, -70.806794</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>-33.36066, -70.80683</t>
+          <t>-33.36069, -70.80679</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>2026/08/20 12:02:06</t>
+          <t>2026/08/20 12:15:02</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>-33.360694, -70.806797</t>
+          <t>-33.360597, -70.80678</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>-33.36069, -70.80680</t>
+          <t>-33.36060, -70.80678</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>00:10:28</t>
+          <t>00:12:22</t>
         </is>
       </c>
       <c r="L114" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="M114" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N114" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="115">
@@ -7085,53 +7085,53 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2026/08/20 12:02:40</t>
+          <t>2026/08/20 12:15:44</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>-33.360688, -70.806794</t>
+          <t>-33.3606, -70.806775</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>-33.36069, -70.80679</t>
+          <t>-33.36060, -70.80678</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>2026/08/20 12:15:02</t>
+          <t>2026/08/20 12:45:32</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>-33.360597, -70.80678</t>
+          <t>-33.361012, -70.806724</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>-33.36060, -70.80678</t>
+          <t>-33.36101, -70.80672</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>00:12:22</t>
+          <t>00:29:48</t>
         </is>
       </c>
       <c r="L115" t="n">
-        <v>0.02</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M115" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N115" t="n">
         <v>4</v>
@@ -7144,56 +7144,56 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2026/08/20 12:15:44</t>
+          <t>2026/08/20 12:45:47</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>-33.3606, -70.806775</t>
+          <t>-33.361103, -70.806688</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>-33.36060, -70.80678</t>
+          <t>-33.36110, -70.80669</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>2026/08/20 12:45:32</t>
+          <t>2026/08/20 12:56:06</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>-33.361012, -70.806724</t>
+          <t>-33.3613, -70.806624</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>-33.36101, -70.80672</t>
+          <t>-33.36130, -70.80662</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>00:29:48</t>
+          <t>00:10:19</t>
         </is>
       </c>
       <c r="L116" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="M116" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N116" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="117">
@@ -7203,7 +7203,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -7212,41 +7212,41 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2026/08/20 12:45:47</t>
+          <t>2026/08/20 12:56:47</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>-33.361103, -70.806688</t>
+          <t>-33.361299, -70.80662</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>-33.36110, -70.80669</t>
+          <t>-33.36130, -70.80662</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/08/20 12:56:06</t>
+          <t>2026/08/20 13:03:06</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>-33.3613, -70.806624</t>
+          <t>-33.361269, -70.806681</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>-33.36130, -70.80662</t>
+          <t>-33.36127, -70.80668</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>00:10:19</t>
+          <t>00:06:19</t>
         </is>
       </c>
       <c r="L117" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="M117" t="n">
         <v>3</v>
@@ -7262,56 +7262,56 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2026/08/20 12:56:47</t>
+          <t>2026/08/20 13:03:47</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>-33.361299, -70.80662</t>
+          <t>-33.361267, -70.806681</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>-33.36130, -70.80662</t>
+          <t>-33.36127, -70.80668</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2026/08/20 13:03:06</t>
+          <t>2026/08/20 13:14:57</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>-33.361269, -70.806681</t>
+          <t>-33.361644, -70.806868</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>-33.36127, -70.80668</t>
+          <t>-33.36164, -70.80687</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>00:06:19</t>
+          <t>00:11:10</t>
         </is>
       </c>
       <c r="L118" t="n">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="M118" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119">
@@ -7321,7 +7321,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -7330,47 +7330,47 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2026/08/20 13:03:47</t>
+          <t>2026/08/20 13:15:48</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>-33.361267, -70.806681</t>
+          <t>-33.361646, -70.806858</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>-33.36127, -70.80668</t>
+          <t>-33.36165, -70.80686</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>2026/08/20 13:14:57</t>
+          <t>2026/08/20 13:32:31</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>-33.361644, -70.806868</t>
+          <t>-33.361957, -70.807051</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>-33.36164, -70.80687</t>
+          <t>-33.36196, -70.80705</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>00:11:10</t>
+          <t>00:16:43</t>
         </is>
       </c>
       <c r="L119" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="M119" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N119" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="120">
@@ -7380,7 +7380,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -7389,47 +7389,47 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>2026/08/20 13:15:48</t>
+          <t>2026/08/20 13:32:48</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>-33.361646, -70.806858</t>
+          <t>-33.361971, -70.807041</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>-33.36165, -70.80686</t>
+          <t>-33.36197, -70.80704</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>2026/08/20 13:32:31</t>
+          <t>2026/08/20 13:44:59</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>-33.361957, -70.807051</t>
+          <t>-33.36194, -70.807078</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>-33.36196, -70.80705</t>
+          <t>-33.36194, -70.80708</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>00:16:43</t>
+          <t>00:12:11</t>
         </is>
       </c>
       <c r="L120" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="M120" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N120" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="121">
@@ -7439,56 +7439,56 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>2026/08/20 13:32:48</t>
+          <t>2026/08/20 13:45:48</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>-33.361971, -70.807041</t>
+          <t>-33.36195, -70.807078</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>-33.36197, -70.80704</t>
+          <t>-33.36195, -70.80708</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>2026/08/20 13:44:59</t>
+          <t>2026/08/20 15:33:13</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>-33.36194, -70.807078</t>
+          <t>-33.361426, -70.807088</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>-33.36194, -70.80708</t>
+          <t>-33.36143, -70.80709</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>00:12:11</t>
+          <t>01:47:25</t>
         </is>
       </c>
       <c r="L121" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="M121" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N121" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122">
@@ -7498,56 +7498,56 @@
         </is>
       </c>
       <c r="C122" t="n">
+        <v>12</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2026/08/20 15:34:13</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>-33.361319, -70.807106</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>-33.36132, -70.80711</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>2026/08/20 16:28:15</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>-33.36221, -70.807806</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>-33.36221, -70.80781</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>00:54:02</t>
+        </is>
+      </c>
+      <c r="L122" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="M122" t="n">
         <v>11</v>
       </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>Paradas</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>2026/08/20 13:45:48</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>-33.36195, -70.807078</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>-33.36195, -70.80708</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>2026/08/20 15:33:13</t>
-        </is>
-      </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>-33.361426, -70.807088</t>
-        </is>
-      </c>
-      <c r="J122" t="inlineStr">
-        <is>
-          <t>-33.36143, -70.80709</t>
-        </is>
-      </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>01:47:25</t>
-        </is>
-      </c>
-      <c r="L122" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="M122" t="n">
-        <v>2</v>
-      </c>
       <c r="N122" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123">
@@ -7557,7 +7557,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -7566,44 +7566,44 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>2026/08/20 15:34:13</t>
+          <t>2026/08/20 16:29:13</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>-33.361319, -70.807106</t>
+          <t>-33.362205, -70.807787</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>-33.36132, -70.80711</t>
+          <t>-33.36221, -70.80779</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>2026/08/20 16:28:15</t>
+          <t>2026/08/20 16:45:11</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>-33.36221, -70.807806</t>
+          <t>-33.362156, -70.808241</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>-33.36221, -70.80781</t>
+          <t>-33.36216, -70.80824</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>00:54:02</t>
+          <t>00:15:58</t>
         </is>
       </c>
       <c r="L123" t="n">
-        <v>0.31</v>
+        <v>0.06</v>
       </c>
       <c r="M123" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="N123" t="n">
         <v>5</v>
@@ -7616,174 +7616,174 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>2026/08/20 16:29:13</t>
+          <t>2026/08/20 16:45:13</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>-33.362205, -70.807787</t>
+          <t>-33.362154, -70.80825</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>-33.36221, -70.80779</t>
+          <t>-33.36215, -70.80825</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/08/20 16:45:11</t>
+          <t>2026/08/20 16:52:41</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>-33.362156, -70.808241</t>
+          <t>-33.362117, -70.808239</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>-33.36216, -70.80824</t>
+          <t>-33.36212, -70.80824</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>00:15:58</t>
+          <t>00:07:28</t>
         </is>
       </c>
       <c r="L124" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="M124" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N124" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SLP20250425120-AC01</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2026/08/20 16:45:13</t>
+          <t>2026/08/20 16:50:56</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>-33.362154, -70.80825</t>
+          <t>-34.2050133, -70.677245</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>-33.36215, -70.80825</t>
+          <t>-34.20501, -70.67724</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>2026/08/20 16:52:41</t>
+          <t>2026/08/20 17:07:01</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>-33.362117, -70.808239</t>
+          <t>-34.2040833, -70.6789266</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>-33.36212, -70.80824</t>
+          <t>-34.20408, -70.67893</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>00:07:28</t>
+          <t>00:16:05</t>
         </is>
       </c>
       <c r="L125" t="n">
-        <v>0.01</v>
+        <v>0.21</v>
       </c>
       <c r="M125" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N125" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>SLP20250425120-AC01</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2026/08/20 16:50:56</t>
+          <t>2026/08/20 16:53:13</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>-34.2050133, -70.677245</t>
+          <t>-33.362113, -70.808243</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>-34.20501, -70.67724</t>
+          <t>-33.36211, -70.80824</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>2026/08/20 17:07:01</t>
+          <t>2026/08/20 16:59:48</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>-34.2040833, -70.6789266</t>
+          <t>-33.362089, -70.808303</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>-34.20408, -70.67893</t>
+          <t>-33.36209, -70.80830</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>00:16:05</t>
+          <t>00:06:35</t>
         </is>
       </c>
       <c r="L126" t="n">
-        <v>0.21</v>
+        <v>0.02</v>
       </c>
       <c r="M126" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N126" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127">
@@ -7793,66 +7793,66 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2026/08/20 16:53:13</t>
+          <t>2026/08/20 17:00:14</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>-33.362113, -70.808243</t>
+          <t>-33.362101, -70.808285</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>-33.36211, -70.80824</t>
+          <t>-33.36210, -70.80828</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>2026/08/20 16:59:48</t>
+          <t>2026/08/20 17:26:31</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>-33.362089, -70.808303</t>
+          <t>-33.362078, -70.808783</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>-33.36209, -70.80830</t>
+          <t>-33.36208, -70.80878</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>00:06:35</t>
+          <t>00:26:17</t>
         </is>
       </c>
       <c r="L127" t="n">
-        <v>0.02</v>
+        <v>0.11</v>
       </c>
       <c r="M127" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="N127" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>SLP20250425120-AC01</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -7861,106 +7861,106 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>2026/08/20 17:00:14</t>
+          <t>2026/08/20 17:07:10</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>-33.362101, -70.808285</t>
+          <t>-34.2041333, -70.679035</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>-33.36210, -70.80828</t>
+          <t>-34.20413, -70.67903</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026/08/20 17:26:31</t>
+          <t>2026/08/20 18:10:34</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>-33.362078, -70.808783</t>
+          <t>-34.19, -70.7092233</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>-33.36208, -70.80878</t>
+          <t>-34.19000, -70.70922</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>00:26:17</t>
+          <t>01:03:24</t>
         </is>
       </c>
       <c r="L128" t="n">
-        <v>0.11</v>
+        <v>3.54</v>
       </c>
       <c r="M128" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="N128" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>SLP20250425120-AC01</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2026/08/20 17:07:10</t>
+          <t>2026/08/20 17:27:14</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>-34.2041333, -70.679035</t>
+          <t>-33.362084, -70.808781</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>-34.20413, -70.67903</t>
+          <t>-33.36208, -70.80878</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>2026/08/20 18:10:34</t>
+          <t>2026/08/20 17:33:12</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>-34.19, -70.7092233</t>
+          <t>-33.362083, -70.808834</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>-34.19000, -70.70922</t>
+          <t>-33.36208, -70.80883</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>01:03:24</t>
+          <t>00:05:58</t>
         </is>
       </c>
       <c r="L129" t="n">
-        <v>3.54</v>
+        <v>0.01</v>
       </c>
       <c r="M129" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="N129" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130">
@@ -7970,56 +7970,56 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2026/08/20 17:27:14</t>
+          <t>2026/08/20 17:33:14</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>-33.362084, -70.808781</t>
+          <t>-33.362083, -70.808834</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>-33.36208, -70.80878</t>
+          <t>-33.36208, -70.80883</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>2026/08/20 17:33:12</t>
+          <t>2026/08/20 18:06:19</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>-33.362083, -70.808834</t>
+          <t>-33.360021, -70.806945</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>-33.36208, -70.80883</t>
+          <t>-33.36002, -70.80694</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>00:05:58</t>
+          <t>00:33:05</t>
         </is>
       </c>
       <c r="L130" t="n">
-        <v>0.01</v>
+        <v>0.43</v>
       </c>
       <c r="M130" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N130" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="131">
@@ -8029,115 +8029,115 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2026/08/20 17:33:14</t>
+          <t>2026/08/20 18:07:18</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>-33.362083, -70.808834</t>
+          <t>-33.359994, -70.807052</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>-33.36208, -70.80883</t>
+          <t>-33.35999, -70.80705</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/08/20 18:06:19</t>
+          <t>2026/08/20 23:11:39</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>-33.360021, -70.806945</t>
+          <t>-33.360003, -70.80705</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>-33.36002, -70.80694</t>
+          <t>-33.36000, -70.80705</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>00:33:05</t>
+          <t>05:04:21</t>
         </is>
       </c>
       <c r="L131" t="n">
-        <v>0.43</v>
+        <v>0</v>
       </c>
       <c r="M131" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N131" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SLP20250425120-AC01</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2026/08/20 18:07:18</t>
+          <t>2026/08/20 18:11:08</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>-33.359994, -70.807052</t>
+          <t>-34.1899749, -70.7092783</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>-33.35999, -70.80705</t>
+          <t>-34.18997, -70.70928</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/08/20 20:11:39</t>
+          <t>2026/08/20 19:24:55</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>-33.360003, -70.80705</t>
+          <t>-34.167685, -70.7344999</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>-33.36000, -70.80705</t>
+          <t>-34.16768, -70.73450</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>02:04:21</t>
+          <t>01:13:47</t>
         </is>
       </c>
       <c r="L132" t="n">
-        <v>0</v>
+        <v>3.95</v>
       </c>
       <c r="M132" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="N132" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="133">
@@ -8147,31 +8147,31 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>2026/08/20 18:11:08</t>
+          <t>2026/08/20 19:26:10</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>-34.1899749, -70.7092783</t>
+          <t>-34.167915, -70.7331133</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>-34.18997, -70.70928</t>
+          <t>-34.16792, -70.73311</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/08/20 19:27:58</t>
+          <t>2026/08/20 23:27:58</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8186,17 +8186,312 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>01:16:50</t>
+          <t>04:01:48</t>
         </is>
       </c>
       <c r="L133" t="n">
-        <v>4.08</v>
+        <v>0.01</v>
       </c>
       <c r="M133" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="N133" t="n">
-        <v>24</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>OPEL COMBO</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>5</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>2026/08/20 19:32:31</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>-34.167765, -70.7329916</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>-34.16777, -70.73299</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>2026/08/20 23:32:31</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>-34.167765, -70.7329916</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>-34.16777, -70.73299</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>04:00:00</t>
+        </is>
+      </c>
+      <c r="L134" t="n">
+        <v>0</v>
+      </c>
+      <c r="M134" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>10</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2026/08/20 20:06:16</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>-33.4763366, -70.6983866</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>-33.47634, -70.69839</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>2026/08/20 23:46:59</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>-33.4761733, -70.6984316</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69843</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>03:40:43</t>
+        </is>
+      </c>
+      <c r="L135" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M135" t="n">
+        <v>0</v>
+      </c>
+      <c r="N135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>11</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2026/08/20 20:11:57</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>-32.8792383, -70.608805</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>-32.87924, -70.60881</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>2026/08/20 22:11:57</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>-32.8792383, -70.608805</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>-32.87924, -70.60881</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L136" t="n">
+        <v>0</v>
+      </c>
+      <c r="M136" t="n">
+        <v>0</v>
+      </c>
+      <c r="N136" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TGPS-77</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>8</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2026/08/20 20:32:45</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>-32.797595, -70.8870549</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>-32.79760, -70.88705</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>2026/08/20 22:35:17</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>-32.797595, -70.8870549</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>-32.79760, -70.88705</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>02:02:32</t>
+        </is>
+      </c>
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="n">
+        <v>0</v>
+      </c>
+      <c r="N137" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>2</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2026/08/20 21:34:57</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>-33.4366483, -70.6295383</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>-33.43665, -70.62954</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>2026/08/20 23:34:57</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>-33.4366483, -70.6295383</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>-33.43665, -70.62954</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L138" t="n">
+        <v>0</v>
+      </c>
+      <c r="M138" t="n">
+        <v>0</v>
+      </c>
+      <c r="N138" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -8247,13 +8542,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1824.09</v>
+        <v>1824.06</v>
       </c>
       <c r="C2" t="n">
         <v>49</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>150</v>
@@ -8285,13 +8580,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>952.02</v>
+        <v>951.88</v>
       </c>
       <c r="C4" t="n">
         <v>63</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>131</v>
@@ -8481,7 +8776,7 @@
         <v>56</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>127</v>
@@ -8494,10 +8789,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>318.95</v>
+        <v>333.98</v>
       </c>
       <c r="C15" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -8519,7 +8814,7 @@
         <v>32</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
         <v>138</v>
@@ -8570,13 +8865,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1044.41</v>
+        <v>1044.36</v>
       </c>
       <c r="C19" t="n">
         <v>48</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>137</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-21T16:31Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N138"/>
+  <dimension ref="A1:N139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8202,11 +8202,11 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
@@ -8215,41 +8215,41 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2026/08/20 19:32:31</t>
+          <t>2026/08/20 19:31:55</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>-34.167765, -70.7329916</t>
+          <t>-34.167908, -70.733115</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>-34.16777, -70.73299</t>
+          <t>-34.16791, -70.73311</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/08/20 23:32:31</t>
+          <t>2026/08/20 23:59:57</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>-34.167765, -70.7329916</t>
+          <t>-34.167784, -70.73308</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>-34.16777, -70.73299</t>
+          <t>-34.16778, -70.73308</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>04:28:02</t>
         </is>
       </c>
       <c r="L134" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="M134" t="n">
         <v>0</v>
@@ -8261,11 +8261,11 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
@@ -8274,41 +8274,41 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>2026/08/20 20:06:16</t>
+          <t>2026/08/20 19:32:31</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>-33.4763366, -70.6983866</t>
+          <t>-34.167765, -70.7329916</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>-33.47634, -70.69839</t>
+          <t>-34.16777, -70.73299</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026/08/20 23:46:59</t>
+          <t>2026/08/20 23:32:31</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>-33.4761733, -70.6984316</t>
+          <t>-34.167765, -70.7329916</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>-33.47617, -70.69843</t>
+          <t>-34.16777, -70.73299</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>03:40:43</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L135" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="M135" t="n">
         <v>0</v>
@@ -8320,11 +8320,11 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
@@ -8333,41 +8333,41 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>2026/08/20 20:11:57</t>
+          <t>2026/08/20 20:06:16</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>-32.8792383, -70.608805</t>
+          <t>-33.4763366, -70.6983866</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>-32.87924, -70.60881</t>
+          <t>-33.47634, -70.69839</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/08/20 22:11:57</t>
+          <t>2026/08/20 23:46:59</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>-32.8792383, -70.608805</t>
+          <t>-33.4761733, -70.6984316</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>-32.87924, -70.60881</t>
+          <t>-33.47617, -70.69843</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>03:40:43</t>
         </is>
       </c>
       <c r="L136" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="M136" t="n">
         <v>0</v>
@@ -8379,11 +8379,11 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>SUZUKI CARRY SKDB-52</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
@@ -8392,37 +8392,37 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2026/08/20 20:32:45</t>
+          <t>2026/08/20 20:11:57</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>-32.797595, -70.8870549</t>
+          <t>-32.8792383, -70.608805</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>-32.79760, -70.88705</t>
+          <t>-32.87924, -70.60881</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>2026/08/20 22:35:17</t>
+          <t>2026/08/20 22:11:57</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>-32.797595, -70.8870549</t>
+          <t>-32.8792383, -70.608805</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>-32.79760, -70.88705</t>
+          <t>-32.87924, -70.60881</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>02:02:32</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="L137" t="n">
@@ -8438,11 +8438,11 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
@@ -8451,37 +8451,37 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2026/08/20 21:34:57</t>
+          <t>2026/08/20 20:32:45</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>-33.4366483, -70.6295383</t>
+          <t>-32.797595, -70.8870549</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>-33.43665, -70.62954</t>
+          <t>-32.79760, -70.88705</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/08/20 23:34:57</t>
+          <t>2026/08/20 22:35:17</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>-33.4366483, -70.6295383</t>
+          <t>-32.797595, -70.8870549</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>-33.43665, -70.62954</t>
+          <t>-32.79760, -70.88705</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>02:02:32</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -8491,6 +8491,65 @@
         <v>0</v>
       </c>
       <c r="N138" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>2</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>2026/08/20 21:34:57</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>-33.4366483, -70.6295383</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>-33.43665, -70.62954</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>2026/08/20 23:34:57</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>-33.4366483, -70.6295383</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>-33.43665, -70.62954</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L139" t="n">
+        <v>0</v>
+      </c>
+      <c r="M139" t="n">
+        <v>0</v>
+      </c>
+      <c r="N139" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8884,13 +8943,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>677.4299999999999</v>
+        <v>681.21</v>
       </c>
       <c r="C20" t="n">
         <v>74</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-22T04:30Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N135"/>
+  <dimension ref="A1:N137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/08/21 20:23:31</t>
+          <t>2026/08/21 23:22:41</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>164:00:53</t>
+          <t>167:00:03</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/08/21 20:42:03</t>
+          <t>2026/08/21 23:42:03</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>163:59:36</t>
+          <t>166:59:36</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/08/21 20:56:04</t>
+          <t>2026/08/21 23:56:04</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>163:59:14</t>
+          <t>166:59:14</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/08/21 20:57:21</t>
+          <t>2026/08/21 23:57:21</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>163:58:13</t>
+          <t>166:58:13</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>2026/08/21 20:11:38</t>
+          <t>2026/08/21 23:11:38</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5236,7 +5236,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>90:00:16</t>
+          <t>93:00:16</t>
         </is>
       </c>
       <c r="L83" t="n">
@@ -7876,7 +7876,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>2026/08/21 20:13:23</t>
+          <t>2026/08/21 23:13:04</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>26:06:05</t>
+          <t>29:05:46</t>
         </is>
       </c>
       <c r="L128" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/08/21 20:08:32</t>
+          <t>2026/08/21 22:08:32</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>04:05:40</t>
+          <t>06:05:40</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/08/21 20:01:51</t>
+          <t>2026/08/21 22:01:51</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>02:23:22</t>
+          <t>04:23:22</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>2026/08/21 19:46:21</t>
+          <t>2026/08/21 23:46:21</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L133" t="n">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/08/21 20:00:46</t>
+          <t>2026/08/21 22:00:46</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L134" t="n">
@@ -8289,7 +8289,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>2026/08/21 21:01:02</t>
+          <t>2026/08/21 23:01:02</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>00:39:30</t>
+          <t>02:39:30</t>
         </is>
       </c>
       <c r="L135" t="n">
@@ -8314,6 +8314,124 @@
         <v>0</v>
       </c>
       <c r="N135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>14</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2026/08/21 21:15:45</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>-33.4762983, -70.6983616</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>-33.47630, -70.69836</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>2026/08/21 21:31:02</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>-33.4745866, -70.6957833</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>-33.47459, -70.69578</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>00:15:17</t>
+        </is>
+      </c>
+      <c r="L136" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="M136" t="n">
+        <v>33</v>
+      </c>
+      <c r="N136" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>15</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2026/08/21 21:32:17</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.6984066</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69841</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>2026/08/21 23:34:10</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.6984066</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69841</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>02:01:53</t>
+        </is>
+      </c>
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="n">
+        <v>0</v>
+      </c>
+      <c r="N137" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8593,13 +8711,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1179.4</v>
+        <v>1190.46</v>
       </c>
       <c r="C14" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>132</v>
@@ -8631,10 +8749,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>493.21</v>
+        <v>496.54</v>
       </c>
       <c r="C16" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-23T04:34Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N143"/>
+  <dimension ref="A1:N145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/22 20:42:03</t>
+          <t>2026/08/22 23:42:03</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>163:59:11</t>
+          <t>166:59:11</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/08/22 20:56:04</t>
+          <t>2026/08/22 23:56:04</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>163:58:49</t>
+          <t>166:58:49</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/08/22 20:57:44</t>
+          <t>2026/08/22 23:57:20</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>164:00:06</t>
+          <t>166:59:42</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/08/22 20:08:32</t>
+          <t>2026/08/22 22:08:32</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>28:05:40</t>
+          <t>30:05:40</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>2026/08/22 20:00:46</t>
+          <t>2026/08/22 22:00:46</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>26:00:00</t>
+          <t>28:00:00</t>
         </is>
       </c>
       <c r="L132" t="n">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>2026/08/22 21:03:11</t>
+          <t>2026/08/22 23:03:26</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>07:03:54</t>
+          <t>09:04:09</t>
         </is>
       </c>
       <c r="L140" t="n">
@@ -8643,26 +8643,26 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>2026/08/22 20:50:20</t>
+          <t>2026/08/22 23:02:57</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>-33.0872833, -71.3623833</t>
+          <t>-33.0872033, -71.3622033</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>-33.08728, -71.36238</t>
+          <t>-33.08720, -71.36220</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>08:12:37</t>
         </is>
       </c>
       <c r="L141" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="M141" t="n">
         <v>0</v>
@@ -8702,7 +8702,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>2026/08/22 20:00:30</t>
+          <t>2026/08/22 22:00:30</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L142" t="n">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/08/22 20:50:59</t>
+          <t>2026/08/22 22:50:59</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>02:31:52</t>
+          <t>04:31:52</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -8786,6 +8786,124 @@
         <v>0</v>
       </c>
       <c r="N143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TGPS-77</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>7</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>2026/08/22 19:37:41</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>-32.7976233, -70.8871166</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>-32.79762, -70.88712</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>2026/08/22 23:37:41</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>-32.7976233, -70.8871166</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>-32.79762, -70.88712</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>04:00:00</t>
+        </is>
+      </c>
+      <c r="L144" t="n">
+        <v>0</v>
+      </c>
+      <c r="M144" t="n">
+        <v>0</v>
+      </c>
+      <c r="N144" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>7</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>2026/08/22 21:17:26</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>-33.4762866, -70.6982883</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>-33.47629, -70.69829</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>2026/08/22 23:19:32</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.698385</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>-33.47617, -70.69839</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>02:02:06</t>
+        </is>
+      </c>
+      <c r="L145" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M145" t="n">
+        <v>0</v>
+      </c>
+      <c r="N145" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8837,13 +8955,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2374.59</v>
+        <v>2374.55</v>
       </c>
       <c r="C2" t="n">
         <v>55</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>150</v>
@@ -8856,7 +8974,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>853.95</v>
+        <v>859.86</v>
       </c>
       <c r="C3" t="n">
         <v>10</v>
@@ -9065,13 +9183,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1194.62</v>
+        <v>1197.57</v>
       </c>
       <c r="C14" t="n">
         <v>63</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>132</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-24T04:41Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/08/23 20:40:38</t>
+          <t>2026/08/23 23:40:38</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>163:57:46</t>
+          <t>166:57:46</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/08/23 20:56:10</t>
+          <t>2026/08/23 23:56:10</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>163:58:55</t>
+          <t>166:58:55</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/08/23 20:08:09</t>
+          <t>2026/08/23 23:08:09</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>163:09:02</t>
+          <t>166:09:02</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -3392,7 +3392,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>2026/08/23 21:01:38</t>
+          <t>2026/08/23 23:01:21</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>150:50:10</t>
+          <t>152:49:53</t>
         </is>
       </c>
       <c r="L52" t="n">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>2026/08/23 20:08:32</t>
+          <t>2026/08/23 22:08:32</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>52:05:40</t>
+          <t>54:05:40</t>
         </is>
       </c>
       <c r="L136" t="n">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/08/23 20:12:40</t>
+          <t>2026/08/23 23:10:11</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>30:13:23</t>
+          <t>33:10:54</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>2026/08/23 19:11:41</t>
+          <t>2026/08/23 23:11:41</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>05:14:05</t>
+          <t>09:14:05</t>
         </is>
       </c>
       <c r="L144" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/08/23 19:59:00</t>
+          <t>2026/08/23 23:59:00</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="L145" t="n">
@@ -8910,11 +8910,11 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>MITSUBISHI L200 PHZF-89</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D146" t="inlineStr">
         <is>
@@ -8923,37 +8923,37 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>2026/08/23 17:30:36</t>
+          <t>2026/08/23 17:47:25</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>-32.7422066, -70.7271033</t>
+          <t>-33.4363983, -70.6291883</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>-32.74221, -70.72710</t>
+          <t>-33.43640, -70.62919</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>2026/08/23 19:31:01</t>
+          <t>2026/08/23 23:47:25</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>-32.7422066, -70.7271033</t>
+          <t>-33.4363983, -70.6291883</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>-32.74221, -70.72710</t>
+          <t>-33.43640, -70.62919</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>02:00:25</t>
+          <t>06:00:00</t>
         </is>
       </c>
       <c r="L146" t="n">
@@ -8969,11 +8969,11 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 PHZF-89</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D147" t="inlineStr">
         <is>
@@ -8982,37 +8982,37 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2026/08/23 17:47:25</t>
+          <t>2026/08/23 18:11:00</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>-33.4363983, -70.6291883</t>
+          <t>-32.7976066, -70.887115</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>-33.43640, -70.62919</t>
+          <t>-32.79761, -70.88711</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/08/23 19:47:25</t>
+          <t>2026/08/23 22:11:00</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>-33.4363983, -70.6291883</t>
+          <t>-32.7976066, -70.887115</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>-33.43640, -70.62919</t>
+          <t>-32.79761, -70.88711</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L147" t="n">
@@ -9028,7 +9028,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -9041,41 +9041,41 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2026/08/23 18:11:00</t>
+          <t>2026/08/23 18:24:21</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>-32.7976066, -70.887115</t>
+          <t>-33.0873033, -71.3623316</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>-32.79761, -70.88711</t>
+          <t>-33.08730, -71.36233</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2026/08/23 20:11:00</t>
+          <t>2026/08/23 23:14:27</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>-32.7976066, -70.887115</t>
+          <t>-33.0872449, -71.3622933</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>-32.79761, -70.88711</t>
+          <t>-33.08724, -71.36229</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:50:06</t>
         </is>
       </c>
       <c r="L148" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="M148" t="n">
         <v>0</v>
@@ -9087,11 +9087,11 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>OPEL COMBO</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D149" t="inlineStr">
         <is>
@@ -9100,37 +9100,37 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2026/08/23 18:24:21</t>
+          <t>2026/08/23 21:40:15</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>-33.0873033, -71.3623316</t>
+          <t>-32.7431983, -70.729625</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>-33.08730, -71.36233</t>
+          <t>-32.74320, -70.72962</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>2026/08/23 19:14:27</t>
+          <t>2026/08/23 23:43:28</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>-33.0872449, -71.3622933</t>
+          <t>-32.7431233, -70.7297133</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>-33.08724, -71.36229</t>
+          <t>-32.74312, -70.72971</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>00:50:06</t>
+          <t>02:03:13</t>
         </is>
       </c>
       <c r="L149" t="n">
@@ -9457,10 +9457,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>573.29</v>
+        <v>573.76</v>
       </c>
       <c r="C16" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-24T16:34Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N149"/>
+  <dimension ref="A1:N150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9140,6 +9140,65 @@
         <v>0</v>
       </c>
       <c r="N149" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>6</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>2026/08/23 21:45:31</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>-32.842015, -70.936779</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>-32.84202, -70.93678</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>2026/08/23 23:49:01</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>-32.841607, -70.936759</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>-32.84161, -70.93676</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>02:03:30</t>
+        </is>
+      </c>
+      <c r="L150" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M150" t="n">
+        <v>0</v>
+      </c>
+      <c r="N150" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9533,13 +9592,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>528.8</v>
+        <v>582.6900000000001</v>
       </c>
       <c r="C20" t="n">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>138</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-25T04:36Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N150"/>
+  <dimension ref="A1:N154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/08/24 21:01:21</t>
+          <t>2026/08/24 23:01:39</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>164:49:54</t>
+          <t>166:50:12</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/08/24 20:40:38</t>
+          <t>2026/08/24 23:40:38</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>163:57:37</t>
+          <t>166:57:37</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/24 20:56:10</t>
+          <t>2026/08/24 23:56:10</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>164:00:19</t>
+          <t>167:00:19</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/08/24 20:45:08</t>
+          <t>2026/08/24 23:44:41</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>163:47:30</t>
+          <t>166:47:03</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>2026/08/24 20:35:08</t>
+          <t>2026/08/24 23:35:07</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>54:35:51</t>
+          <t>57:35:50</t>
         </is>
       </c>
       <c r="L138" t="n">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>2026/08/24 20:22:20</t>
+          <t>2026/08/24 23:22:23</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -8776,7 +8776,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>03:03:36</t>
+          <t>06:03:39</t>
         </is>
       </c>
       <c r="L143" t="n">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>2026/08/24 20:39:34</t>
+          <t>2026/08/24 22:39:34</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -8894,7 +8894,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>02:01:02</t>
+          <t>04:01:02</t>
         </is>
       </c>
       <c r="L145" t="n">
@@ -9056,26 +9056,26 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2026/08/24 21:07:31</t>
+          <t>2026/08/24 22:44:13</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>-33.0872733, -71.3622799</t>
+          <t>-33.0871966, -71.3622199</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>-33.08727, -71.36228</t>
+          <t>-33.08720, -71.36222</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>02:00:11</t>
+          <t>03:36:53</t>
         </is>
       </c>
       <c r="L148" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="M148" t="n">
         <v>0</v>
@@ -9115,26 +9115,26 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>2026/08/24 19:48:08</t>
+          <t>2026/08/24 19:42:58</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>-32.7431166, -70.7297283</t>
+          <t>-32.741235, -70.7290683</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>-32.74312, -70.72973</t>
+          <t>-32.74124, -70.72907</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>00:29:23</t>
+          <t>00:24:13</t>
         </is>
       </c>
       <c r="L149" t="n">
-        <v>0.52</v>
+        <v>0.28</v>
       </c>
       <c r="M149" t="n">
         <v>13</v>
@@ -9174,32 +9174,268 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026/08/24 19:50:39</t>
+          <t>2026/08/24 19:50:14</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>-32.8427833, -70.604975</t>
+          <t>-32.8431183, -70.604415</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>-32.84278, -70.60497</t>
+          <t>-32.84312, -70.60442</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>00:10:27</t>
+          <t>00:10:02</t>
         </is>
       </c>
       <c r="L150" t="n">
-        <v>1.23</v>
+        <v>1.17</v>
       </c>
       <c r="M150" t="n">
         <v>36</v>
       </c>
       <c r="N150" t="n">
         <v>18</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>OPEL COMBO</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>16</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>2026/08/24 19:44:13</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>-32.7430733, -70.7296433</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>-32.74307, -70.72964</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>2026/08/24 23:48:08</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>-32.7431166, -70.7297283</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>-32.74312, -70.72973</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>04:03:55</t>
+        </is>
+      </c>
+      <c r="L151" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M151" t="n">
+        <v>0</v>
+      </c>
+      <c r="N151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>SUZUKI CARRY SKDB-52</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>16</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>2026/08/24 19:50:39</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>-32.8427833, -70.604975</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>-32.84278, -70.60497</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>2026/08/24 22:51:10</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>-32.8791616, -70.608775</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>-32.87916, -70.60877</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>03:00:31</t>
+        </is>
+      </c>
+      <c r="L152" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="M152" t="n">
+        <v>71</v>
+      </c>
+      <c r="N152" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TGPS-77</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>14</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>2026/08/24 20:09:09</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>-32.7976083, -70.88708</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>-32.79761, -70.88708</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>2026/08/24 22:19:20</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>-32.7976083, -70.88708</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>-32.79761, -70.88708</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>02:10:11</t>
+        </is>
+      </c>
+      <c r="L153" t="n">
+        <v>0</v>
+      </c>
+      <c r="M153" t="n">
+        <v>0</v>
+      </c>
+      <c r="N153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>4</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2026/08/24 21:24:15</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>-33.4369433, -70.6294266</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>-33.43694, -70.62943</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>2026/08/24 23:25:26</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>-33.4369433, -70.6294266</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>-33.43694, -70.62943</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>02:01:11</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -9250,13 +9486,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2524.95</v>
+        <v>2524.92</v>
       </c>
       <c r="C2" t="n">
         <v>63</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>150</v>
@@ -9497,13 +9733,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>298.7</v>
+        <v>303.87</v>
       </c>
       <c r="C15" t="n">
         <v>25</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>156</v>
@@ -9516,13 +9752,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>739.4400000000001</v>
+        <v>739.21</v>
       </c>
       <c r="C16" t="n">
         <v>60</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
         <v>135</v>
@@ -9573,10 +9809,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>968.67</v>
+        <v>977.7</v>
       </c>
       <c r="C19" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-26T04:37Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N153"/>
+  <dimension ref="A1:N155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/08/25 21:01:38</t>
+          <t>2026/08/25 23:01:42</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>164:59:27</t>
+          <t>166:59:31</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/08/25 20:41:10</t>
+          <t>2026/08/25 23:41:10</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>163:58:09</t>
+          <t>166:58:09</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/08/25 20:56:10</t>
+          <t>2026/08/25 23:56:10</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>164:00:19</t>
+          <t>167:00:19</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/25 20:45:06</t>
+          <t>2026/08/25 23:44:46</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>163:45:58</t>
+          <t>166:45:38</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -8230,7 +8230,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>2026/08/25 20:53:53</t>
+          <t>2026/08/25 23:53:30</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>78:54:36</t>
+          <t>81:54:13</t>
         </is>
       </c>
       <c r="L134" t="n">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>2026/08/25 21:04:52</t>
+          <t>2026/08/25 23:04:53</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>09:58:06</t>
+          <t>11:58:07</t>
         </is>
       </c>
       <c r="L147" t="n">
@@ -9056,7 +9056,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>2026/08/25 20:34:44</t>
+          <t>2026/08/25 22:34:44</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>03:06:48</t>
+          <t>05:06:48</t>
         </is>
       </c>
       <c r="L148" t="n">
@@ -9115,7 +9115,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>2026/08/25 20:02:38</t>
+          <t>2026/08/25 22:02:38</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9130,7 +9130,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L149" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>2026/08/25 20:10:59</t>
+          <t>2026/08/25 22:10:59</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L150" t="n">
@@ -9233,7 +9233,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2026/08/25 20:19:48</t>
+          <t>2026/08/25 23:19:48</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>02:03:12</t>
+          <t>05:03:12</t>
         </is>
       </c>
       <c r="L151" t="n">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>2026/08/25 20:20:52</t>
+          <t>2026/08/25 22:20:52</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -9307,7 +9307,7 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>02:00:20</t>
+          <t>04:00:20</t>
         </is>
       </c>
       <c r="L152" t="n">
@@ -9323,11 +9323,11 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>OPEL COMBO</t>
+          <t>MITSUBISHI L200 PHZF-89</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D153" t="inlineStr">
         <is>
@@ -9336,46 +9336,164 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2026/08/25 20:58:30</t>
+          <t>2026/08/25 19:45:49</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>-32.7432, -70.729635</t>
+          <t>-33.4363633, -70.6293016</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>-32.74320, -70.72964</t>
+          <t>-33.43636, -70.62930</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>2026/08/25 21:05:36</t>
+          <t>2026/08/25 23:45:49</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>-32.7431083, -70.7296783</t>
+          <t>-33.4363633, -70.6293016</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>-32.74311, -70.72968</t>
+          <t>-33.43636, -70.62930</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>00:07:06</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L153" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="M153" t="n">
         <v>0</v>
       </c>
       <c r="N153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>8</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2026/08/25 20:20:47</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>-33.4761983, -70.6984133</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>-33.47620, -70.69841</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>2026/08/25 22:21:10</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>-33.4761983, -70.6984133</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>-33.47620, -70.69841</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>02:00:23</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" t="n">
+        <v>0</v>
+      </c>
+      <c r="N154" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>OPEL COMBO</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>9</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2026/08/25 20:58:30</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>-32.7432, -70.729635</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>-32.74320, -70.72964</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>2026/08/25 23:05:36</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>-32.7431083, -70.7296783</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>-32.74311, -70.72968</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>02:07:06</t>
+        </is>
+      </c>
+      <c r="L155" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M155" t="n">
+        <v>0</v>
+      </c>
+      <c r="N155" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9655,13 +9773,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>862.41</v>
+        <v>862.39</v>
       </c>
       <c r="C14" t="n">
         <v>58</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>132</v>
@@ -9674,13 +9792,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>236.37</v>
+        <v>236.31</v>
       </c>
       <c r="C15" t="n">
         <v>23</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>125</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-27T18:50Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -2066,7 +2066,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>CHANGAN HUNTER TKCS-53</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -2084,48 +2084,48 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>-33.4763233, -70.698395</t>
+          <t>-34.2063083, -70.6737416</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>-33.47632, -70.69840</t>
+          <t>-34.20631, -70.67374</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026/08/20 09:58:02</t>
+          <t>2026/08/20 09:16:19</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>-33.3623583, -70.6701283</t>
+          <t>-34.2072049, -70.6775133</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>-33.36236, -70.67013</t>
+          <t>-34.20720, -70.67751</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>01:09:29</t>
+          <t>00:27:46</t>
         </is>
       </c>
       <c r="L30" t="n">
-        <v>20.47</v>
+        <v>1.07</v>
       </c>
       <c r="M30" t="n">
-        <v>84</v>
+        <v>13</v>
       </c>
       <c r="N30" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -2143,42 +2143,42 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>-34.2063083, -70.6737416</t>
+          <t>-33.4763233, -70.698395</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>-34.20631, -70.67374</t>
+          <t>-33.47632, -70.69840</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026/08/20 09:16:19</t>
+          <t>2026/08/20 09:58:02</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>-34.2072049, -70.6775133</t>
+          <t>-33.3623583, -70.6701283</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>-34.20720, -70.67751</t>
+          <t>-33.36236, -70.67013</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>00:27:46</t>
+          <t>01:09:29</t>
         </is>
       </c>
       <c r="L31" t="n">
-        <v>1.07</v>
+        <v>20.47</v>
       </c>
       <c r="M31" t="n">
-        <v>13</v>
+        <v>84</v>
       </c>
       <c r="N31" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-29T10:48Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/08/28 22:41:36</t>
+          <t>2026/08/28 23:41:36</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>165:59:33</t>
+          <t>166:59:33</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/28 21:56:11</t>
+          <t>2026/08/28 23:56:11</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>165:00:07</t>
+          <t>167:00:07</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/08/28 21:58:01</t>
+          <t>2026/08/28 23:57:33</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>165:00:23</t>
+          <t>166:59:55</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026/08/28 22:24:42</t>
+          <t>2026/08/28 23:22:38</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>164:02:21</t>
+          <t>165:00:17</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>2026/08/28 21:04:45</t>
+          <t>2026/08/28 23:04:45</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7242,7 +7242,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>36:00:00</t>
+          <t>38:00:00</t>
         </is>
       </c>
       <c r="L117" t="n">
@@ -10621,129 +10621,129 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCS-53</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2026/08/28 16:19:43</t>
+          <t>2026/08/28 16:26:31</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>-33.0873216, -71.3623166</t>
+          <t>-33.3620566, -70.6701166</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>-33.08732, -71.36232</t>
+          <t>-33.36206, -70.67012</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>2026/08/28 22:19:43</t>
+          <t>2026/08/28 20:38:31</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>-33.0873216, -71.3623166</t>
+          <t>-33.476265, -70.6983133</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>-33.08732, -71.36232</t>
+          <t>-33.47626, -70.69831</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>06:00:00</t>
+          <t>04:12:00</t>
         </is>
       </c>
       <c r="L175" t="n">
-        <v>0</v>
+        <v>18.06</v>
       </c>
       <c r="M175" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="N175" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MITSUBISHI L200 LVHX-40</t>
+          <t>SLP20250425120-AC01</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>2026/08/28 16:26:31</t>
+          <t>2026/08/28 16:27:33</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>-33.3620566, -70.6701166</t>
+          <t>-33.360797, -70.806852</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>-33.36206, -70.67012</t>
+          <t>-33.36080, -70.80685</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>2026/08/28 20:38:31</t>
+          <t>2026/08/28 16:51:51</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>-33.476265, -70.6983133</t>
+          <t>-33.360841, -70.80691</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>-33.47626, -70.69831</t>
+          <t>-33.36084, -70.80691</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>04:12:00</t>
+          <t>00:24:18</t>
         </is>
       </c>
       <c r="L176" t="n">
-        <v>18.06</v>
+        <v>0.03</v>
       </c>
       <c r="M176" t="n">
-        <v>107</v>
+        <v>3</v>
       </c>
       <c r="N176" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>SLP20250425120-AC01</t>
+          <t>SUZUKI CARRY SKDB-52</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D177" t="inlineStr">
         <is>
@@ -10752,57 +10752,57 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2026/08/28 16:27:33</t>
+          <t>2026/08/28 16:37:27</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>-33.360797, -70.806852</t>
+          <t>-32.8792166, -70.6087616</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>-33.36080, -70.80685</t>
+          <t>-32.87922, -70.60876</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>2026/08/28 16:51:51</t>
+          <t>2026/08/28 22:07:21</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>-33.360841, -70.80691</t>
+          <t>-32.8792133, -70.6087949</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>-33.36084, -70.80691</t>
+          <t>-32.87921, -70.60879</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>00:24:18</t>
+          <t>05:29:54</t>
         </is>
       </c>
       <c r="L177" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="M177" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N177" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>SUZUKI CARRY SKDB-52</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D178" t="inlineStr">
         <is>
@@ -10811,47 +10811,47 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>2026/08/28 16:37:27</t>
+          <t>2026/08/28 16:37:40</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>-32.8792166, -70.6087616</t>
+          <t>-33.361352, -70.806634</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>-32.87922, -70.60876</t>
+          <t>-33.36135, -70.80663</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>2026/08/28 22:07:21</t>
+          <t>2026/08/28 16:45:32</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>-32.8792133, -70.6087949</t>
+          <t>-33.361306, -70.806612</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>-32.87921, -70.60879</t>
+          <t>-33.36131, -70.80661</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>05:29:54</t>
+          <t>00:07:52</t>
         </is>
       </c>
       <c r="L178" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="M178" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N178" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="179">
@@ -10861,50 +10861,50 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>2026/08/28 16:37:40</t>
+          <t>2026/08/28 16:46:13</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>-33.361352, -70.806634</t>
+          <t>-33.361304, -70.806644</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>-33.36135, -70.80663</t>
+          <t>-33.36130, -70.80664</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>2026/08/28 16:45:32</t>
+          <t>2026/08/28 17:24:35</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>-33.361306, -70.806612</t>
+          <t>-33.360513, -70.8068</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>-33.36131, -70.80661</t>
+          <t>-33.36051, -70.80680</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>00:07:52</t>
+          <t>00:38:22</t>
         </is>
       </c>
       <c r="L179" t="n">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
       <c r="M179" t="n">
         <v>3</v>
@@ -10916,11 +10916,11 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>SLP20250627045-AC02</t>
+          <t>SLP20250425120-AC01</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D180" t="inlineStr">
         <is>
@@ -10929,47 +10929,47 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2026/08/28 16:46:13</t>
+          <t>2026/08/28 17:02:37</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>-33.361304, -70.806644</t>
+          <t>-33.360794, -70.806873</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>-33.36130, -70.80664</t>
+          <t>-33.36079, -70.80687</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>2026/08/28 17:24:35</t>
+          <t>2026/08/28 17:18:20</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>-33.360513, -70.8068</t>
+          <t>-33.360811, -70.806838</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>-33.36051, -70.80680</t>
+          <t>-33.36081, -70.80684</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>00:38:22</t>
+          <t>00:15:43</t>
         </is>
       </c>
       <c r="L180" t="n">
-        <v>0.11</v>
+        <v>0.02</v>
       </c>
       <c r="M180" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N180" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="181">
@@ -10979,7 +10979,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
@@ -10988,100 +10988,100 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>2026/08/28 17:02:37</t>
+          <t>2026/08/28 17:18:38</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>-33.360794, -70.806873</t>
+          <t>-33.360813, -70.806844</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>-33.36079, -70.80687</t>
+          <t>-33.36081, -70.80684</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026/08/28 17:18:20</t>
+          <t>2026/08/28 23:29:40</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>-33.360811, -70.806838</t>
+          <t>-33.360025, -70.807053</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>-33.36081, -70.80684</t>
+          <t>-33.36003, -70.80705</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>00:15:43</t>
+          <t>06:11:02</t>
         </is>
       </c>
       <c r="L181" t="n">
-        <v>0.02</v>
+        <v>0.11</v>
       </c>
       <c r="M181" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N181" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>SLP20250425120-AC01</t>
+          <t>SLP20250627045-AC02</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>2026/08/28 17:18:38</t>
+          <t>2026/08/28 17:25:34</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>-33.360813, -70.806844</t>
+          <t>-33.360213, -70.806813</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>-33.36081, -70.80684</t>
+          <t>-33.36021, -70.80681</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>2026/08/28 22:29:40</t>
+          <t>2026/08/28 23:29:52</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>-33.360025, -70.807053</t>
+          <t>-33.359974, -70.807216</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>-33.36003, -70.80705</t>
+          <t>-33.35997, -70.80722</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>05:11:02</t>
+          <t>06:04:18</t>
         </is>
       </c>
       <c r="L182" t="n">
-        <v>0.11</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M182" t="n">
         <v>0</v>
@@ -11093,11 +11093,11 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>SLP20250627045-AC02</t>
+          <t>JAC X200 SJTJ-50</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D183" t="inlineStr">
         <is>
@@ -11106,41 +11106,41 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>2026/08/28 17:25:34</t>
+          <t>2026/08/28 18:42:41</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>-33.360213, -70.806813</t>
+          <t>-32.74337, -70.7326683</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>-33.36021, -70.80681</t>
+          <t>-32.74337, -70.73267</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>2026/08/28 22:29:53</t>
+          <t>2026/08/28 23:59:32</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>-33.359974, -70.807216</t>
+          <t>-32.7432833, -70.7326983</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>-33.35997, -70.80722</t>
+          <t>-32.74328, -70.73270</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>05:04:19</t>
+          <t>05:16:51</t>
         </is>
       </c>
       <c r="L183" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="M183" t="n">
         <v>0</v>
@@ -11152,11 +11152,11 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>JAC X200 SJTJ-50</t>
+          <t>CHANGAN HUNTER TGPS-77</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D184" t="inlineStr">
         <is>
@@ -11165,41 +11165,41 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2026/08/28 18:42:41</t>
+          <t>2026/08/28 19:31:27</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>-32.74337, -70.7326683</t>
+          <t>-32.7976416, -70.8870883</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>-32.74337, -70.73267</t>
+          <t>-32.79764, -70.88709</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>2026/08/28 22:42:02</t>
+          <t>2026/08/28 23:31:27</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>-32.7432833, -70.7326983</t>
+          <t>-32.7976416, -70.8870883</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>-32.74328, -70.73270</t>
+          <t>-32.79764, -70.88709</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>03:59:21</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L184" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="M184" t="n">
         <v>0</v>
@@ -11211,60 +11211,60 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TGPS-77</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Paradas</t>
+          <t>Recorridos</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>2026/08/28 19:31:27</t>
+          <t>2026/08/28 20:38:38</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>-32.7976416, -70.8870883</t>
+          <t>-33.47631, -70.6983583</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>-32.79764, -70.88709</t>
+          <t>-33.47631, -70.69836</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>2026/08/28 21:31:27</t>
+          <t>2026/08/28 21:16:54</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>-32.7976416, -70.8870883</t>
+          <t>-33.4762116, -70.6983366</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>-32.79764, -70.88709</t>
+          <t>-33.47621, -70.69834</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>00:38:16</t>
         </is>
       </c>
       <c r="L185" t="n">
-        <v>0</v>
+        <v>8.17</v>
       </c>
       <c r="M185" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="N185" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="186">
@@ -11274,31 +11274,31 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>2026/08/28 20:38:38</t>
+          <t>2026/08/28 21:18:07</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>-33.47631, -70.6983583</t>
+          <t>-33.47616, -70.69842</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>-33.47631, -70.69836</t>
+          <t>-33.47616, -70.69842</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>2026/08/28 21:18:07</t>
+          <t>2026/08/28 23:18:07</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -11313,17 +11313,17 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>00:39:29</t>
+          <t>02:00:00</t>
         </is>
       </c>
       <c r="L186" t="n">
-        <v>8.18</v>
+        <v>0</v>
       </c>
       <c r="M186" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="N186" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -11412,13 +11412,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>881.59</v>
+        <v>881.6</v>
       </c>
       <c r="C4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>142</v>
@@ -11602,13 +11602,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>618.64</v>
+        <v>618.63</v>
       </c>
       <c r="C14" t="n">
         <v>47</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>126</v>
@@ -11621,10 +11621,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>255.46</v>
+        <v>267.96</v>
       </c>
       <c r="C15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-30T09:44Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/08/29 22:56:36</t>
+          <t>2026/08/29 23:56:36</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>166:00:32</t>
+          <t>167:00:32</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>2026/08/29 21:51:24</t>
+          <t>2026/08/29 23:51:24</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>22:00:17</t>
+          <t>24:00:17</t>
         </is>
       </c>
       <c r="L180" t="n">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>2026/08/29 22:57:15</t>
+          <t>2026/08/29 23:57:15</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>21:00:01</t>
+          <t>22:00:01</t>
         </is>
       </c>
       <c r="L181" t="n">
@@ -12124,7 +12124,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>2026/08/29 22:56:07</t>
+          <t>2026/08/29 23:56:06</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -12139,7 +12139,7 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>06:05:19</t>
+          <t>07:05:18</t>
         </is>
       </c>
       <c r="L200" t="n">
@@ -12478,7 +12478,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>2026/08/29 21:14:08</t>
+          <t>2026/08/29 23:14:08</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -12493,7 +12493,7 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>02:00:00</t>
+          <t>04:00:00</t>
         </is>
       </c>
       <c r="L206" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-31T10:33Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/08/30 22:56:36</t>
+          <t>2026/08/30 23:56:36</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>166:00:26</t>
+          <t>167:00:26</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -11062,7 +11062,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>2026/08/30 21:51:24</t>
+          <t>2026/08/30 23:51:24</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -11077,7 +11077,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>46:00:17</t>
+          <t>48:00:17</t>
         </is>
       </c>
       <c r="L182" t="n">
@@ -12360,7 +12360,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>2026/08/30 22:58:45</t>
+          <t>2026/08/30 23:59:06</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>30:00:15</t>
+          <t>31:00:36</t>
         </is>
       </c>
       <c r="L204" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-31T18:47Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -13073,16 +13073,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>891.77</v>
+        <v>931.8099999999999</v>
       </c>
       <c r="C20" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D20" t="n">
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-08-31T23:37Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N209"/>
+  <dimension ref="A1:N210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12680,6 +12680,65 @@
         <v>0</v>
       </c>
       <c r="N209" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN AMAROK KPDV-13</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>6</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>2026/08/30 21:45:07</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>-32.841655, -70.936796</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>-32.84166, -70.93680</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>2026/08/30 23:53:33</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>-32.841583, -70.936855</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>-32.84158, -70.93685</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>02:08:26</t>
+        </is>
+      </c>
+      <c r="L210" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M210" t="n">
+        <v>0</v>
+      </c>
+      <c r="N210" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13073,13 +13132,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>931.8099999999999</v>
+        <v>937.62</v>
       </c>
       <c r="C20" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
         <v>142</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-01T09:10Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/08/31 22:41:45</t>
+          <t>2026/08/31 23:41:45</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>166:01:07</t>
+          <t>167:01:07</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/08/31 22:56:52</t>
+          <t>2026/08/31 23:56:52</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>166:00:42</t>
+          <t>167:00:42</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -11534,7 +11534,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>2026/08/31 22:59:07</t>
+          <t>2026/08/31 23:58:45</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -11549,7 +11549,7 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>54:00:37</t>
+          <t>55:00:15</t>
         </is>
       </c>
       <c r="L190" t="n">
@@ -12242,7 +12242,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>2026/08/31 22:47:29</t>
+          <t>2026/08/31 23:47:29</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -12257,7 +12257,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>06:03:15</t>
+          <t>07:03:15</t>
         </is>
       </c>
       <c r="L202" t="n">
@@ -12301,7 +12301,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>2026/08/31 22:56:46</t>
+          <t>2026/08/31 23:56:46</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>06:01:06</t>
+          <t>07:01:06</t>
         </is>
       </c>
       <c r="L203" t="n">
@@ -12419,7 +12419,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>2026/08/31 21:39:17</t>
+          <t>2026/08/31 23:39:17</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -12434,7 +12434,7 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>02:00:58</t>
+          <t>04:00:58</t>
         </is>
       </c>
       <c r="L205" t="n">
@@ -12478,7 +12478,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>2026/08/31 21:40:09</t>
+          <t>2026/08/31 23:40:09</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -12493,7 +12493,7 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>02:00:44</t>
+          <t>04:00:44</t>
         </is>
       </c>
       <c r="L206" t="n">
@@ -12537,7 +12537,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>2026/08/31 21:42:59</t>
+          <t>2026/08/31 23:42:59</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -12552,7 +12552,7 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>02:03:02</t>
+          <t>04:03:02</t>
         </is>
       </c>
       <c r="L207" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-02T08:23Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/09/01 22:22:24</t>
+          <t>2026/09/01 23:22:26</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>166:00:05</t>
+          <t>167:00:07</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/09/01 22:41:45</t>
+          <t>2026/09/01 23:41:45</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:00:35</t>
+          <t>167:00:35</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026/09/01 22:56:52</t>
+          <t>2026/09/01 23:56:52</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>166:00:42</t>
+          <t>167:00:42</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -5575,7 +5575,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>2026/09/01 21:04:45</t>
+          <t>2026/09/01 23:04:45</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>132:00:00</t>
+          <t>134:00:00</t>
         </is>
       </c>
       <c r="L89" t="n">
@@ -10295,7 +10295,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>2026/09/01 22:08:25</t>
+          <t>2026/09/01 23:08:27</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>92:11:11</t>
+          <t>93:11:13</t>
         </is>
       </c>
       <c r="L169" t="n">
@@ -11475,7 +11475,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>2026/09/01 22:13:21</t>
+          <t>2026/09/01 23:13:21</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -11490,7 +11490,7 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>77:14:51</t>
+          <t>78:14:51</t>
         </is>
       </c>
       <c r="L189" t="n">
@@ -12301,7 +12301,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>2026/09/01 22:44:09</t>
+          <t>2026/09/01 23:44:12</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>29:59:55</t>
+          <t>30:59:58</t>
         </is>
       </c>
       <c r="L203" t="n">
@@ -12773,7 +12773,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>2026/09/01 21:42:08</t>
+          <t>2026/09/01 23:42:08</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -12788,7 +12788,7 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>08:00:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="L211" t="n">
@@ -13127,7 +13127,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>2026/09/01 22:04:51</t>
+          <t>2026/09/01 23:04:51</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -13142,7 +13142,7 @@
       </c>
       <c r="K217" t="inlineStr">
         <is>
-          <t>05:01:12</t>
+          <t>06:01:12</t>
         </is>
       </c>
       <c r="L217" t="n">

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-03T08:33Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N222"/>
+  <dimension ref="A1:N223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -737,7 +737,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/09/02 22:22:27</t>
+          <t>2026/09/02 23:22:27</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>165:58:41</t>
+          <t>166:58:41</t>
         </is>
       </c>
       <c r="L7" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026/09/02 22:41:41</t>
+          <t>2026/09/02 23:41:41</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>166:00:31</t>
+          <t>167:00:31</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026/09/02 22:56:09</t>
+          <t>2026/09/02 23:56:09</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>165:59:59</t>
+          <t>166:59:59</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>2026/09/02 21:04:45</t>
+          <t>2026/09/02 23:04:45</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>156:00:00</t>
+          <t>158:00:00</t>
         </is>
       </c>
       <c r="L33" t="n">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>2026/09/02 22:01:21</t>
+          <t>2026/09/02 23:01:39</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>149:55:35</t>
+          <t>150:55:53</t>
         </is>
       </c>
       <c r="L93" t="n">
@@ -9528,7 +9528,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>2026/09/02 22:58:06</t>
+          <t>2026/09/02 23:57:38</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>117:00:52</t>
+          <t>118:00:24</t>
         </is>
       </c>
       <c r="L156" t="n">
@@ -11711,7 +11711,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>2026/09/02 22:11:22</t>
+          <t>2026/09/02 23:11:38</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -11726,7 +11726,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>53:27:08</t>
+          <t>54:27:24</t>
         </is>
       </c>
       <c r="L193" t="n">
@@ -13009,7 +13009,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>2026/09/02 22:59:19</t>
+          <t>2026/09/02 23:59:19</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -13024,7 +13024,7 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>11:01:01</t>
+          <t>12:01:01</t>
         </is>
       </c>
       <c r="L215" t="n">
@@ -13186,7 +13186,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>2026/09/02 21:59:36</t>
+          <t>2026/09/02 23:59:36</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -13201,7 +13201,7 @@
       </c>
       <c r="K218" t="inlineStr">
         <is>
-          <t>04:01:14</t>
+          <t>06:01:14</t>
         </is>
       </c>
       <c r="L218" t="n">
@@ -13447,6 +13447,65 @@
         <v>0</v>
       </c>
       <c r="N222" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 PHZF-89</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>7</v>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>2026/09/02 21:27:21</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>-33.4368599, -70.62946</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>-33.43686, -70.62946</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>2026/09/02 23:27:21</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>-33.4368599, -70.62946</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>-33.43686, -70.62946</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L223" t="n">
+        <v>0</v>
+      </c>
+      <c r="M223" t="n">
+        <v>0</v>
+      </c>
+      <c r="N223" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13745,13 +13804,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>241.14</v>
+        <v>241.02</v>
       </c>
       <c r="C15" t="n">
         <v>25</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>126</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-04T08:28Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N206"/>
+  <dimension ref="A1:N207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,7 +796,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/09/03 22:01:38</t>
+          <t>2026/09/03 23:01:15</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>165:43:00</t>
+          <t>166:42:37</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/09/03 22:24:40</t>
+          <t>2026/09/03 23:23:09</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>165:59:51</t>
+          <t>166:58:20</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026/09/03 22:41:41</t>
+          <t>2026/09/03 23:41:41</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>166:00:05</t>
+          <t>167:00:05</t>
         </is>
       </c>
       <c r="L13" t="n">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026/09/03 22:56:09</t>
+          <t>2026/09/03 23:56:09</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>165:59:58</t>
+          <t>166:59:58</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/09/03 21:04:45</t>
+          <t>2026/09/03 23:04:45</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>164:00:00</t>
+          <t>166:00:00</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026/09/03 22:31:22</t>
+          <t>2026/09/03 23:31:38</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>164:00:01</t>
+          <t>165:00:17</t>
         </is>
       </c>
       <c r="L22" t="n">
@@ -7640,7 +7640,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>2026/09/03 21:57:28</t>
+          <t>2026/09/03 23:57:30</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>140:00:14</t>
+          <t>142:00:16</t>
         </is>
       </c>
       <c r="L124" t="n">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>2026/09/03 22:12:03</t>
+          <t>2026/09/03 23:11:37</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>77:27:49</t>
+          <t>78:27:23</t>
         </is>
       </c>
       <c r="L167" t="n">
@@ -12183,7 +12183,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>2026/09/03 21:41:26</t>
+          <t>2026/09/03 23:41:26</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -12198,7 +12198,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>04:01:02</t>
+          <t>06:01:02</t>
         </is>
       </c>
       <c r="L201" t="n">
@@ -12242,7 +12242,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>2026/09/03 22:44:06</t>
+          <t>2026/09/03 23:44:07</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -12257,7 +12257,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>05:01:22</t>
+          <t>06:01:23</t>
         </is>
       </c>
       <c r="L202" t="n">
@@ -12503,6 +12503,65 @@
         <v>0</v>
       </c>
       <c r="N206" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>MITSUBISHI L200 LVHX-40</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>12</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Paradas</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>2026/09/03 21:11:55</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>-33.47614, -70.69841</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>-33.47614, -70.69841</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>2026/09/03 23:11:55</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>-33.47614, -70.69841</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>-33.47614, -70.69841</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="L207" t="n">
+        <v>0</v>
+      </c>
+      <c r="M207" t="n">
+        <v>0</v>
+      </c>
+      <c r="N207" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12782,13 +12841,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>954.5599999999999</v>
+        <v>954.55</v>
       </c>
       <c r="C14" t="n">
         <v>51</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>127</v>

</xml_diff>

<commit_message>
chore: actualiza recorrido 2026-09-05T08:03Z
</commit_message>
<xml_diff>
--- a/REPORTE DE RECORRIDO.xlsx
+++ b/REPORTE DE RECORRIDO.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N203"/>
+  <dimension ref="A1:N204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,7 +619,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/09/04 22:01:22</t>
+          <t>2026/09/04 23:01:39</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>166:00:01</t>
+          <t>167:00:18</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -855,7 +855,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/09/04 22:25:08</t>
+          <t>2026/09/04 23:23:09</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -870,7 +870,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>166:02:30</t>
+          <t>167:00:31</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026/09/04 22:31:20</t>
+          <t>2026/09/04 23:31:22</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>165:59:42</t>
+          <t>166:59:44</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026/09/04 22:42:06</t>
+          <t>2026/09/04 23:42:06</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>166:00:30</t>
+          <t>167:00:30</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026/09/04 22:56:11</t>
+          <t>2026/09/04 23:56:11</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>166:00:00</t>
+          <t>167:00:00</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026/09/04 21:04:45</t>
+          <t>2026/09/04 23:04:45</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>164:00:00</t>
+          <t>166:00:00</t>
         </is>
       </c>
       <c r="L18" t="n">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>2026/09/04 22:11:21</t>
+          <t>2026/09/04 23:11:30</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>101:27:07</t>
+          <t>102:27:16</t>
         </is>
       </c>
       <c r="L131" t="n">
@@ -10354,7 +10354,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>2026/09/04 22:46:33</t>
+          <t>2026/09/04 23:46:07</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>59:05:52</t>
+          <t>60:05:26</t>
         </is>
       </c>
       <c r="L170" t="n">
@@ -12242,7 +12242,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>2026/09/04 21:52:42</t>
+          <t>2026/09/04 23:52:42</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -12257,7 +12257,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>02:00:46</t>
+          <t>04:00:46</t>
         </is>
       </c>
       <c r="L202" t="n">
@@ -12273,59 +12273,118 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>CHANGAN HUNTER TKCL-70</t>
+          <t>MITSUBISHI L200 LVHX-40</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Recorridos</t>
+          <t>Paradas</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>2026/09/04 22:03:47</t>
+          <t>2026/09/04 21:13:08</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>-32.838483, -70.954875</t>
+          <t>-33.4761199, -70.6980899</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>-32.83848, -70.95488</t>
+          <t>-33.47612, -70.69809</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>2026/09/04 22:24:25</t>
+          <t>2026/09/04 23:15:29</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>-32.779806, -70.979927</t>
+          <t>-33.4761866, -70.6983983</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>-32.77981, -70.97993</t>
+          <t>-33.47619, -70.69840</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>00:20:38</t>
+          <t>02:02:21</t>
         </is>
       </c>
       <c r="L203" t="n">
-        <v>6.93</v>
+        <v>0.03</v>
       </c>
       <c r="M203" t="n">
         <v>0</v>
       </c>
       <c r="N203" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>CHANGAN HUNTER TKCL-70</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>5</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Recorridos</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>2026/09/04 22:03:47</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>-32.838483, -70.954875</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>-32.83848, -70.95488</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>2026/09/04 22:24:25</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>-32.779806, -70.979927</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>-32.77981, -70.97993</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>00:20:38</t>
+        </is>
+      </c>
+      <c r="L204" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="M204" t="n">
+        <v>0</v>
+      </c>
+      <c r="N204" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12605,13 +12664,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>988.89</v>
+        <v>988.75</v>
       </c>
       <c r="C14" t="n">
         <v>52</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>127</v>

</xml_diff>